<commit_message>
Fixed the clamping both max and 0 qty items
</commit_message>
<xml_diff>
--- a/FoodBank Files/Food Bank recipients.xlsx
+++ b/FoodBank Files/Food Bank recipients.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\icarusjay\Downloads\xampp\htdocs\Capstone Project\FoodBank Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\icarusjay\Downloads\xampp\htdocs\FoodBank Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A3CE95-4BDA-4E41-A01E-DC6D3B43AC60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0588E9AF-5FEF-425E-8D51-C4BDCD4F31E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7185" yWindow="585" windowWidth="15120" windowHeight="12510" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="15120" windowHeight="12510" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Directory" sheetId="1" r:id="rId1"/>
@@ -2057,9 +2057,6 @@
     <t>focuses on helping abandoned, neglected and exploited children, needy women, families, older and disabled people by providing shelter and other basic needs for survival, protection, development and participation.</t>
   </si>
   <si>
-    <t>Cordova, Mactan Cebu</t>
-  </si>
-  <si>
     <t>Maria Regin Imfanso Balaga</t>
   </si>
   <si>
@@ -2246,6 +2243,9 @@
   </si>
   <si>
     <t xml:space="preserve">Sta Fe, Bantayan Island  and Sitio Tigbao, San Jose Rd., Talamban, Cebu                </t>
+  </si>
+  <si>
+    <t>Cordova, Mactan, Cebu</t>
   </si>
 </sst>
 </file>
@@ -2781,115 +2781,115 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3521,7 +3521,7 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" s="32"/>
-      <c r="B9" s="87" t="s">
+      <c r="B9" s="52" t="s">
         <v>0</v>
       </c>
       <c r="C9" s="51"/>
@@ -3537,88 +3537,88 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" s="32"/>
-      <c r="B10" s="52" t="s">
+      <c r="B10" s="86" t="s">
         <v>1</v>
       </c>
-      <c r="C10" s="52"/>
-      <c r="D10" s="52"/>
-      <c r="E10" s="52"/>
-      <c r="F10" s="52"/>
-      <c r="G10" s="52"/>
-      <c r="H10" s="52"/>
-      <c r="I10" s="52"/>
-      <c r="J10" s="52"/>
-      <c r="K10" s="52"/>
+      <c r="C10" s="86"/>
+      <c r="D10" s="86"/>
+      <c r="E10" s="86"/>
+      <c r="F10" s="86"/>
+      <c r="G10" s="86"/>
+      <c r="H10" s="86"/>
+      <c r="I10" s="86"/>
+      <c r="J10" s="86"/>
+      <c r="K10" s="86"/>
       <c r="L10" s="32"/>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" s="32"/>
-      <c r="B11" s="52"/>
-      <c r="C11" s="52"/>
-      <c r="D11" s="52"/>
-      <c r="E11" s="52"/>
-      <c r="F11" s="52"/>
-      <c r="G11" s="52"/>
-      <c r="H11" s="52"/>
-      <c r="I11" s="52"/>
-      <c r="J11" s="52"/>
-      <c r="K11" s="52"/>
+      <c r="B11" s="86"/>
+      <c r="C11" s="86"/>
+      <c r="D11" s="86"/>
+      <c r="E11" s="86"/>
+      <c r="F11" s="86"/>
+      <c r="G11" s="86"/>
+      <c r="H11" s="86"/>
+      <c r="I11" s="86"/>
+      <c r="J11" s="86"/>
+      <c r="K11" s="86"/>
       <c r="L11" s="32"/>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" s="32"/>
-      <c r="B12" s="88" t="s">
+      <c r="B12" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="C12" s="88"/>
-      <c r="D12" s="88"/>
-      <c r="E12" s="88"/>
-      <c r="F12" s="88"/>
-      <c r="G12" s="88"/>
-      <c r="H12" s="88"/>
-      <c r="I12" s="88"/>
-      <c r="J12" s="88"/>
-      <c r="K12" s="88"/>
+      <c r="C12" s="53"/>
+      <c r="D12" s="53"/>
+      <c r="E12" s="53"/>
+      <c r="F12" s="53"/>
+      <c r="G12" s="53"/>
+      <c r="H12" s="53"/>
+      <c r="I12" s="53"/>
+      <c r="J12" s="53"/>
+      <c r="K12" s="53"/>
       <c r="L12" s="32"/>
     </row>
     <row r="13" spans="1:12">
       <c r="A13" s="32"/>
-      <c r="B13" s="82" t="s">
+      <c r="B13" s="54" t="s">
         <v>3</v>
       </c>
-      <c r="C13" s="83"/>
-      <c r="D13" s="84"/>
-      <c r="E13" s="82" t="s">
+      <c r="C13" s="55"/>
+      <c r="D13" s="56"/>
+      <c r="E13" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="F13" s="83"/>
-      <c r="G13" s="84"/>
-      <c r="H13" s="82" t="s">
+      <c r="F13" s="55"/>
+      <c r="G13" s="56"/>
+      <c r="H13" s="54" t="s">
         <v>5</v>
       </c>
-      <c r="I13" s="83"/>
-      <c r="J13" s="83"/>
-      <c r="K13" s="84"/>
+      <c r="I13" s="55"/>
+      <c r="J13" s="55"/>
+      <c r="K13" s="56"/>
       <c r="L13" s="32"/>
     </row>
     <row r="14" spans="1:12">
       <c r="A14" s="32"/>
-      <c r="B14" s="66" t="s">
+      <c r="B14" s="57" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="67"/>
-      <c r="D14" s="68"/>
-      <c r="E14" s="66" t="s">
+      <c r="C14" s="58"/>
+      <c r="D14" s="59"/>
+      <c r="E14" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="F14" s="67"/>
-      <c r="G14" s="68"/>
-      <c r="H14" s="69" t="s">
+      <c r="F14" s="58"/>
+      <c r="G14" s="59"/>
+      <c r="H14" s="60" t="s">
         <v>8</v>
       </c>
-      <c r="I14" s="70"/>
-      <c r="J14" s="70"/>
-      <c r="K14" s="71"/>
+      <c r="I14" s="61"/>
+      <c r="J14" s="61"/>
+      <c r="K14" s="62"/>
       <c r="L14" s="32"/>
     </row>
     <row r="15" spans="1:12">
@@ -3626,39 +3626,39 @@
       <c r="B15" s="63" t="s">
         <v>9</v>
       </c>
-      <c r="C15" s="81"/>
-      <c r="D15" s="64"/>
+      <c r="C15" s="64"/>
+      <c r="D15" s="65"/>
       <c r="E15" s="63" t="s">
         <v>10</v>
       </c>
-      <c r="F15" s="81"/>
-      <c r="G15" s="64"/>
-      <c r="H15" s="78" t="s">
+      <c r="F15" s="64"/>
+      <c r="G15" s="65"/>
+      <c r="H15" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="I15" s="79"/>
-      <c r="J15" s="79"/>
-      <c r="K15" s="80"/>
+      <c r="I15" s="67"/>
+      <c r="J15" s="67"/>
+      <c r="K15" s="68"/>
       <c r="L15" s="32"/>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" s="32"/>
-      <c r="B16" s="66" t="s">
+      <c r="B16" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="67"/>
-      <c r="D16" s="68"/>
-      <c r="E16" s="66" t="s">
+      <c r="C16" s="58"/>
+      <c r="D16" s="59"/>
+      <c r="E16" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="F16" s="67"/>
-      <c r="G16" s="68"/>
-      <c r="H16" s="69" t="s">
+      <c r="F16" s="58"/>
+      <c r="G16" s="59"/>
+      <c r="H16" s="60" t="s">
         <v>14</v>
       </c>
-      <c r="I16" s="70"/>
-      <c r="J16" s="70"/>
-      <c r="K16" s="71"/>
+      <c r="I16" s="61"/>
+      <c r="J16" s="61"/>
+      <c r="K16" s="62"/>
       <c r="L16" s="32"/>
     </row>
     <row r="17" spans="1:16">
@@ -3666,39 +3666,39 @@
       <c r="B17" s="63" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="81"/>
-      <c r="D17" s="64"/>
+      <c r="C17" s="64"/>
+      <c r="D17" s="65"/>
       <c r="E17" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="F17" s="81"/>
-      <c r="G17" s="64"/>
-      <c r="H17" s="78" t="s">
+      <c r="F17" s="64"/>
+      <c r="G17" s="65"/>
+      <c r="H17" s="66" t="s">
         <v>17</v>
       </c>
-      <c r="I17" s="79"/>
-      <c r="J17" s="79"/>
-      <c r="K17" s="80"/>
+      <c r="I17" s="67"/>
+      <c r="J17" s="67"/>
+      <c r="K17" s="68"/>
       <c r="L17" s="32"/>
     </row>
     <row r="18" spans="1:16">
       <c r="A18" s="32"/>
-      <c r="B18" s="66" t="s">
+      <c r="B18" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="67"/>
-      <c r="D18" s="68"/>
-      <c r="E18" s="66" t="s">
+      <c r="C18" s="58"/>
+      <c r="D18" s="59"/>
+      <c r="E18" s="57" t="s">
         <v>19</v>
       </c>
-      <c r="F18" s="67"/>
-      <c r="G18" s="68"/>
-      <c r="H18" s="69" t="s">
+      <c r="F18" s="58"/>
+      <c r="G18" s="59"/>
+      <c r="H18" s="60" t="s">
         <v>20</v>
       </c>
-      <c r="I18" s="70"/>
-      <c r="J18" s="70"/>
-      <c r="K18" s="71"/>
+      <c r="I18" s="61"/>
+      <c r="J18" s="61"/>
+      <c r="K18" s="62"/>
       <c r="L18" s="32"/>
     </row>
     <row r="19" spans="1:16">
@@ -3706,39 +3706,39 @@
       <c r="B19" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="81"/>
-      <c r="D19" s="64"/>
+      <c r="C19" s="64"/>
+      <c r="D19" s="65"/>
       <c r="E19" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="F19" s="81"/>
-      <c r="G19" s="64"/>
-      <c r="H19" s="78" t="s">
+      <c r="F19" s="64"/>
+      <c r="G19" s="65"/>
+      <c r="H19" s="66" t="s">
         <v>23</v>
       </c>
-      <c r="I19" s="79"/>
-      <c r="J19" s="79"/>
-      <c r="K19" s="80"/>
+      <c r="I19" s="67"/>
+      <c r="J19" s="67"/>
+      <c r="K19" s="68"/>
       <c r="L19" s="32"/>
     </row>
     <row r="20" spans="1:16">
       <c r="A20" s="32"/>
-      <c r="B20" s="66" t="s">
+      <c r="B20" s="57" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="67"/>
-      <c r="D20" s="68"/>
-      <c r="E20" s="66" t="s">
+      <c r="C20" s="58"/>
+      <c r="D20" s="59"/>
+      <c r="E20" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="F20" s="67"/>
-      <c r="G20" s="68"/>
-      <c r="H20" s="69" t="s">
+      <c r="F20" s="58"/>
+      <c r="G20" s="59"/>
+      <c r="H20" s="60" t="s">
         <v>26</v>
       </c>
-      <c r="I20" s="70"/>
-      <c r="J20" s="70"/>
-      <c r="K20" s="71"/>
+      <c r="I20" s="61"/>
+      <c r="J20" s="61"/>
+      <c r="K20" s="62"/>
       <c r="L20" s="32"/>
     </row>
     <row r="21" spans="1:16">
@@ -3746,39 +3746,39 @@
       <c r="B21" s="63" t="s">
         <v>27</v>
       </c>
-      <c r="C21" s="81"/>
-      <c r="D21" s="64"/>
+      <c r="C21" s="64"/>
+      <c r="D21" s="65"/>
       <c r="E21" s="63" t="s">
         <v>28</v>
       </c>
-      <c r="F21" s="81"/>
-      <c r="G21" s="64"/>
-      <c r="H21" s="78" t="s">
+      <c r="F21" s="64"/>
+      <c r="G21" s="65"/>
+      <c r="H21" s="66" t="s">
         <v>29</v>
       </c>
-      <c r="I21" s="79"/>
-      <c r="J21" s="79"/>
-      <c r="K21" s="80"/>
+      <c r="I21" s="67"/>
+      <c r="J21" s="67"/>
+      <c r="K21" s="68"/>
       <c r="L21" s="32"/>
     </row>
     <row r="22" spans="1:16">
       <c r="A22" s="32"/>
-      <c r="B22" s="66" t="s">
+      <c r="B22" s="57" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="67"/>
-      <c r="D22" s="68"/>
-      <c r="E22" s="66" t="s">
+      <c r="C22" s="58"/>
+      <c r="D22" s="59"/>
+      <c r="E22" s="57" t="s">
         <v>31</v>
       </c>
-      <c r="F22" s="67"/>
-      <c r="G22" s="68"/>
-      <c r="H22" s="69" t="s">
+      <c r="F22" s="58"/>
+      <c r="G22" s="59"/>
+      <c r="H22" s="60" t="s">
         <v>32</v>
       </c>
-      <c r="I22" s="70"/>
-      <c r="J22" s="70"/>
-      <c r="K22" s="71"/>
+      <c r="I22" s="61"/>
+      <c r="J22" s="61"/>
+      <c r="K22" s="62"/>
       <c r="L22" s="32"/>
     </row>
     <row r="23" spans="1:16">
@@ -3801,18 +3801,18 @@
     </row>
     <row r="24" spans="1:16">
       <c r="A24" s="32"/>
-      <c r="B24" s="65" t="s">
+      <c r="B24" s="69" t="s">
         <v>33</v>
       </c>
-      <c r="C24" s="65"/>
-      <c r="D24" s="65"/>
-      <c r="E24" s="65"/>
-      <c r="F24" s="65"/>
-      <c r="G24" s="65"/>
-      <c r="H24" s="65"/>
-      <c r="I24" s="65"/>
-      <c r="J24" s="65"/>
-      <c r="K24" s="65"/>
+      <c r="C24" s="69"/>
+      <c r="D24" s="69"/>
+      <c r="E24" s="69"/>
+      <c r="F24" s="69"/>
+      <c r="G24" s="69"/>
+      <c r="H24" s="69"/>
+      <c r="I24" s="69"/>
+      <c r="J24" s="69"/>
+      <c r="K24" s="69"/>
       <c r="L24" s="32"/>
       <c r="M24" s="32"/>
       <c r="N24" s="32"/>
@@ -3821,64 +3821,64 @@
     </row>
     <row r="25" spans="1:16">
       <c r="A25" s="32"/>
-      <c r="B25" s="82" t="s">
+      <c r="B25" s="54" t="s">
         <v>34</v>
       </c>
-      <c r="C25" s="83"/>
-      <c r="D25" s="83"/>
-      <c r="E25" s="83"/>
-      <c r="F25" s="84"/>
-      <c r="G25" s="82" t="s">
+      <c r="C25" s="55"/>
+      <c r="D25" s="55"/>
+      <c r="E25" s="55"/>
+      <c r="F25" s="56"/>
+      <c r="G25" s="54" t="s">
         <v>5</v>
       </c>
-      <c r="H25" s="85"/>
-      <c r="I25" s="85"/>
-      <c r="J25" s="85"/>
-      <c r="K25" s="86"/>
+      <c r="H25" s="70"/>
+      <c r="I25" s="70"/>
+      <c r="J25" s="70"/>
+      <c r="K25" s="71"/>
       <c r="L25" s="63"/>
-      <c r="M25" s="64"/>
+      <c r="M25" s="65"/>
       <c r="N25" s="32"/>
       <c r="O25"/>
       <c r="P25"/>
     </row>
     <row r="26" spans="1:16">
       <c r="A26" s="32"/>
-      <c r="B26" s="55" t="s">
+      <c r="B26" s="72" t="s">
         <v>35</v>
       </c>
-      <c r="C26" s="55"/>
-      <c r="D26" s="55"/>
-      <c r="E26" s="55"/>
-      <c r="F26" s="55"/>
-      <c r="G26" s="56" t="s">
+      <c r="C26" s="72"/>
+      <c r="D26" s="72"/>
+      <c r="E26" s="72"/>
+      <c r="F26" s="72"/>
+      <c r="G26" s="73" t="s">
         <v>36</v>
       </c>
-      <c r="H26" s="56"/>
-      <c r="I26" s="56"/>
-      <c r="J26" s="56"/>
-      <c r="K26" s="56"/>
+      <c r="H26" s="73"/>
+      <c r="I26" s="73"/>
+      <c r="J26" s="73"/>
+      <c r="K26" s="73"/>
       <c r="L26" s="63"/>
-      <c r="M26" s="64"/>
+      <c r="M26" s="65"/>
       <c r="N26" s="32"/>
       <c r="O26"/>
       <c r="P26"/>
     </row>
     <row r="27" spans="1:16">
       <c r="A27" s="32"/>
-      <c r="B27" s="53" t="s">
+      <c r="B27" s="74" t="s">
         <v>37</v>
       </c>
-      <c r="C27" s="53"/>
-      <c r="D27" s="53"/>
-      <c r="E27" s="53"/>
-      <c r="F27" s="53"/>
-      <c r="G27" s="54" t="s">
+      <c r="C27" s="74"/>
+      <c r="D27" s="74"/>
+      <c r="E27" s="74"/>
+      <c r="F27" s="74"/>
+      <c r="G27" s="75" t="s">
         <v>38</v>
       </c>
-      <c r="H27" s="54"/>
-      <c r="I27" s="54"/>
-      <c r="J27" s="54"/>
-      <c r="K27" s="54"/>
+      <c r="H27" s="75"/>
+      <c r="I27" s="75"/>
+      <c r="J27" s="75"/>
+      <c r="K27" s="75"/>
       <c r="L27" s="76" t="s">
         <v>39</v>
       </c>
@@ -3889,64 +3889,64 @@
     </row>
     <row r="28" spans="1:16">
       <c r="A28" s="32"/>
-      <c r="B28" s="55" t="s">
+      <c r="B28" s="72" t="s">
         <v>40</v>
       </c>
-      <c r="C28" s="55"/>
-      <c r="D28" s="55"/>
-      <c r="E28" s="55"/>
-      <c r="F28" s="55"/>
-      <c r="G28" s="56" t="s">
+      <c r="C28" s="72"/>
+      <c r="D28" s="72"/>
+      <c r="E28" s="72"/>
+      <c r="F28" s="72"/>
+      <c r="G28" s="73" t="s">
         <v>41</v>
       </c>
-      <c r="H28" s="56"/>
-      <c r="I28" s="56"/>
-      <c r="J28" s="56"/>
-      <c r="K28" s="56"/>
+      <c r="H28" s="73"/>
+      <c r="I28" s="73"/>
+      <c r="J28" s="73"/>
+      <c r="K28" s="73"/>
       <c r="L28" s="63"/>
-      <c r="M28" s="64"/>
+      <c r="M28" s="65"/>
       <c r="N28" s="32"/>
       <c r="O28"/>
       <c r="P28"/>
     </row>
     <row r="29" spans="1:16">
       <c r="A29" s="32"/>
-      <c r="B29" s="53" t="s">
+      <c r="B29" s="74" t="s">
         <v>42</v>
       </c>
-      <c r="C29" s="53"/>
-      <c r="D29" s="53"/>
-      <c r="E29" s="53"/>
-      <c r="F29" s="53"/>
-      <c r="G29" s="54" t="s">
+      <c r="C29" s="74"/>
+      <c r="D29" s="74"/>
+      <c r="E29" s="74"/>
+      <c r="F29" s="74"/>
+      <c r="G29" s="75" t="s">
         <v>43</v>
       </c>
-      <c r="H29" s="54"/>
-      <c r="I29" s="54"/>
-      <c r="J29" s="54"/>
-      <c r="K29" s="54"/>
+      <c r="H29" s="75"/>
+      <c r="I29" s="75"/>
+      <c r="J29" s="75"/>
+      <c r="K29" s="75"/>
       <c r="L29" s="63"/>
-      <c r="M29" s="64"/>
+      <c r="M29" s="65"/>
       <c r="N29" s="32"/>
       <c r="O29"/>
       <c r="P29"/>
     </row>
     <row r="30" spans="1:16">
       <c r="A30" s="32"/>
-      <c r="B30" s="55" t="s">
+      <c r="B30" s="72" t="s">
         <v>44</v>
       </c>
-      <c r="C30" s="55"/>
-      <c r="D30" s="55"/>
-      <c r="E30" s="55"/>
-      <c r="F30" s="55"/>
-      <c r="G30" s="56" t="s">
+      <c r="C30" s="72"/>
+      <c r="D30" s="72"/>
+      <c r="E30" s="72"/>
+      <c r="F30" s="72"/>
+      <c r="G30" s="73" t="s">
         <v>45</v>
       </c>
-      <c r="H30" s="56"/>
-      <c r="I30" s="56"/>
-      <c r="J30" s="56"/>
-      <c r="K30" s="56"/>
+      <c r="H30" s="73"/>
+      <c r="I30" s="73"/>
+      <c r="J30" s="73"/>
+      <c r="K30" s="73"/>
       <c r="L30" s="76" t="s">
         <v>46</v>
       </c>
@@ -3957,42 +3957,42 @@
     </row>
     <row r="31" spans="1:16">
       <c r="A31" s="32"/>
-      <c r="B31" s="53" t="s">
+      <c r="B31" s="74" t="s">
         <v>47</v>
       </c>
-      <c r="C31" s="53"/>
-      <c r="D31" s="53"/>
-      <c r="E31" s="53"/>
-      <c r="F31" s="53"/>
-      <c r="G31" s="78" t="s">
+      <c r="C31" s="74"/>
+      <c r="D31" s="74"/>
+      <c r="E31" s="74"/>
+      <c r="F31" s="74"/>
+      <c r="G31" s="66" t="s">
         <v>48</v>
       </c>
-      <c r="H31" s="79"/>
-      <c r="I31" s="79"/>
-      <c r="J31" s="79"/>
-      <c r="K31" s="80"/>
+      <c r="H31" s="67"/>
+      <c r="I31" s="67"/>
+      <c r="J31" s="67"/>
+      <c r="K31" s="68"/>
       <c r="L31" s="63"/>
-      <c r="M31" s="64"/>
+      <c r="M31" s="65"/>
       <c r="N31" s="32"/>
       <c r="O31"/>
       <c r="P31"/>
     </row>
     <row r="32" spans="1:16">
       <c r="A32" s="32"/>
-      <c r="B32" s="55" t="s">
+      <c r="B32" s="72" t="s">
         <v>49</v>
       </c>
-      <c r="C32" s="55"/>
-      <c r="D32" s="55"/>
-      <c r="E32" s="55"/>
-      <c r="F32" s="55"/>
-      <c r="G32" s="56" t="s">
+      <c r="C32" s="72"/>
+      <c r="D32" s="72"/>
+      <c r="E32" s="72"/>
+      <c r="F32" s="72"/>
+      <c r="G32" s="73" t="s">
         <v>50</v>
       </c>
-      <c r="H32" s="56"/>
-      <c r="I32" s="56"/>
-      <c r="J32" s="56"/>
-      <c r="K32" s="56"/>
+      <c r="H32" s="73"/>
+      <c r="I32" s="73"/>
+      <c r="J32" s="73"/>
+      <c r="K32" s="73"/>
       <c r="L32" s="76" t="s">
         <v>51</v>
       </c>
@@ -4003,42 +4003,42 @@
     </row>
     <row r="33" spans="1:16">
       <c r="A33" s="32"/>
-      <c r="B33" s="53" t="s">
+      <c r="B33" s="74" t="s">
         <v>52</v>
       </c>
-      <c r="C33" s="53"/>
-      <c r="D33" s="53"/>
-      <c r="E33" s="53"/>
-      <c r="F33" s="53"/>
-      <c r="G33" s="78" t="s">
+      <c r="C33" s="74"/>
+      <c r="D33" s="74"/>
+      <c r="E33" s="74"/>
+      <c r="F33" s="74"/>
+      <c r="G33" s="66" t="s">
         <v>48</v>
       </c>
-      <c r="H33" s="79"/>
-      <c r="I33" s="79"/>
-      <c r="J33" s="79"/>
-      <c r="K33" s="80"/>
+      <c r="H33" s="67"/>
+      <c r="I33" s="67"/>
+      <c r="J33" s="67"/>
+      <c r="K33" s="68"/>
       <c r="L33" s="63"/>
-      <c r="M33" s="64"/>
+      <c r="M33" s="65"/>
       <c r="N33" s="32"/>
       <c r="O33"/>
       <c r="P33"/>
     </row>
     <row r="34" spans="1:16">
       <c r="A34" s="32"/>
-      <c r="B34" s="55" t="s">
+      <c r="B34" s="72" t="s">
         <v>53</v>
       </c>
-      <c r="C34" s="55"/>
-      <c r="D34" s="55"/>
-      <c r="E34" s="55"/>
-      <c r="F34" s="55"/>
-      <c r="G34" s="56" t="s">
+      <c r="C34" s="72"/>
+      <c r="D34" s="72"/>
+      <c r="E34" s="72"/>
+      <c r="F34" s="72"/>
+      <c r="G34" s="73" t="s">
         <v>54</v>
       </c>
-      <c r="H34" s="56"/>
-      <c r="I34" s="56"/>
-      <c r="J34" s="56"/>
-      <c r="K34" s="56"/>
+      <c r="H34" s="73"/>
+      <c r="I34" s="73"/>
+      <c r="J34" s="73"/>
+      <c r="K34" s="73"/>
       <c r="L34" s="76" t="s">
         <v>55</v>
       </c>
@@ -4049,350 +4049,350 @@
     </row>
     <row r="35" spans="1:16">
       <c r="A35" s="32"/>
-      <c r="B35" s="53" t="s">
+      <c r="B35" s="74" t="s">
         <v>56</v>
       </c>
-      <c r="C35" s="53"/>
-      <c r="D35" s="53"/>
-      <c r="E35" s="53"/>
-      <c r="F35" s="53"/>
-      <c r="G35" s="54" t="s">
+      <c r="C35" s="74"/>
+      <c r="D35" s="74"/>
+      <c r="E35" s="74"/>
+      <c r="F35" s="74"/>
+      <c r="G35" s="75" t="s">
         <v>57</v>
       </c>
-      <c r="H35" s="54"/>
-      <c r="I35" s="54"/>
-      <c r="J35" s="54"/>
-      <c r="K35" s="54"/>
+      <c r="H35" s="75"/>
+      <c r="I35" s="75"/>
+      <c r="J35" s="75"/>
+      <c r="K35" s="75"/>
       <c r="L35" s="63"/>
-      <c r="M35" s="64"/>
+      <c r="M35" s="65"/>
       <c r="N35" s="32"/>
       <c r="O35"/>
       <c r="P35"/>
     </row>
     <row r="36" spans="1:16">
       <c r="A36" s="32"/>
-      <c r="B36" s="55" t="s">
+      <c r="B36" s="72" t="s">
         <v>58</v>
       </c>
-      <c r="C36" s="55"/>
-      <c r="D36" s="55"/>
-      <c r="E36" s="55"/>
-      <c r="F36" s="55"/>
-      <c r="G36" s="56" t="s">
+      <c r="C36" s="72"/>
+      <c r="D36" s="72"/>
+      <c r="E36" s="72"/>
+      <c r="F36" s="72"/>
+      <c r="G36" s="73" t="s">
         <v>59</v>
       </c>
-      <c r="H36" s="56"/>
-      <c r="I36" s="56"/>
-      <c r="J36" s="56"/>
-      <c r="K36" s="56"/>
-      <c r="L36" s="74"/>
-      <c r="M36" s="75"/>
+      <c r="H36" s="73"/>
+      <c r="I36" s="73"/>
+      <c r="J36" s="73"/>
+      <c r="K36" s="73"/>
+      <c r="L36" s="78"/>
+      <c r="M36" s="79"/>
       <c r="N36" s="32"/>
       <c r="O36"/>
       <c r="P36"/>
     </row>
     <row r="37" spans="1:16">
       <c r="A37" s="32"/>
-      <c r="B37" s="53" t="s">
+      <c r="B37" s="74" t="s">
         <v>60</v>
       </c>
-      <c r="C37" s="53"/>
-      <c r="D37" s="53"/>
-      <c r="E37" s="53"/>
-      <c r="F37" s="53"/>
-      <c r="G37" s="54" t="s">
+      <c r="C37" s="74"/>
+      <c r="D37" s="74"/>
+      <c r="E37" s="74"/>
+      <c r="F37" s="74"/>
+      <c r="G37" s="75" t="s">
         <v>61</v>
       </c>
-      <c r="H37" s="54"/>
-      <c r="I37" s="54"/>
-      <c r="J37" s="54"/>
-      <c r="K37" s="54"/>
-      <c r="L37" s="74"/>
-      <c r="M37" s="75"/>
+      <c r="H37" s="75"/>
+      <c r="I37" s="75"/>
+      <c r="J37" s="75"/>
+      <c r="K37" s="75"/>
+      <c r="L37" s="78"/>
+      <c r="M37" s="79"/>
       <c r="N37" s="32"/>
       <c r="O37"/>
       <c r="P37"/>
     </row>
     <row r="38" spans="1:16">
       <c r="A38" s="32"/>
-      <c r="B38" s="55" t="s">
+      <c r="B38" s="72" t="s">
         <v>62</v>
       </c>
-      <c r="C38" s="55"/>
-      <c r="D38" s="55"/>
-      <c r="E38" s="55"/>
-      <c r="F38" s="55"/>
-      <c r="G38" s="56" t="s">
+      <c r="C38" s="72"/>
+      <c r="D38" s="72"/>
+      <c r="E38" s="72"/>
+      <c r="F38" s="72"/>
+      <c r="G38" s="73" t="s">
         <v>63</v>
       </c>
-      <c r="H38" s="56"/>
-      <c r="I38" s="56"/>
-      <c r="J38" s="56"/>
-      <c r="K38" s="56"/>
+      <c r="H38" s="73"/>
+      <c r="I38" s="73"/>
+      <c r="J38" s="73"/>
+      <c r="K38" s="73"/>
       <c r="L38" s="63"/>
-      <c r="M38" s="64"/>
+      <c r="M38" s="65"/>
       <c r="N38" s="32"/>
       <c r="O38"/>
       <c r="P38"/>
     </row>
     <row r="39" spans="1:16">
       <c r="A39" s="32"/>
-      <c r="B39" s="53" t="s">
+      <c r="B39" s="74" t="s">
         <v>64</v>
       </c>
-      <c r="C39" s="53"/>
-      <c r="D39" s="53"/>
-      <c r="E39" s="53"/>
-      <c r="F39" s="53"/>
-      <c r="G39" s="54" t="s">
+      <c r="C39" s="74"/>
+      <c r="D39" s="74"/>
+      <c r="E39" s="74"/>
+      <c r="F39" s="74"/>
+      <c r="G39" s="75" t="s">
         <v>65</v>
       </c>
-      <c r="H39" s="54"/>
-      <c r="I39" s="54"/>
-      <c r="J39" s="54"/>
-      <c r="K39" s="54"/>
+      <c r="H39" s="75"/>
+      <c r="I39" s="75"/>
+      <c r="J39" s="75"/>
+      <c r="K39" s="75"/>
       <c r="L39" s="63"/>
-      <c r="M39" s="64"/>
+      <c r="M39" s="65"/>
       <c r="N39" s="32"/>
       <c r="O39"/>
       <c r="P39"/>
     </row>
     <row r="40" spans="1:16">
       <c r="A40" s="32"/>
-      <c r="B40" s="55" t="s">
+      <c r="B40" s="72" t="s">
         <v>66</v>
       </c>
-      <c r="C40" s="55"/>
-      <c r="D40" s="55"/>
-      <c r="E40" s="55"/>
-      <c r="F40" s="55"/>
-      <c r="G40" s="56" t="s">
+      <c r="C40" s="72"/>
+      <c r="D40" s="72"/>
+      <c r="E40" s="72"/>
+      <c r="F40" s="72"/>
+      <c r="G40" s="73" t="s">
         <v>67</v>
       </c>
-      <c r="H40" s="56"/>
-      <c r="I40" s="56"/>
-      <c r="J40" s="56"/>
-      <c r="K40" s="56"/>
-      <c r="L40" s="74"/>
-      <c r="M40" s="75"/>
+      <c r="H40" s="73"/>
+      <c r="I40" s="73"/>
+      <c r="J40" s="73"/>
+      <c r="K40" s="73"/>
+      <c r="L40" s="78"/>
+      <c r="M40" s="79"/>
       <c r="N40" s="32"/>
       <c r="O40"/>
       <c r="P40"/>
     </row>
     <row r="41" spans="1:16">
       <c r="A41" s="32"/>
-      <c r="B41" s="53" t="s">
+      <c r="B41" s="74" t="s">
         <v>68</v>
       </c>
-      <c r="C41" s="53"/>
-      <c r="D41" s="53"/>
-      <c r="E41" s="53"/>
-      <c r="F41" s="53"/>
-      <c r="G41" s="54" t="s">
+      <c r="C41" s="74"/>
+      <c r="D41" s="74"/>
+      <c r="E41" s="74"/>
+      <c r="F41" s="74"/>
+      <c r="G41" s="75" t="s">
         <v>69</v>
       </c>
-      <c r="H41" s="54"/>
-      <c r="I41" s="54"/>
-      <c r="J41" s="54"/>
-      <c r="K41" s="54"/>
-      <c r="L41" s="74"/>
-      <c r="M41" s="75"/>
+      <c r="H41" s="75"/>
+      <c r="I41" s="75"/>
+      <c r="J41" s="75"/>
+      <c r="K41" s="75"/>
+      <c r="L41" s="78"/>
+      <c r="M41" s="79"/>
       <c r="N41" s="32"/>
       <c r="O41"/>
       <c r="P41"/>
     </row>
     <row r="42" spans="1:16">
       <c r="A42" s="32"/>
-      <c r="B42" s="55" t="s">
+      <c r="B42" s="72" t="s">
         <v>70</v>
       </c>
-      <c r="C42" s="55"/>
-      <c r="D42" s="55"/>
-      <c r="E42" s="55"/>
-      <c r="F42" s="55"/>
-      <c r="G42" s="56" t="s">
+      <c r="C42" s="72"/>
+      <c r="D42" s="72"/>
+      <c r="E42" s="72"/>
+      <c r="F42" s="72"/>
+      <c r="G42" s="73" t="s">
         <v>71</v>
       </c>
-      <c r="H42" s="56"/>
-      <c r="I42" s="56"/>
-      <c r="J42" s="56"/>
-      <c r="K42" s="56"/>
+      <c r="H42" s="73"/>
+      <c r="I42" s="73"/>
+      <c r="J42" s="73"/>
+      <c r="K42" s="73"/>
       <c r="L42" s="63"/>
-      <c r="M42" s="64"/>
+      <c r="M42" s="65"/>
       <c r="N42" s="32"/>
       <c r="O42"/>
       <c r="P42"/>
     </row>
     <row r="43" spans="1:16">
       <c r="A43" s="32"/>
-      <c r="B43" s="53" t="s">
+      <c r="B43" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="C43" s="53"/>
-      <c r="D43" s="53"/>
-      <c r="E43" s="53"/>
-      <c r="F43" s="53"/>
-      <c r="G43" s="54" t="s">
+      <c r="C43" s="74"/>
+      <c r="D43" s="74"/>
+      <c r="E43" s="74"/>
+      <c r="F43" s="74"/>
+      <c r="G43" s="75" t="s">
         <v>73</v>
       </c>
-      <c r="H43" s="54"/>
-      <c r="I43" s="54"/>
-      <c r="J43" s="54"/>
-      <c r="K43" s="54"/>
+      <c r="H43" s="75"/>
+      <c r="I43" s="75"/>
+      <c r="J43" s="75"/>
+      <c r="K43" s="75"/>
       <c r="L43" s="63"/>
-      <c r="M43" s="64"/>
+      <c r="M43" s="65"/>
       <c r="N43" s="32"/>
       <c r="O43"/>
       <c r="P43"/>
     </row>
     <row r="44" spans="1:16">
       <c r="A44" s="32"/>
-      <c r="B44" s="55" t="s">
+      <c r="B44" s="72" t="s">
         <v>74</v>
       </c>
-      <c r="C44" s="55"/>
-      <c r="D44" s="55"/>
-      <c r="E44" s="55"/>
-      <c r="F44" s="55"/>
-      <c r="G44" s="56" t="s">
+      <c r="C44" s="72"/>
+      <c r="D44" s="72"/>
+      <c r="E44" s="72"/>
+      <c r="F44" s="72"/>
+      <c r="G44" s="73" t="s">
         <v>75</v>
       </c>
-      <c r="H44" s="56"/>
-      <c r="I44" s="56"/>
-      <c r="J44" s="56"/>
-      <c r="K44" s="56"/>
+      <c r="H44" s="73"/>
+      <c r="I44" s="73"/>
+      <c r="J44" s="73"/>
+      <c r="K44" s="73"/>
       <c r="L44" s="63"/>
-      <c r="M44" s="64"/>
+      <c r="M44" s="65"/>
       <c r="N44" s="32"/>
       <c r="O44"/>
       <c r="P44"/>
     </row>
     <row r="45" spans="1:16">
       <c r="A45" s="32"/>
-      <c r="B45" s="53" t="s">
+      <c r="B45" s="74" t="s">
         <v>76</v>
       </c>
-      <c r="C45" s="53"/>
-      <c r="D45" s="53"/>
-      <c r="E45" s="53"/>
-      <c r="F45" s="53"/>
-      <c r="G45" s="54" t="s">
+      <c r="C45" s="74"/>
+      <c r="D45" s="74"/>
+      <c r="E45" s="74"/>
+      <c r="F45" s="74"/>
+      <c r="G45" s="75" t="s">
         <v>77</v>
       </c>
-      <c r="H45" s="54"/>
-      <c r="I45" s="54"/>
-      <c r="J45" s="54"/>
-      <c r="K45" s="54"/>
-      <c r="L45" s="74"/>
-      <c r="M45" s="75"/>
+      <c r="H45" s="75"/>
+      <c r="I45" s="75"/>
+      <c r="J45" s="75"/>
+      <c r="K45" s="75"/>
+      <c r="L45" s="78"/>
+      <c r="M45" s="79"/>
       <c r="N45" s="32"/>
       <c r="O45"/>
       <c r="P45"/>
     </row>
     <row r="46" spans="1:16">
       <c r="A46" s="32"/>
-      <c r="B46" s="55" t="s">
+      <c r="B46" s="72" t="s">
         <v>78</v>
       </c>
-      <c r="C46" s="55"/>
-      <c r="D46" s="55"/>
-      <c r="E46" s="55"/>
-      <c r="F46" s="55"/>
-      <c r="G46" s="56" t="s">
+      <c r="C46" s="72"/>
+      <c r="D46" s="72"/>
+      <c r="E46" s="72"/>
+      <c r="F46" s="72"/>
+      <c r="G46" s="73" t="s">
         <v>79</v>
       </c>
-      <c r="H46" s="56"/>
-      <c r="I46" s="56"/>
-      <c r="J46" s="56"/>
-      <c r="K46" s="56"/>
+      <c r="H46" s="73"/>
+      <c r="I46" s="73"/>
+      <c r="J46" s="73"/>
+      <c r="K46" s="73"/>
       <c r="L46" s="63"/>
-      <c r="M46" s="64"/>
+      <c r="M46" s="65"/>
       <c r="N46" s="32"/>
       <c r="O46"/>
       <c r="P46"/>
     </row>
     <row r="47" spans="1:16">
       <c r="A47" s="32"/>
-      <c r="B47" s="53" t="s">
+      <c r="B47" s="74" t="s">
         <v>80</v>
       </c>
-      <c r="C47" s="53"/>
-      <c r="D47" s="53"/>
-      <c r="E47" s="53"/>
-      <c r="F47" s="53"/>
-      <c r="G47" s="54" t="s">
+      <c r="C47" s="74"/>
+      <c r="D47" s="74"/>
+      <c r="E47" s="74"/>
+      <c r="F47" s="74"/>
+      <c r="G47" s="75" t="s">
         <v>81</v>
       </c>
-      <c r="H47" s="54"/>
-      <c r="I47" s="54"/>
-      <c r="J47" s="54"/>
-      <c r="K47" s="54"/>
+      <c r="H47" s="75"/>
+      <c r="I47" s="75"/>
+      <c r="J47" s="75"/>
+      <c r="K47" s="75"/>
       <c r="L47" s="63"/>
-      <c r="M47" s="64"/>
+      <c r="M47" s="65"/>
       <c r="N47" s="32"/>
       <c r="O47"/>
       <c r="P47"/>
     </row>
     <row r="48" spans="1:16">
       <c r="A48" s="32"/>
-      <c r="B48" s="66" t="s">
+      <c r="B48" s="57" t="s">
         <v>82</v>
       </c>
-      <c r="C48" s="67"/>
-      <c r="D48" s="67"/>
-      <c r="E48" s="67"/>
-      <c r="F48" s="68"/>
-      <c r="G48" s="69" t="s">
+      <c r="C48" s="58"/>
+      <c r="D48" s="58"/>
+      <c r="E48" s="58"/>
+      <c r="F48" s="59"/>
+      <c r="G48" s="60" t="s">
         <v>83</v>
       </c>
-      <c r="H48" s="70"/>
-      <c r="I48" s="70"/>
-      <c r="J48" s="70"/>
-      <c r="K48" s="71"/>
+      <c r="H48" s="61"/>
+      <c r="I48" s="61"/>
+      <c r="J48" s="61"/>
+      <c r="K48" s="62"/>
       <c r="L48" s="63"/>
-      <c r="M48" s="64"/>
+      <c r="M48" s="65"/>
       <c r="N48" s="32"/>
       <c r="O48"/>
       <c r="P48"/>
     </row>
     <row r="49" spans="1:16">
       <c r="A49" s="32"/>
-      <c r="B49" s="72" t="s">
+      <c r="B49" s="80" t="s">
         <v>84</v>
       </c>
-      <c r="C49" s="72"/>
-      <c r="D49" s="72"/>
-      <c r="E49" s="72"/>
-      <c r="F49" s="72"/>
-      <c r="G49" s="73" t="s">
+      <c r="C49" s="80"/>
+      <c r="D49" s="80"/>
+      <c r="E49" s="80"/>
+      <c r="F49" s="80"/>
+      <c r="G49" s="81" t="s">
         <v>85</v>
       </c>
-      <c r="H49" s="73"/>
-      <c r="I49" s="73"/>
-      <c r="J49" s="73"/>
-      <c r="K49" s="73"/>
+      <c r="H49" s="81"/>
+      <c r="I49" s="81"/>
+      <c r="J49" s="81"/>
+      <c r="K49" s="81"/>
       <c r="L49" s="63"/>
-      <c r="M49" s="64"/>
+      <c r="M49" s="65"/>
       <c r="N49" s="32"/>
       <c r="O49"/>
       <c r="P49"/>
     </row>
     <row r="50" spans="1:16">
       <c r="A50" s="32"/>
-      <c r="B50" s="59" t="s">
+      <c r="B50" s="82" t="s">
         <v>86</v>
       </c>
-      <c r="C50" s="60"/>
-      <c r="D50" s="60"/>
-      <c r="E50" s="60"/>
-      <c r="F50" s="61"/>
-      <c r="G50" s="62"/>
-      <c r="H50" s="60"/>
-      <c r="I50" s="60"/>
-      <c r="J50" s="60"/>
-      <c r="K50" s="61"/>
+      <c r="C50" s="83"/>
+      <c r="D50" s="83"/>
+      <c r="E50" s="83"/>
+      <c r="F50" s="84"/>
+      <c r="G50" s="85"/>
+      <c r="H50" s="83"/>
+      <c r="I50" s="83"/>
+      <c r="J50" s="83"/>
+      <c r="K50" s="84"/>
       <c r="L50" s="63"/>
-      <c r="M50" s="64"/>
+      <c r="M50" s="65"/>
       <c r="N50" s="32"/>
       <c r="O50"/>
       <c r="P50"/>
@@ -4417,18 +4417,18 @@
     </row>
     <row r="52" spans="1:16">
       <c r="A52" s="32"/>
-      <c r="B52" s="65" t="s">
+      <c r="B52" s="69" t="s">
         <v>87</v>
       </c>
-      <c r="C52" s="65"/>
-      <c r="D52" s="65"/>
-      <c r="E52" s="65"/>
-      <c r="F52" s="65"/>
-      <c r="G52" s="65"/>
-      <c r="H52" s="65"/>
-      <c r="I52" s="65"/>
-      <c r="J52" s="65"/>
-      <c r="K52" s="65"/>
+      <c r="C52" s="69"/>
+      <c r="D52" s="69"/>
+      <c r="E52" s="69"/>
+      <c r="F52" s="69"/>
+      <c r="G52" s="69"/>
+      <c r="H52" s="69"/>
+      <c r="I52" s="69"/>
+      <c r="J52" s="69"/>
+      <c r="K52" s="69"/>
       <c r="L52" s="32"/>
       <c r="M52"/>
       <c r="N52"/>
@@ -4437,20 +4437,20 @@
     </row>
     <row r="53" spans="1:16">
       <c r="A53" s="32"/>
-      <c r="B53" s="53" t="s">
+      <c r="B53" s="74" t="s">
         <v>88</v>
       </c>
-      <c r="C53" s="53"/>
-      <c r="D53" s="53"/>
-      <c r="E53" s="53"/>
-      <c r="F53" s="53"/>
-      <c r="G53" s="54" t="s">
+      <c r="C53" s="74"/>
+      <c r="D53" s="74"/>
+      <c r="E53" s="74"/>
+      <c r="F53" s="74"/>
+      <c r="G53" s="75" t="s">
         <v>89</v>
       </c>
-      <c r="H53" s="54"/>
-      <c r="I53" s="54"/>
-      <c r="J53" s="54"/>
-      <c r="K53" s="54"/>
+      <c r="H53" s="75"/>
+      <c r="I53" s="75"/>
+      <c r="J53" s="75"/>
+      <c r="K53" s="75"/>
       <c r="L53" s="32"/>
       <c r="M53"/>
       <c r="N53"/>
@@ -4459,20 +4459,20 @@
     </row>
     <row r="54" spans="1:16">
       <c r="A54" s="32"/>
-      <c r="B54" s="55" t="s">
+      <c r="B54" s="72" t="s">
         <v>90</v>
       </c>
-      <c r="C54" s="55"/>
-      <c r="D54" s="55"/>
-      <c r="E54" s="55"/>
-      <c r="F54" s="55"/>
-      <c r="G54" s="56">
+      <c r="C54" s="72"/>
+      <c r="D54" s="72"/>
+      <c r="E54" s="72"/>
+      <c r="F54" s="72"/>
+      <c r="G54" s="73">
         <v>1349</v>
       </c>
-      <c r="H54" s="56"/>
-      <c r="I54" s="56"/>
-      <c r="J54" s="56"/>
-      <c r="K54" s="56"/>
+      <c r="H54" s="73"/>
+      <c r="I54" s="73"/>
+      <c r="J54" s="73"/>
+      <c r="K54" s="73"/>
       <c r="L54" s="32"/>
       <c r="M54"/>
       <c r="N54"/>
@@ -4481,20 +4481,20 @@
     </row>
     <row r="55" spans="1:16">
       <c r="A55" s="32"/>
-      <c r="B55" s="53" t="s">
+      <c r="B55" s="74" t="s">
         <v>91</v>
       </c>
-      <c r="C55" s="53"/>
-      <c r="D55" s="53"/>
-      <c r="E55" s="53"/>
-      <c r="F55" s="53"/>
-      <c r="G55" s="54">
+      <c r="C55" s="74"/>
+      <c r="D55" s="74"/>
+      <c r="E55" s="74"/>
+      <c r="F55" s="74"/>
+      <c r="G55" s="75">
         <v>1555</v>
       </c>
-      <c r="H55" s="54"/>
-      <c r="I55" s="54"/>
-      <c r="J55" s="54"/>
-      <c r="K55" s="54"/>
+      <c r="H55" s="75"/>
+      <c r="I55" s="75"/>
+      <c r="J55" s="75"/>
+      <c r="K55" s="75"/>
       <c r="L55" s="32"/>
       <c r="M55"/>
       <c r="N55"/>
@@ -4503,20 +4503,20 @@
     </row>
     <row r="56" spans="1:16">
       <c r="A56" s="32"/>
-      <c r="B56" s="55" t="s">
+      <c r="B56" s="72" t="s">
         <v>92</v>
       </c>
-      <c r="C56" s="55"/>
-      <c r="D56" s="55"/>
-      <c r="E56" s="55"/>
-      <c r="F56" s="55"/>
-      <c r="G56" s="56" t="s">
+      <c r="C56" s="72"/>
+      <c r="D56" s="72"/>
+      <c r="E56" s="72"/>
+      <c r="F56" s="72"/>
+      <c r="G56" s="73" t="s">
         <v>93</v>
       </c>
-      <c r="H56" s="56"/>
-      <c r="I56" s="56"/>
-      <c r="J56" s="56"/>
-      <c r="K56" s="56"/>
+      <c r="H56" s="73"/>
+      <c r="I56" s="73"/>
+      <c r="J56" s="73"/>
+      <c r="K56" s="73"/>
       <c r="L56" s="32"/>
       <c r="M56"/>
       <c r="N56"/>
@@ -4525,20 +4525,20 @@
     </row>
     <row r="57" spans="1:16">
       <c r="A57" s="32"/>
-      <c r="B57" s="53" t="s">
+      <c r="B57" s="74" t="s">
         <v>94</v>
       </c>
-      <c r="C57" s="53"/>
-      <c r="D57" s="53"/>
-      <c r="E57" s="53"/>
-      <c r="F57" s="53"/>
-      <c r="G57" s="54" t="s">
+      <c r="C57" s="74"/>
+      <c r="D57" s="74"/>
+      <c r="E57" s="74"/>
+      <c r="F57" s="74"/>
+      <c r="G57" s="75" t="s">
         <v>95</v>
       </c>
-      <c r="H57" s="54"/>
-      <c r="I57" s="54"/>
-      <c r="J57" s="54"/>
-      <c r="K57" s="54"/>
+      <c r="H57" s="75"/>
+      <c r="I57" s="75"/>
+      <c r="J57" s="75"/>
+      <c r="K57" s="75"/>
       <c r="L57" s="32"/>
       <c r="M57"/>
       <c r="N57"/>
@@ -4547,20 +4547,20 @@
     </row>
     <row r="58" spans="1:16">
       <c r="A58" s="32"/>
-      <c r="B58" s="55" t="s">
+      <c r="B58" s="72" t="s">
         <v>96</v>
       </c>
-      <c r="C58" s="55"/>
-      <c r="D58" s="55"/>
-      <c r="E58" s="55"/>
-      <c r="F58" s="55"/>
-      <c r="G58" s="56" t="s">
+      <c r="C58" s="72"/>
+      <c r="D58" s="72"/>
+      <c r="E58" s="72"/>
+      <c r="F58" s="72"/>
+      <c r="G58" s="73" t="s">
         <v>97</v>
       </c>
-      <c r="H58" s="56"/>
-      <c r="I58" s="56"/>
-      <c r="J58" s="56"/>
-      <c r="K58" s="56"/>
+      <c r="H58" s="73"/>
+      <c r="I58" s="73"/>
+      <c r="J58" s="73"/>
+      <c r="K58" s="73"/>
       <c r="L58" s="32"/>
       <c r="M58"/>
       <c r="N58"/>
@@ -4569,20 +4569,20 @@
     </row>
     <row r="59" spans="1:16">
       <c r="A59" s="32"/>
-      <c r="B59" s="53" t="s">
+      <c r="B59" s="74" t="s">
         <v>98</v>
       </c>
-      <c r="C59" s="53"/>
-      <c r="D59" s="53"/>
-      <c r="E59" s="53"/>
-      <c r="F59" s="53"/>
-      <c r="G59" s="54" t="s">
+      <c r="C59" s="74"/>
+      <c r="D59" s="74"/>
+      <c r="E59" s="74"/>
+      <c r="F59" s="74"/>
+      <c r="G59" s="75" t="s">
         <v>99</v>
       </c>
-      <c r="H59" s="54"/>
-      <c r="I59" s="54"/>
-      <c r="J59" s="54"/>
-      <c r="K59" s="54"/>
+      <c r="H59" s="75"/>
+      <c r="I59" s="75"/>
+      <c r="J59" s="75"/>
+      <c r="K59" s="75"/>
       <c r="L59" s="32"/>
       <c r="M59"/>
       <c r="N59"/>
@@ -4591,20 +4591,20 @@
     </row>
     <row r="60" spans="1:16">
       <c r="A60" s="32"/>
-      <c r="B60" s="55" t="s">
+      <c r="B60" s="72" t="s">
         <v>100</v>
       </c>
-      <c r="C60" s="55"/>
-      <c r="D60" s="55"/>
-      <c r="E60" s="55"/>
-      <c r="F60" s="55"/>
-      <c r="G60" s="56" t="s">
+      <c r="C60" s="72"/>
+      <c r="D60" s="72"/>
+      <c r="E60" s="72"/>
+      <c r="F60" s="72"/>
+      <c r="G60" s="73" t="s">
         <v>101</v>
       </c>
-      <c r="H60" s="56"/>
-      <c r="I60" s="56"/>
-      <c r="J60" s="56"/>
-      <c r="K60" s="56"/>
+      <c r="H60" s="73"/>
+      <c r="I60" s="73"/>
+      <c r="J60" s="73"/>
+      <c r="K60" s="73"/>
       <c r="L60" s="32"/>
       <c r="M60"/>
       <c r="N60"/>
@@ -4613,20 +4613,20 @@
     </row>
     <row r="61" spans="1:16">
       <c r="A61" s="32"/>
-      <c r="B61" s="53" t="s">
+      <c r="B61" s="74" t="s">
         <v>102</v>
       </c>
-      <c r="C61" s="53"/>
-      <c r="D61" s="53"/>
-      <c r="E61" s="53"/>
-      <c r="F61" s="53"/>
-      <c r="G61" s="54" t="s">
+      <c r="C61" s="74"/>
+      <c r="D61" s="74"/>
+      <c r="E61" s="74"/>
+      <c r="F61" s="74"/>
+      <c r="G61" s="75" t="s">
         <v>103</v>
       </c>
-      <c r="H61" s="54"/>
-      <c r="I61" s="54"/>
-      <c r="J61" s="54"/>
-      <c r="K61" s="54"/>
+      <c r="H61" s="75"/>
+      <c r="I61" s="75"/>
+      <c r="J61" s="75"/>
+      <c r="K61" s="75"/>
       <c r="L61" s="32"/>
       <c r="M61"/>
       <c r="N61"/>
@@ -4635,20 +4635,20 @@
     </row>
     <row r="62" spans="1:16">
       <c r="A62" s="32"/>
-      <c r="B62" s="55" t="s">
+      <c r="B62" s="72" t="s">
         <v>104</v>
       </c>
-      <c r="C62" s="55"/>
-      <c r="D62" s="55"/>
-      <c r="E62" s="55"/>
-      <c r="F62" s="55"/>
-      <c r="G62" s="56" t="s">
+      <c r="C62" s="72"/>
+      <c r="D62" s="72"/>
+      <c r="E62" s="72"/>
+      <c r="F62" s="72"/>
+      <c r="G62" s="73" t="s">
         <v>105</v>
       </c>
-      <c r="H62" s="56"/>
-      <c r="I62" s="56"/>
-      <c r="J62" s="56"/>
-      <c r="K62" s="56"/>
+      <c r="H62" s="73"/>
+      <c r="I62" s="73"/>
+      <c r="J62" s="73"/>
+      <c r="K62" s="73"/>
       <c r="L62" s="32"/>
       <c r="M62"/>
       <c r="N62"/>
@@ -4657,20 +4657,20 @@
     </row>
     <row r="63" spans="1:16">
       <c r="A63" s="32"/>
-      <c r="B63" s="53" t="s">
+      <c r="B63" s="74" t="s">
         <v>106</v>
       </c>
-      <c r="C63" s="53"/>
-      <c r="D63" s="53"/>
-      <c r="E63" s="53"/>
-      <c r="F63" s="53"/>
-      <c r="G63" s="54" t="s">
+      <c r="C63" s="74"/>
+      <c r="D63" s="74"/>
+      <c r="E63" s="74"/>
+      <c r="F63" s="74"/>
+      <c r="G63" s="75" t="s">
         <v>107</v>
       </c>
-      <c r="H63" s="54"/>
-      <c r="I63" s="54"/>
-      <c r="J63" s="54"/>
-      <c r="K63" s="54"/>
+      <c r="H63" s="75"/>
+      <c r="I63" s="75"/>
+      <c r="J63" s="75"/>
+      <c r="K63" s="75"/>
       <c r="L63" s="32"/>
       <c r="M63"/>
       <c r="N63"/>
@@ -4679,20 +4679,20 @@
     </row>
     <row r="64" spans="1:16">
       <c r="A64" s="32"/>
-      <c r="B64" s="55" t="s">
+      <c r="B64" s="72" t="s">
         <v>108</v>
       </c>
-      <c r="C64" s="55"/>
-      <c r="D64" s="55"/>
-      <c r="E64" s="55"/>
-      <c r="F64" s="55"/>
-      <c r="G64" s="56">
+      <c r="C64" s="72"/>
+      <c r="D64" s="72"/>
+      <c r="E64" s="72"/>
+      <c r="F64" s="72"/>
+      <c r="G64" s="73">
         <v>166</v>
       </c>
-      <c r="H64" s="56"/>
-      <c r="I64" s="56"/>
-      <c r="J64" s="56"/>
-      <c r="K64" s="56"/>
+      <c r="H64" s="73"/>
+      <c r="I64" s="73"/>
+      <c r="J64" s="73"/>
+      <c r="K64" s="73"/>
       <c r="L64" s="32"/>
       <c r="M64"/>
       <c r="N64"/>
@@ -4701,20 +4701,20 @@
     </row>
     <row r="65" spans="1:16">
       <c r="A65" s="32"/>
-      <c r="B65" s="53" t="s">
+      <c r="B65" s="74" t="s">
         <v>109</v>
       </c>
-      <c r="C65" s="53"/>
-      <c r="D65" s="53"/>
-      <c r="E65" s="53"/>
-      <c r="F65" s="53"/>
-      <c r="G65" s="54" t="s">
+      <c r="C65" s="74"/>
+      <c r="D65" s="74"/>
+      <c r="E65" s="74"/>
+      <c r="F65" s="74"/>
+      <c r="G65" s="75" t="s">
         <v>110</v>
       </c>
-      <c r="H65" s="54"/>
-      <c r="I65" s="54"/>
-      <c r="J65" s="54"/>
-      <c r="K65" s="54"/>
+      <c r="H65" s="75"/>
+      <c r="I65" s="75"/>
+      <c r="J65" s="75"/>
+      <c r="K65" s="75"/>
       <c r="L65" s="32"/>
       <c r="M65"/>
       <c r="N65"/>
@@ -4723,20 +4723,20 @@
     </row>
     <row r="66" spans="1:16">
       <c r="A66" s="32"/>
-      <c r="B66" s="55" t="s">
+      <c r="B66" s="72" t="s">
         <v>111</v>
       </c>
-      <c r="C66" s="55"/>
-      <c r="D66" s="55"/>
-      <c r="E66" s="55"/>
-      <c r="F66" s="55"/>
-      <c r="G66" s="56" t="s">
+      <c r="C66" s="72"/>
+      <c r="D66" s="72"/>
+      <c r="E66" s="72"/>
+      <c r="F66" s="72"/>
+      <c r="G66" s="73" t="s">
         <v>112</v>
       </c>
-      <c r="H66" s="56"/>
-      <c r="I66" s="56"/>
-      <c r="J66" s="56"/>
-      <c r="K66" s="56"/>
+      <c r="H66" s="73"/>
+      <c r="I66" s="73"/>
+      <c r="J66" s="73"/>
+      <c r="K66" s="73"/>
       <c r="L66" s="32"/>
       <c r="M66"/>
       <c r="N66"/>
@@ -4745,20 +4745,20 @@
     </row>
     <row r="67" spans="1:16">
       <c r="A67" s="32"/>
-      <c r="B67" s="53" t="s">
+      <c r="B67" s="74" t="s">
         <v>113</v>
       </c>
-      <c r="C67" s="53"/>
-      <c r="D67" s="53"/>
-      <c r="E67" s="53"/>
-      <c r="F67" s="53"/>
-      <c r="G67" s="54" t="s">
+      <c r="C67" s="74"/>
+      <c r="D67" s="74"/>
+      <c r="E67" s="74"/>
+      <c r="F67" s="74"/>
+      <c r="G67" s="75" t="s">
         <v>114</v>
       </c>
-      <c r="H67" s="54"/>
-      <c r="I67" s="54"/>
-      <c r="J67" s="54"/>
-      <c r="K67" s="54"/>
+      <c r="H67" s="75"/>
+      <c r="I67" s="75"/>
+      <c r="J67" s="75"/>
+      <c r="K67" s="75"/>
       <c r="L67" s="32"/>
       <c r="M67"/>
       <c r="N67"/>
@@ -4767,20 +4767,20 @@
     </row>
     <row r="68" spans="1:16">
       <c r="A68" s="32"/>
-      <c r="B68" s="55" t="s">
+      <c r="B68" s="72" t="s">
         <v>115</v>
       </c>
-      <c r="C68" s="55"/>
-      <c r="D68" s="55"/>
-      <c r="E68" s="55"/>
-      <c r="F68" s="55"/>
-      <c r="G68" s="56" t="s">
+      <c r="C68" s="72"/>
+      <c r="D68" s="72"/>
+      <c r="E68" s="72"/>
+      <c r="F68" s="72"/>
+      <c r="G68" s="73" t="s">
         <v>116</v>
       </c>
-      <c r="H68" s="56"/>
-      <c r="I68" s="56"/>
-      <c r="J68" s="56"/>
-      <c r="K68" s="56"/>
+      <c r="H68" s="73"/>
+      <c r="I68" s="73"/>
+      <c r="J68" s="73"/>
+      <c r="K68" s="73"/>
       <c r="L68" s="32"/>
       <c r="M68"/>
       <c r="N68"/>
@@ -4789,20 +4789,20 @@
     </row>
     <row r="69" spans="1:16">
       <c r="A69" s="32"/>
-      <c r="B69" s="53" t="s">
+      <c r="B69" s="74" t="s">
         <v>117</v>
       </c>
-      <c r="C69" s="53"/>
-      <c r="D69" s="53"/>
-      <c r="E69" s="53"/>
-      <c r="F69" s="53"/>
-      <c r="G69" s="54" t="s">
+      <c r="C69" s="74"/>
+      <c r="D69" s="74"/>
+      <c r="E69" s="74"/>
+      <c r="F69" s="74"/>
+      <c r="G69" s="75" t="s">
         <v>118</v>
       </c>
-      <c r="H69" s="54"/>
-      <c r="I69" s="54"/>
-      <c r="J69" s="54"/>
-      <c r="K69" s="54"/>
+      <c r="H69" s="75"/>
+      <c r="I69" s="75"/>
+      <c r="J69" s="75"/>
+      <c r="K69" s="75"/>
       <c r="L69" s="32"/>
       <c r="M69"/>
       <c r="N69"/>
@@ -4811,20 +4811,20 @@
     </row>
     <row r="70" spans="1:16">
       <c r="A70" s="32"/>
-      <c r="B70" s="55" t="s">
+      <c r="B70" s="72" t="s">
         <v>119</v>
       </c>
-      <c r="C70" s="55"/>
-      <c r="D70" s="55"/>
-      <c r="E70" s="55"/>
-      <c r="F70" s="55"/>
-      <c r="G70" s="56" t="s">
+      <c r="C70" s="72"/>
+      <c r="D70" s="72"/>
+      <c r="E70" s="72"/>
+      <c r="F70" s="72"/>
+      <c r="G70" s="73" t="s">
         <v>120</v>
       </c>
-      <c r="H70" s="56"/>
-      <c r="I70" s="56"/>
-      <c r="J70" s="56"/>
-      <c r="K70" s="56"/>
+      <c r="H70" s="73"/>
+      <c r="I70" s="73"/>
+      <c r="J70" s="73"/>
+      <c r="K70" s="73"/>
       <c r="L70" s="32"/>
       <c r="M70"/>
       <c r="N70"/>
@@ -4833,20 +4833,20 @@
     </row>
     <row r="71" spans="1:16">
       <c r="A71" s="32"/>
-      <c r="B71" s="53" t="s">
+      <c r="B71" s="74" t="s">
         <v>121</v>
       </c>
-      <c r="C71" s="53"/>
-      <c r="D71" s="53"/>
-      <c r="E71" s="53"/>
-      <c r="F71" s="53"/>
-      <c r="G71" s="54" t="s">
+      <c r="C71" s="74"/>
+      <c r="D71" s="74"/>
+      <c r="E71" s="74"/>
+      <c r="F71" s="74"/>
+      <c r="G71" s="75" t="s">
         <v>122</v>
       </c>
-      <c r="H71" s="54"/>
-      <c r="I71" s="54"/>
-      <c r="J71" s="54"/>
-      <c r="K71" s="54"/>
+      <c r="H71" s="75"/>
+      <c r="I71" s="75"/>
+      <c r="J71" s="75"/>
+      <c r="K71" s="75"/>
       <c r="L71" s="32"/>
       <c r="M71"/>
       <c r="N71"/>
@@ -4855,20 +4855,20 @@
     </row>
     <row r="72" spans="1:16">
       <c r="A72" s="32"/>
-      <c r="B72" s="55" t="s">
+      <c r="B72" s="72" t="s">
         <v>123</v>
       </c>
-      <c r="C72" s="55"/>
-      <c r="D72" s="55"/>
-      <c r="E72" s="55"/>
-      <c r="F72" s="55"/>
-      <c r="G72" s="56" t="s">
+      <c r="C72" s="72"/>
+      <c r="D72" s="72"/>
+      <c r="E72" s="72"/>
+      <c r="F72" s="72"/>
+      <c r="G72" s="73" t="s">
         <v>124</v>
       </c>
-      <c r="H72" s="56"/>
-      <c r="I72" s="56"/>
-      <c r="J72" s="56"/>
-      <c r="K72" s="56"/>
+      <c r="H72" s="73"/>
+      <c r="I72" s="73"/>
+      <c r="J72" s="73"/>
+      <c r="K72" s="73"/>
       <c r="L72" s="32"/>
       <c r="M72"/>
       <c r="N72"/>
@@ -4877,20 +4877,20 @@
     </row>
     <row r="73" spans="1:16">
       <c r="A73" s="32"/>
-      <c r="B73" s="53" t="s">
+      <c r="B73" s="74" t="s">
         <v>125</v>
       </c>
-      <c r="C73" s="53"/>
-      <c r="D73" s="53"/>
-      <c r="E73" s="53"/>
-      <c r="F73" s="53"/>
-      <c r="G73" s="57" t="s">
+      <c r="C73" s="74"/>
+      <c r="D73" s="74"/>
+      <c r="E73" s="74"/>
+      <c r="F73" s="74"/>
+      <c r="G73" s="87" t="s">
         <v>126</v>
       </c>
-      <c r="H73" s="57"/>
-      <c r="I73" s="57"/>
-      <c r="J73" s="57"/>
-      <c r="K73" s="57"/>
+      <c r="H73" s="87"/>
+      <c r="I73" s="87"/>
+      <c r="J73" s="87"/>
+      <c r="K73" s="87"/>
       <c r="L73" s="32"/>
       <c r="M73"/>
       <c r="N73"/>
@@ -4899,20 +4899,20 @@
     </row>
     <row r="74" spans="1:16">
       <c r="A74" s="32"/>
-      <c r="B74" s="55" t="s">
+      <c r="B74" s="72" t="s">
         <v>127</v>
       </c>
-      <c r="C74" s="55"/>
-      <c r="D74" s="55"/>
-      <c r="E74" s="55"/>
-      <c r="F74" s="55"/>
-      <c r="G74" s="58" t="s">
+      <c r="C74" s="72"/>
+      <c r="D74" s="72"/>
+      <c r="E74" s="72"/>
+      <c r="F74" s="72"/>
+      <c r="G74" s="88" t="s">
         <v>128</v>
       </c>
-      <c r="H74" s="58"/>
-      <c r="I74" s="58"/>
-      <c r="J74" s="58"/>
-      <c r="K74" s="58"/>
+      <c r="H74" s="88"/>
+      <c r="I74" s="88"/>
+      <c r="J74" s="88"/>
+      <c r="K74" s="88"/>
       <c r="L74" s="32"/>
       <c r="M74"/>
       <c r="N74"/>
@@ -5049,148 +5049,6 @@
     <row r="120" customFormat="1"/>
   </sheetData>
   <mergeCells count="166">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="B9:K9"/>
-    <mergeCell ref="B12:K12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="E13:G13"/>
-    <mergeCell ref="H13:K13"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="E14:G14"/>
-    <mergeCell ref="H14:K14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="H15:K15"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="E16:G16"/>
-    <mergeCell ref="H16:K16"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="E17:G17"/>
-    <mergeCell ref="H17:K17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="H18:K18"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="H19:K19"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="H20:K20"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="H21:K21"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="H22:K22"/>
-    <mergeCell ref="B24:K24"/>
-    <mergeCell ref="B25:F25"/>
-    <mergeCell ref="G25:K25"/>
-    <mergeCell ref="L25:M25"/>
-    <mergeCell ref="B26:F26"/>
-    <mergeCell ref="G26:K26"/>
-    <mergeCell ref="L26:M26"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="G27:K27"/>
-    <mergeCell ref="L27:M27"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="G28:K28"/>
-    <mergeCell ref="L28:M28"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="G29:K29"/>
-    <mergeCell ref="L29:M29"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="G30:K30"/>
-    <mergeCell ref="L30:M30"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="G31:K31"/>
-    <mergeCell ref="L31:M31"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="G32:K32"/>
-    <mergeCell ref="L32:M32"/>
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="G33:K33"/>
-    <mergeCell ref="L33:M33"/>
-    <mergeCell ref="B34:F34"/>
-    <mergeCell ref="G34:K34"/>
-    <mergeCell ref="L34:M34"/>
-    <mergeCell ref="B35:F35"/>
-    <mergeCell ref="G35:K35"/>
-    <mergeCell ref="L35:M35"/>
-    <mergeCell ref="B36:F36"/>
-    <mergeCell ref="G36:K36"/>
-    <mergeCell ref="L36:M36"/>
-    <mergeCell ref="B37:F37"/>
-    <mergeCell ref="G37:K37"/>
-    <mergeCell ref="L37:M37"/>
-    <mergeCell ref="B38:F38"/>
-    <mergeCell ref="G38:K38"/>
-    <mergeCell ref="L38:M38"/>
-    <mergeCell ref="B39:F39"/>
-    <mergeCell ref="G39:K39"/>
-    <mergeCell ref="L39:M39"/>
-    <mergeCell ref="B40:F40"/>
-    <mergeCell ref="G40:K40"/>
-    <mergeCell ref="L40:M40"/>
-    <mergeCell ref="B41:F41"/>
-    <mergeCell ref="G41:K41"/>
-    <mergeCell ref="L41:M41"/>
-    <mergeCell ref="B42:F42"/>
-    <mergeCell ref="G42:K42"/>
-    <mergeCell ref="L42:M42"/>
-    <mergeCell ref="B43:F43"/>
-    <mergeCell ref="G43:K43"/>
-    <mergeCell ref="L43:M43"/>
-    <mergeCell ref="B44:F44"/>
-    <mergeCell ref="G44:K44"/>
-    <mergeCell ref="L44:M44"/>
-    <mergeCell ref="B45:F45"/>
-    <mergeCell ref="G45:K45"/>
-    <mergeCell ref="L45:M45"/>
-    <mergeCell ref="B46:F46"/>
-    <mergeCell ref="G46:K46"/>
-    <mergeCell ref="L46:M46"/>
-    <mergeCell ref="B47:F47"/>
-    <mergeCell ref="G47:K47"/>
-    <mergeCell ref="L47:M47"/>
-    <mergeCell ref="B48:F48"/>
-    <mergeCell ref="G48:K48"/>
-    <mergeCell ref="L48:M48"/>
-    <mergeCell ref="B49:F49"/>
-    <mergeCell ref="G49:K49"/>
-    <mergeCell ref="L49:M49"/>
-    <mergeCell ref="B50:F50"/>
-    <mergeCell ref="G50:K50"/>
-    <mergeCell ref="L50:M50"/>
-    <mergeCell ref="B52:K52"/>
-    <mergeCell ref="B53:F53"/>
-    <mergeCell ref="G53:K53"/>
-    <mergeCell ref="B54:F54"/>
-    <mergeCell ref="G54:K54"/>
-    <mergeCell ref="B55:F55"/>
-    <mergeCell ref="G55:K55"/>
-    <mergeCell ref="B56:F56"/>
-    <mergeCell ref="G56:K56"/>
-    <mergeCell ref="B57:F57"/>
-    <mergeCell ref="G57:K57"/>
-    <mergeCell ref="B58:F58"/>
-    <mergeCell ref="G58:K58"/>
-    <mergeCell ref="B59:F59"/>
-    <mergeCell ref="G59:K59"/>
-    <mergeCell ref="B60:F60"/>
-    <mergeCell ref="G60:K60"/>
-    <mergeCell ref="G69:K69"/>
-    <mergeCell ref="B70:F70"/>
-    <mergeCell ref="G70:K70"/>
-    <mergeCell ref="B61:F61"/>
-    <mergeCell ref="G61:K61"/>
-    <mergeCell ref="B62:F62"/>
-    <mergeCell ref="G62:K62"/>
-    <mergeCell ref="B63:F63"/>
-    <mergeCell ref="G63:K63"/>
-    <mergeCell ref="B64:F64"/>
-    <mergeCell ref="G64:K64"/>
-    <mergeCell ref="B65:F65"/>
-    <mergeCell ref="G65:K65"/>
     <mergeCell ref="B77:F77"/>
     <mergeCell ref="G77:K77"/>
     <mergeCell ref="B78:F78"/>
@@ -5215,6 +5073,148 @@
     <mergeCell ref="B68:F68"/>
     <mergeCell ref="G68:K68"/>
     <mergeCell ref="B69:F69"/>
+    <mergeCell ref="G69:K69"/>
+    <mergeCell ref="B70:F70"/>
+    <mergeCell ref="G70:K70"/>
+    <mergeCell ref="B61:F61"/>
+    <mergeCell ref="G61:K61"/>
+    <mergeCell ref="B62:F62"/>
+    <mergeCell ref="G62:K62"/>
+    <mergeCell ref="B63:F63"/>
+    <mergeCell ref="G63:K63"/>
+    <mergeCell ref="B64:F64"/>
+    <mergeCell ref="G64:K64"/>
+    <mergeCell ref="B65:F65"/>
+    <mergeCell ref="G65:K65"/>
+    <mergeCell ref="B56:F56"/>
+    <mergeCell ref="G56:K56"/>
+    <mergeCell ref="B57:F57"/>
+    <mergeCell ref="G57:K57"/>
+    <mergeCell ref="B58:F58"/>
+    <mergeCell ref="G58:K58"/>
+    <mergeCell ref="B59:F59"/>
+    <mergeCell ref="G59:K59"/>
+    <mergeCell ref="B60:F60"/>
+    <mergeCell ref="G60:K60"/>
+    <mergeCell ref="B50:F50"/>
+    <mergeCell ref="G50:K50"/>
+    <mergeCell ref="L50:M50"/>
+    <mergeCell ref="B52:K52"/>
+    <mergeCell ref="B53:F53"/>
+    <mergeCell ref="G53:K53"/>
+    <mergeCell ref="B54:F54"/>
+    <mergeCell ref="G54:K54"/>
+    <mergeCell ref="B55:F55"/>
+    <mergeCell ref="G55:K55"/>
+    <mergeCell ref="B47:F47"/>
+    <mergeCell ref="G47:K47"/>
+    <mergeCell ref="L47:M47"/>
+    <mergeCell ref="B48:F48"/>
+    <mergeCell ref="G48:K48"/>
+    <mergeCell ref="L48:M48"/>
+    <mergeCell ref="B49:F49"/>
+    <mergeCell ref="G49:K49"/>
+    <mergeCell ref="L49:M49"/>
+    <mergeCell ref="B44:F44"/>
+    <mergeCell ref="G44:K44"/>
+    <mergeCell ref="L44:M44"/>
+    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="G45:K45"/>
+    <mergeCell ref="L45:M45"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="G46:K46"/>
+    <mergeCell ref="L46:M46"/>
+    <mergeCell ref="B41:F41"/>
+    <mergeCell ref="G41:K41"/>
+    <mergeCell ref="L41:M41"/>
+    <mergeCell ref="B42:F42"/>
+    <mergeCell ref="G42:K42"/>
+    <mergeCell ref="L42:M42"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="G43:K43"/>
+    <mergeCell ref="L43:M43"/>
+    <mergeCell ref="B38:F38"/>
+    <mergeCell ref="G38:K38"/>
+    <mergeCell ref="L38:M38"/>
+    <mergeCell ref="B39:F39"/>
+    <mergeCell ref="G39:K39"/>
+    <mergeCell ref="L39:M39"/>
+    <mergeCell ref="B40:F40"/>
+    <mergeCell ref="G40:K40"/>
+    <mergeCell ref="L40:M40"/>
+    <mergeCell ref="B35:F35"/>
+    <mergeCell ref="G35:K35"/>
+    <mergeCell ref="L35:M35"/>
+    <mergeCell ref="B36:F36"/>
+    <mergeCell ref="G36:K36"/>
+    <mergeCell ref="L36:M36"/>
+    <mergeCell ref="B37:F37"/>
+    <mergeCell ref="G37:K37"/>
+    <mergeCell ref="L37:M37"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="G32:K32"/>
+    <mergeCell ref="L32:M32"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="G33:K33"/>
+    <mergeCell ref="L33:M33"/>
+    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="G34:K34"/>
+    <mergeCell ref="L34:M34"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="G29:K29"/>
+    <mergeCell ref="L29:M29"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="G30:K30"/>
+    <mergeCell ref="L30:M30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="G31:K31"/>
+    <mergeCell ref="L31:M31"/>
+    <mergeCell ref="L25:M25"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="G26:K26"/>
+    <mergeCell ref="L26:M26"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="G27:K27"/>
+    <mergeCell ref="L27:M27"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="G28:K28"/>
+    <mergeCell ref="L28:M28"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="H21:K21"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="H22:K22"/>
+    <mergeCell ref="B24:K24"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="G25:K25"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="H18:K18"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="H19:K19"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="H20:K20"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="H15:K15"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="H16:K16"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="E17:G17"/>
+    <mergeCell ref="H17:K17"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="B9:K9"/>
+    <mergeCell ref="B12:K12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="H13:K13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="H14:K14"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="L30" r:id="rId1" tooltip="mailto:ccfi_sugbu@yahoo.com" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -6658,7 +6658,7 @@
         <v>449</v>
       </c>
       <c r="D2" s="35" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>132</v>
@@ -6700,7 +6700,7 @@
         <v>458</v>
       </c>
       <c r="D3" s="36" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>459</v>
@@ -6734,7 +6734,7 @@
         <v>463</v>
       </c>
       <c r="D4" s="36" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>464</v>
@@ -6776,7 +6776,7 @@
         <v>470</v>
       </c>
       <c r="D5" s="36" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>471</v>
@@ -6818,7 +6818,7 @@
         <v>477</v>
       </c>
       <c r="D6" s="36" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>478</v>
@@ -6860,10 +6860,10 @@
         <v>484</v>
       </c>
       <c r="D7" s="36" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>485</v>
@@ -6902,10 +6902,10 @@
         <v>491</v>
       </c>
       <c r="D8" s="36" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>492</v>
@@ -6923,7 +6923,7 @@
         <v>30</v>
       </c>
       <c r="K8" s="45" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="L8" s="6">
         <v>2</v>
@@ -6944,7 +6944,7 @@
         <v>497</v>
       </c>
       <c r="D9" s="36" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>498</v>
@@ -6965,7 +6965,7 @@
         <v>30</v>
       </c>
       <c r="K9" s="46" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="L9" s="3">
         <v>30</v>
@@ -6986,7 +6986,7 @@
         <v>503</v>
       </c>
       <c r="D10" s="36" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>504</v>
@@ -7020,7 +7020,7 @@
         <v>510</v>
       </c>
       <c r="D11" s="36" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>511</v>
@@ -7054,10 +7054,10 @@
         <v>517</v>
       </c>
       <c r="D12" s="36" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>518</v>
@@ -7088,7 +7088,7 @@
         <v>522</v>
       </c>
       <c r="D13" s="36" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>511</v>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="C14" s="90"/>
       <c r="D14" s="92" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="E14" s="90" t="s">
         <v>528</v>
@@ -7184,7 +7184,7 @@
         <v>537</v>
       </c>
       <c r="D16" s="36" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>538</v>
@@ -7205,7 +7205,7 @@
         <v>20</v>
       </c>
       <c r="K16" s="47" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="L16" s="3"/>
       <c r="M16" s="3">
@@ -7253,7 +7253,7 @@
         <v>548</v>
       </c>
       <c r="D18" s="36" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>549</v>
@@ -7287,7 +7287,7 @@
         <v>554</v>
       </c>
       <c r="D19" s="36" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>555</v>
@@ -7308,7 +7308,7 @@
         <v>21</v>
       </c>
       <c r="K19" s="45" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="L19" s="6">
         <v>6</v>
@@ -7329,7 +7329,7 @@
         <v>560</v>
       </c>
       <c r="D20" s="36" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>561</v>
@@ -7363,7 +7363,7 @@
         <v>566</v>
       </c>
       <c r="D21" s="36" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>567</v>
@@ -7397,7 +7397,7 @@
         <v>573</v>
       </c>
       <c r="D22" s="36" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>574</v>
@@ -7418,7 +7418,7 @@
         <v>25</v>
       </c>
       <c r="K22" s="46" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="L22" s="3">
         <v>12</v>
@@ -7436,10 +7436,10 @@
         <v>579</v>
       </c>
       <c r="C23" s="37" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D23" s="36" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>580</v>
@@ -7460,7 +7460,7 @@
         <v>21</v>
       </c>
       <c r="K23" s="50" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="L23" s="6">
         <v>7</v>
@@ -7481,7 +7481,7 @@
         <v>586</v>
       </c>
       <c r="D24" s="36" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>587</v>
@@ -7515,7 +7515,7 @@
         <v>592</v>
       </c>
       <c r="D25" s="36" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>593</v>
@@ -7555,7 +7555,7 @@
         <v>600</v>
       </c>
       <c r="D26" s="36" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>528</v>
@@ -7576,7 +7576,7 @@
         <v>22</v>
       </c>
       <c r="K26" s="46" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="L26" s="3">
         <v>0</v>
@@ -7597,7 +7597,7 @@
         <v>605</v>
       </c>
       <c r="D27" s="36" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>606</v>
@@ -7639,10 +7639,10 @@
         <v>612</v>
       </c>
       <c r="D28" s="36" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>613</v>
@@ -7681,7 +7681,7 @@
         <v>470</v>
       </c>
       <c r="D29" s="36" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="E29" s="6" t="s">
         <v>618</v>
@@ -7723,7 +7723,7 @@
         <v>624</v>
       </c>
       <c r="D30" s="36" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>625</v>
@@ -7757,10 +7757,10 @@
         <v>631</v>
       </c>
       <c r="D31" s="36" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="F31" s="6" t="s">
         <v>632</v>
@@ -7799,7 +7799,7 @@
         <v>637</v>
       </c>
       <c r="D32" s="36" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>638</v>
@@ -7833,7 +7833,7 @@
         <v>642</v>
       </c>
       <c r="D33" s="36" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="E33" s="6" t="s">
         <v>643</v>
@@ -7854,7 +7854,7 @@
         <v>68</v>
       </c>
       <c r="K33" s="50" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="L33" s="6">
         <v>28</v>
@@ -7875,7 +7875,7 @@
         <v>649</v>
       </c>
       <c r="D34" s="36" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>650</v>
@@ -7917,7 +7917,7 @@
         <v>659</v>
       </c>
       <c r="D35" s="36" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="E35" s="6" t="s">
         <v>660</v>
@@ -7938,7 +7938,7 @@
         <v>14</v>
       </c>
       <c r="K35" s="50" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="L35" s="6">
         <v>14</v>
@@ -7959,7 +7959,7 @@
         <v>666</v>
       </c>
       <c r="D36" s="36" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>667</v>
@@ -7978,7 +7978,7 @@
         <v>25</v>
       </c>
       <c r="K36" s="46" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="L36" s="3">
         <v>23</v>
@@ -7999,20 +7999,20 @@
         <v>672</v>
       </c>
       <c r="D37" s="92" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="E37" s="90" t="s">
+        <v>728</v>
+      </c>
+      <c r="F37" s="6" t="s">
         <v>673</v>
-      </c>
-      <c r="F37" s="6" t="s">
-        <v>674</v>
       </c>
       <c r="G37" s="6"/>
       <c r="H37" s="34" t="s">
+        <v>674</v>
+      </c>
+      <c r="I37" s="7" t="s">
         <v>675</v>
-      </c>
-      <c r="I37" s="7" t="s">
-        <v>676</v>
       </c>
       <c r="J37" s="6"/>
       <c r="K37" s="44"/>
@@ -8027,14 +8027,14 @@
       <c r="D38" s="92"/>
       <c r="E38" s="90"/>
       <c r="F38" s="6" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="G38" s="6"/>
       <c r="H38" s="34" t="s">
+        <v>677</v>
+      </c>
+      <c r="I38" s="7" t="s">
         <v>678</v>
-      </c>
-      <c r="I38" s="7" t="s">
-        <v>679</v>
       </c>
       <c r="J38" s="6"/>
       <c r="K38" s="44"/>
@@ -8047,26 +8047,26 @@
         <v>36</v>
       </c>
       <c r="B39" s="3" t="s">
+        <v>679</v>
+      </c>
+      <c r="C39" s="3" t="s">
         <v>680</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="D39" s="36" t="s">
+        <v>701</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>724</v>
+      </c>
+      <c r="F39" s="3" t="s">
         <v>681</v>
-      </c>
-      <c r="D39" s="36" t="s">
-        <v>702</v>
-      </c>
-      <c r="E39" s="3" t="s">
-        <v>725</v>
-      </c>
-      <c r="F39" s="3" t="s">
-        <v>682</v>
       </c>
       <c r="G39" s="3"/>
       <c r="H39" s="33" t="s">
+        <v>682</v>
+      </c>
+      <c r="I39" s="4" t="s">
         <v>683</v>
-      </c>
-      <c r="I39" s="4" t="s">
-        <v>684</v>
       </c>
       <c r="J39" s="3"/>
       <c r="K39" s="10"/>
@@ -8079,32 +8079,32 @@
         <v>37</v>
       </c>
       <c r="B40" s="6" t="s">
+        <v>684</v>
+      </c>
+      <c r="C40" s="37" t="s">
         <v>685</v>
       </c>
-      <c r="C40" s="37" t="s">
+      <c r="D40" s="36" t="s">
+        <v>701</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>722</v>
+      </c>
+      <c r="F40" s="6" t="s">
         <v>686</v>
-      </c>
-      <c r="D40" s="36" t="s">
-        <v>702</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>723</v>
-      </c>
-      <c r="F40" s="6" t="s">
-        <v>687</v>
       </c>
       <c r="G40" s="6"/>
       <c r="H40" s="34" t="s">
+        <v>687</v>
+      </c>
+      <c r="I40" s="7" t="s">
         <v>688</v>
-      </c>
-      <c r="I40" s="7" t="s">
-        <v>689</v>
       </c>
       <c r="J40" s="6">
         <v>60</v>
       </c>
       <c r="K40" s="50" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="L40" s="6">
         <v>60</v>
@@ -8117,26 +8117,26 @@
         <v>38</v>
       </c>
       <c r="B41" s="3" t="s">
+        <v>689</v>
+      </c>
+      <c r="C41" s="38" t="s">
+        <v>706</v>
+      </c>
+      <c r="D41" s="36" t="s">
+        <v>701</v>
+      </c>
+      <c r="E41" s="3" t="s">
         <v>690</v>
       </c>
-      <c r="C41" s="38" t="s">
-        <v>707</v>
-      </c>
-      <c r="D41" s="36" t="s">
-        <v>702</v>
-      </c>
-      <c r="E41" s="3" t="s">
+      <c r="F41" s="3" t="s">
         <v>691</v>
-      </c>
-      <c r="F41" s="3" t="s">
-        <v>692</v>
       </c>
       <c r="G41" s="3"/>
       <c r="H41" s="33" t="s">
+        <v>692</v>
+      </c>
+      <c r="I41" s="4" t="s">
         <v>693</v>
-      </c>
-      <c r="I41" s="4" t="s">
-        <v>694</v>
       </c>
       <c r="J41" s="3"/>
       <c r="K41" s="10"/>
@@ -8149,26 +8149,26 @@
         <v>39</v>
       </c>
       <c r="B42" s="6" t="s">
+        <v>694</v>
+      </c>
+      <c r="C42" s="6" t="s">
         <v>695</v>
       </c>
-      <c r="C42" s="6" t="s">
+      <c r="D42" s="36" t="s">
+        <v>707</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>725</v>
+      </c>
+      <c r="F42" s="6" t="s">
         <v>696</v>
-      </c>
-      <c r="D42" s="36" t="s">
-        <v>708</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>726</v>
-      </c>
-      <c r="F42" s="6" t="s">
-        <v>697</v>
       </c>
       <c r="G42" s="6"/>
       <c r="H42" s="34" t="s">
+        <v>697</v>
+      </c>
+      <c r="I42" s="7" t="s">
         <v>698</v>
-      </c>
-      <c r="I42" s="7" t="s">
-        <v>699</v>
       </c>
       <c r="J42" s="6">
         <v>16</v>
@@ -8193,7 +8193,7 @@
       </c>
       <c r="C43" s="3"/>
       <c r="D43" s="36" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="E43" s="3" t="s">
         <v>300</v>
@@ -8293,42 +8293,42 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="39" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="39" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="39" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
minor fix on taxonomy
</commit_message>
<xml_diff>
--- a/FoodBank Files/Food Bank recipients.xlsx
+++ b/FoodBank Files/Food Bank recipients.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\icarusjay\Downloads\xampp\htdocs\FoodBank Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{447360C0-3F7E-486B-B655-0983FA2E9E4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C20F9425-96FB-4211-8011-E4FA1899A20A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13740" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="728">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="730">
   <si>
     <t>PHASE 4 - B UNIT 1 HVG ARCADE, SUBANGDAKO, MANDAUE CITY</t>
   </si>
@@ -1619,9 +1619,6 @@
     <t>marivic@everlastinghope.org</t>
   </si>
   <si>
-    <t>Father's House Inc</t>
-  </si>
-  <si>
     <t>Talisay City, Cebu</t>
   </si>
   <si>
@@ -1965,9 +1962,6 @@
   </si>
   <si>
     <t>Residential Facility for children who have suffered from abuse, neglect and exploitation.</t>
-  </si>
-  <si>
-    <t>Ilihan, Toledo City Cebu (29 boys 45 girls)</t>
   </si>
   <si>
     <t>Jojin J. Ladroma</t>
@@ -2243,6 +2237,18 @@
   </si>
   <si>
     <t>Health/Medical</t>
+  </si>
+  <si>
+    <t>Lawaan, Cebu</t>
+  </si>
+  <si>
+    <t>Father's House Inc - Talisay</t>
+  </si>
+  <si>
+    <t>Father's House Inc - Lawaan</t>
+  </si>
+  <si>
+    <t>Ilihan, Toledo City Cebu</t>
   </si>
 </sst>
 </file>
@@ -2620,7 +2626,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2768,117 +2774,117 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2890,6 +2896,15 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3508,7 +3523,7 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" s="32"/>
-      <c r="B9" s="86" t="s">
+      <c r="B9" s="51" t="s">
         <v>0</v>
       </c>
       <c r="C9" s="50"/>
@@ -3524,88 +3539,88 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" s="32"/>
-      <c r="B10" s="51" t="s">
+      <c r="B10" s="85" t="s">
         <v>1</v>
       </c>
-      <c r="C10" s="51"/>
-      <c r="D10" s="51"/>
-      <c r="E10" s="51"/>
-      <c r="F10" s="51"/>
-      <c r="G10" s="51"/>
-      <c r="H10" s="51"/>
-      <c r="I10" s="51"/>
-      <c r="J10" s="51"/>
-      <c r="K10" s="51"/>
+      <c r="C10" s="85"/>
+      <c r="D10" s="85"/>
+      <c r="E10" s="85"/>
+      <c r="F10" s="85"/>
+      <c r="G10" s="85"/>
+      <c r="H10" s="85"/>
+      <c r="I10" s="85"/>
+      <c r="J10" s="85"/>
+      <c r="K10" s="85"/>
       <c r="L10" s="32"/>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" s="32"/>
-      <c r="B11" s="51"/>
-      <c r="C11" s="51"/>
-      <c r="D11" s="51"/>
-      <c r="E11" s="51"/>
-      <c r="F11" s="51"/>
-      <c r="G11" s="51"/>
-      <c r="H11" s="51"/>
-      <c r="I11" s="51"/>
-      <c r="J11" s="51"/>
-      <c r="K11" s="51"/>
+      <c r="B11" s="85"/>
+      <c r="C11" s="85"/>
+      <c r="D11" s="85"/>
+      <c r="E11" s="85"/>
+      <c r="F11" s="85"/>
+      <c r="G11" s="85"/>
+      <c r="H11" s="85"/>
+      <c r="I11" s="85"/>
+      <c r="J11" s="85"/>
+      <c r="K11" s="85"/>
       <c r="L11" s="32"/>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" s="32"/>
-      <c r="B12" s="87" t="s">
+      <c r="B12" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="C12" s="87"/>
-      <c r="D12" s="87"/>
-      <c r="E12" s="87"/>
-      <c r="F12" s="87"/>
-      <c r="G12" s="87"/>
-      <c r="H12" s="87"/>
-      <c r="I12" s="87"/>
-      <c r="J12" s="87"/>
-      <c r="K12" s="87"/>
+      <c r="C12" s="52"/>
+      <c r="D12" s="52"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="52"/>
+      <c r="G12" s="52"/>
+      <c r="H12" s="52"/>
+      <c r="I12" s="52"/>
+      <c r="J12" s="52"/>
+      <c r="K12" s="52"/>
       <c r="L12" s="32"/>
     </row>
     <row r="13" spans="1:12">
       <c r="A13" s="32"/>
-      <c r="B13" s="81" t="s">
+      <c r="B13" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="C13" s="82"/>
-      <c r="D13" s="83"/>
-      <c r="E13" s="81" t="s">
+      <c r="C13" s="54"/>
+      <c r="D13" s="55"/>
+      <c r="E13" s="53" t="s">
         <v>4</v>
       </c>
-      <c r="F13" s="82"/>
-      <c r="G13" s="83"/>
-      <c r="H13" s="81" t="s">
+      <c r="F13" s="54"/>
+      <c r="G13" s="55"/>
+      <c r="H13" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="I13" s="82"/>
-      <c r="J13" s="82"/>
-      <c r="K13" s="83"/>
+      <c r="I13" s="54"/>
+      <c r="J13" s="54"/>
+      <c r="K13" s="55"/>
       <c r="L13" s="32"/>
     </row>
     <row r="14" spans="1:12">
       <c r="A14" s="32"/>
-      <c r="B14" s="65" t="s">
+      <c r="B14" s="56" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="66"/>
-      <c r="D14" s="67"/>
-      <c r="E14" s="65" t="s">
+      <c r="C14" s="57"/>
+      <c r="D14" s="58"/>
+      <c r="E14" s="56" t="s">
         <v>7</v>
       </c>
-      <c r="F14" s="66"/>
-      <c r="G14" s="67"/>
-      <c r="H14" s="68" t="s">
+      <c r="F14" s="57"/>
+      <c r="G14" s="58"/>
+      <c r="H14" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="I14" s="69"/>
-      <c r="J14" s="69"/>
-      <c r="K14" s="70"/>
+      <c r="I14" s="60"/>
+      <c r="J14" s="60"/>
+      <c r="K14" s="61"/>
       <c r="L14" s="32"/>
     </row>
     <row r="15" spans="1:12">
@@ -3613,39 +3628,39 @@
       <c r="B15" s="62" t="s">
         <v>9</v>
       </c>
-      <c r="C15" s="80"/>
-      <c r="D15" s="63"/>
+      <c r="C15" s="63"/>
+      <c r="D15" s="64"/>
       <c r="E15" s="62" t="s">
         <v>10</v>
       </c>
-      <c r="F15" s="80"/>
-      <c r="G15" s="63"/>
-      <c r="H15" s="77" t="s">
+      <c r="F15" s="63"/>
+      <c r="G15" s="64"/>
+      <c r="H15" s="65" t="s">
         <v>11</v>
       </c>
-      <c r="I15" s="78"/>
-      <c r="J15" s="78"/>
-      <c r="K15" s="79"/>
+      <c r="I15" s="66"/>
+      <c r="J15" s="66"/>
+      <c r="K15" s="67"/>
       <c r="L15" s="32"/>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" s="32"/>
-      <c r="B16" s="65" t="s">
+      <c r="B16" s="56" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="66"/>
-      <c r="D16" s="67"/>
-      <c r="E16" s="65" t="s">
+      <c r="C16" s="57"/>
+      <c r="D16" s="58"/>
+      <c r="E16" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="F16" s="66"/>
-      <c r="G16" s="67"/>
-      <c r="H16" s="68" t="s">
+      <c r="F16" s="57"/>
+      <c r="G16" s="58"/>
+      <c r="H16" s="59" t="s">
         <v>14</v>
       </c>
-      <c r="I16" s="69"/>
-      <c r="J16" s="69"/>
-      <c r="K16" s="70"/>
+      <c r="I16" s="60"/>
+      <c r="J16" s="60"/>
+      <c r="K16" s="61"/>
       <c r="L16" s="32"/>
     </row>
     <row r="17" spans="1:16">
@@ -3653,39 +3668,39 @@
       <c r="B17" s="62" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="80"/>
-      <c r="D17" s="63"/>
+      <c r="C17" s="63"/>
+      <c r="D17" s="64"/>
       <c r="E17" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="F17" s="80"/>
-      <c r="G17" s="63"/>
-      <c r="H17" s="77" t="s">
+      <c r="F17" s="63"/>
+      <c r="G17" s="64"/>
+      <c r="H17" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="I17" s="78"/>
-      <c r="J17" s="78"/>
-      <c r="K17" s="79"/>
+      <c r="I17" s="66"/>
+      <c r="J17" s="66"/>
+      <c r="K17" s="67"/>
       <c r="L17" s="32"/>
     </row>
     <row r="18" spans="1:16">
       <c r="A18" s="32"/>
-      <c r="B18" s="65" t="s">
+      <c r="B18" s="56" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="66"/>
-      <c r="D18" s="67"/>
-      <c r="E18" s="65" t="s">
+      <c r="C18" s="57"/>
+      <c r="D18" s="58"/>
+      <c r="E18" s="56" t="s">
         <v>19</v>
       </c>
-      <c r="F18" s="66"/>
-      <c r="G18" s="67"/>
-      <c r="H18" s="68" t="s">
+      <c r="F18" s="57"/>
+      <c r="G18" s="58"/>
+      <c r="H18" s="59" t="s">
         <v>20</v>
       </c>
-      <c r="I18" s="69"/>
-      <c r="J18" s="69"/>
-      <c r="K18" s="70"/>
+      <c r="I18" s="60"/>
+      <c r="J18" s="60"/>
+      <c r="K18" s="61"/>
       <c r="L18" s="32"/>
     </row>
     <row r="19" spans="1:16">
@@ -3693,39 +3708,39 @@
       <c r="B19" s="62" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="80"/>
-      <c r="D19" s="63"/>
+      <c r="C19" s="63"/>
+      <c r="D19" s="64"/>
       <c r="E19" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="F19" s="80"/>
-      <c r="G19" s="63"/>
-      <c r="H19" s="77" t="s">
+      <c r="F19" s="63"/>
+      <c r="G19" s="64"/>
+      <c r="H19" s="65" t="s">
         <v>23</v>
       </c>
-      <c r="I19" s="78"/>
-      <c r="J19" s="78"/>
-      <c r="K19" s="79"/>
+      <c r="I19" s="66"/>
+      <c r="J19" s="66"/>
+      <c r="K19" s="67"/>
       <c r="L19" s="32"/>
     </row>
     <row r="20" spans="1:16">
       <c r="A20" s="32"/>
-      <c r="B20" s="65" t="s">
+      <c r="B20" s="56" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="66"/>
-      <c r="D20" s="67"/>
-      <c r="E20" s="65" t="s">
+      <c r="C20" s="57"/>
+      <c r="D20" s="58"/>
+      <c r="E20" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="F20" s="66"/>
-      <c r="G20" s="67"/>
-      <c r="H20" s="68" t="s">
+      <c r="F20" s="57"/>
+      <c r="G20" s="58"/>
+      <c r="H20" s="59" t="s">
         <v>26</v>
       </c>
-      <c r="I20" s="69"/>
-      <c r="J20" s="69"/>
-      <c r="K20" s="70"/>
+      <c r="I20" s="60"/>
+      <c r="J20" s="60"/>
+      <c r="K20" s="61"/>
       <c r="L20" s="32"/>
     </row>
     <row r="21" spans="1:16">
@@ -3733,39 +3748,39 @@
       <c r="B21" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="C21" s="80"/>
-      <c r="D21" s="63"/>
+      <c r="C21" s="63"/>
+      <c r="D21" s="64"/>
       <c r="E21" s="62" t="s">
         <v>28</v>
       </c>
-      <c r="F21" s="80"/>
-      <c r="G21" s="63"/>
-      <c r="H21" s="77" t="s">
+      <c r="F21" s="63"/>
+      <c r="G21" s="64"/>
+      <c r="H21" s="65" t="s">
         <v>29</v>
       </c>
-      <c r="I21" s="78"/>
-      <c r="J21" s="78"/>
-      <c r="K21" s="79"/>
+      <c r="I21" s="66"/>
+      <c r="J21" s="66"/>
+      <c r="K21" s="67"/>
       <c r="L21" s="32"/>
     </row>
     <row r="22" spans="1:16">
       <c r="A22" s="32"/>
-      <c r="B22" s="65" t="s">
+      <c r="B22" s="56" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="66"/>
-      <c r="D22" s="67"/>
-      <c r="E22" s="65" t="s">
+      <c r="C22" s="57"/>
+      <c r="D22" s="58"/>
+      <c r="E22" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="F22" s="66"/>
-      <c r="G22" s="67"/>
-      <c r="H22" s="68" t="s">
+      <c r="F22" s="57"/>
+      <c r="G22" s="58"/>
+      <c r="H22" s="59" t="s">
         <v>32</v>
       </c>
-      <c r="I22" s="69"/>
-      <c r="J22" s="69"/>
-      <c r="K22" s="70"/>
+      <c r="I22" s="60"/>
+      <c r="J22" s="60"/>
+      <c r="K22" s="61"/>
       <c r="L22" s="32"/>
     </row>
     <row r="23" spans="1:16">
@@ -3788,18 +3803,18 @@
     </row>
     <row r="24" spans="1:16">
       <c r="A24" s="32"/>
-      <c r="B24" s="64" t="s">
+      <c r="B24" s="68" t="s">
         <v>33</v>
       </c>
-      <c r="C24" s="64"/>
-      <c r="D24" s="64"/>
-      <c r="E24" s="64"/>
-      <c r="F24" s="64"/>
-      <c r="G24" s="64"/>
-      <c r="H24" s="64"/>
-      <c r="I24" s="64"/>
-      <c r="J24" s="64"/>
-      <c r="K24" s="64"/>
+      <c r="C24" s="68"/>
+      <c r="D24" s="68"/>
+      <c r="E24" s="68"/>
+      <c r="F24" s="68"/>
+      <c r="G24" s="68"/>
+      <c r="H24" s="68"/>
+      <c r="I24" s="68"/>
+      <c r="J24" s="68"/>
+      <c r="K24" s="68"/>
       <c r="L24" s="32"/>
       <c r="M24" s="32"/>
       <c r="N24" s="32"/>
@@ -3808,64 +3823,64 @@
     </row>
     <row r="25" spans="1:16">
       <c r="A25" s="32"/>
-      <c r="B25" s="81" t="s">
+      <c r="B25" s="53" t="s">
         <v>34</v>
       </c>
-      <c r="C25" s="82"/>
-      <c r="D25" s="82"/>
-      <c r="E25" s="82"/>
-      <c r="F25" s="83"/>
-      <c r="G25" s="81" t="s">
+      <c r="C25" s="54"/>
+      <c r="D25" s="54"/>
+      <c r="E25" s="54"/>
+      <c r="F25" s="55"/>
+      <c r="G25" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="H25" s="84"/>
-      <c r="I25" s="84"/>
-      <c r="J25" s="84"/>
-      <c r="K25" s="85"/>
+      <c r="H25" s="69"/>
+      <c r="I25" s="69"/>
+      <c r="J25" s="69"/>
+      <c r="K25" s="70"/>
       <c r="L25" s="62"/>
-      <c r="M25" s="63"/>
+      <c r="M25" s="64"/>
       <c r="N25" s="32"/>
       <c r="O25"/>
       <c r="P25"/>
     </row>
     <row r="26" spans="1:16">
       <c r="A26" s="32"/>
-      <c r="B26" s="54" t="s">
+      <c r="B26" s="71" t="s">
         <v>35</v>
       </c>
-      <c r="C26" s="54"/>
-      <c r="D26" s="54"/>
-      <c r="E26" s="54"/>
-      <c r="F26" s="54"/>
-      <c r="G26" s="55" t="s">
+      <c r="C26" s="71"/>
+      <c r="D26" s="71"/>
+      <c r="E26" s="71"/>
+      <c r="F26" s="71"/>
+      <c r="G26" s="72" t="s">
         <v>36</v>
       </c>
-      <c r="H26" s="55"/>
-      <c r="I26" s="55"/>
-      <c r="J26" s="55"/>
-      <c r="K26" s="55"/>
+      <c r="H26" s="72"/>
+      <c r="I26" s="72"/>
+      <c r="J26" s="72"/>
+      <c r="K26" s="72"/>
       <c r="L26" s="62"/>
-      <c r="M26" s="63"/>
+      <c r="M26" s="64"/>
       <c r="N26" s="32"/>
       <c r="O26"/>
       <c r="P26"/>
     </row>
     <row r="27" spans="1:16">
       <c r="A27" s="32"/>
-      <c r="B27" s="52" t="s">
+      <c r="B27" s="73" t="s">
         <v>37</v>
       </c>
-      <c r="C27" s="52"/>
-      <c r="D27" s="52"/>
-      <c r="E27" s="52"/>
-      <c r="F27" s="52"/>
-      <c r="G27" s="53" t="s">
+      <c r="C27" s="73"/>
+      <c r="D27" s="73"/>
+      <c r="E27" s="73"/>
+      <c r="F27" s="73"/>
+      <c r="G27" s="74" t="s">
         <v>38</v>
       </c>
-      <c r="H27" s="53"/>
-      <c r="I27" s="53"/>
-      <c r="J27" s="53"/>
-      <c r="K27" s="53"/>
+      <c r="H27" s="74"/>
+      <c r="I27" s="74"/>
+      <c r="J27" s="74"/>
+      <c r="K27" s="74"/>
       <c r="L27" s="75" t="s">
         <v>39</v>
       </c>
@@ -3876,64 +3891,64 @@
     </row>
     <row r="28" spans="1:16">
       <c r="A28" s="32"/>
-      <c r="B28" s="54" t="s">
+      <c r="B28" s="71" t="s">
         <v>40</v>
       </c>
-      <c r="C28" s="54"/>
-      <c r="D28" s="54"/>
-      <c r="E28" s="54"/>
-      <c r="F28" s="54"/>
-      <c r="G28" s="55" t="s">
+      <c r="C28" s="71"/>
+      <c r="D28" s="71"/>
+      <c r="E28" s="71"/>
+      <c r="F28" s="71"/>
+      <c r="G28" s="72" t="s">
         <v>41</v>
       </c>
-      <c r="H28" s="55"/>
-      <c r="I28" s="55"/>
-      <c r="J28" s="55"/>
-      <c r="K28" s="55"/>
+      <c r="H28" s="72"/>
+      <c r="I28" s="72"/>
+      <c r="J28" s="72"/>
+      <c r="K28" s="72"/>
       <c r="L28" s="62"/>
-      <c r="M28" s="63"/>
+      <c r="M28" s="64"/>
       <c r="N28" s="32"/>
       <c r="O28"/>
       <c r="P28"/>
     </row>
     <row r="29" spans="1:16">
       <c r="A29" s="32"/>
-      <c r="B29" s="52" t="s">
+      <c r="B29" s="73" t="s">
         <v>42</v>
       </c>
-      <c r="C29" s="52"/>
-      <c r="D29" s="52"/>
-      <c r="E29" s="52"/>
-      <c r="F29" s="52"/>
-      <c r="G29" s="53" t="s">
+      <c r="C29" s="73"/>
+      <c r="D29" s="73"/>
+      <c r="E29" s="73"/>
+      <c r="F29" s="73"/>
+      <c r="G29" s="74" t="s">
         <v>43</v>
       </c>
-      <c r="H29" s="53"/>
-      <c r="I29" s="53"/>
-      <c r="J29" s="53"/>
-      <c r="K29" s="53"/>
+      <c r="H29" s="74"/>
+      <c r="I29" s="74"/>
+      <c r="J29" s="74"/>
+      <c r="K29" s="74"/>
       <c r="L29" s="62"/>
-      <c r="M29" s="63"/>
+      <c r="M29" s="64"/>
       <c r="N29" s="32"/>
       <c r="O29"/>
       <c r="P29"/>
     </row>
     <row r="30" spans="1:16">
       <c r="A30" s="32"/>
-      <c r="B30" s="54" t="s">
+      <c r="B30" s="71" t="s">
         <v>44</v>
       </c>
-      <c r="C30" s="54"/>
-      <c r="D30" s="54"/>
-      <c r="E30" s="54"/>
-      <c r="F30" s="54"/>
-      <c r="G30" s="55" t="s">
+      <c r="C30" s="71"/>
+      <c r="D30" s="71"/>
+      <c r="E30" s="71"/>
+      <c r="F30" s="71"/>
+      <c r="G30" s="72" t="s">
         <v>45</v>
       </c>
-      <c r="H30" s="55"/>
-      <c r="I30" s="55"/>
-      <c r="J30" s="55"/>
-      <c r="K30" s="55"/>
+      <c r="H30" s="72"/>
+      <c r="I30" s="72"/>
+      <c r="J30" s="72"/>
+      <c r="K30" s="72"/>
       <c r="L30" s="75" t="s">
         <v>46</v>
       </c>
@@ -3944,42 +3959,42 @@
     </row>
     <row r="31" spans="1:16">
       <c r="A31" s="32"/>
-      <c r="B31" s="52" t="s">
+      <c r="B31" s="73" t="s">
         <v>47</v>
       </c>
-      <c r="C31" s="52"/>
-      <c r="D31" s="52"/>
-      <c r="E31" s="52"/>
-      <c r="F31" s="52"/>
-      <c r="G31" s="77" t="s">
+      <c r="C31" s="73"/>
+      <c r="D31" s="73"/>
+      <c r="E31" s="73"/>
+      <c r="F31" s="73"/>
+      <c r="G31" s="65" t="s">
         <v>48</v>
       </c>
-      <c r="H31" s="78"/>
-      <c r="I31" s="78"/>
-      <c r="J31" s="78"/>
-      <c r="K31" s="79"/>
+      <c r="H31" s="66"/>
+      <c r="I31" s="66"/>
+      <c r="J31" s="66"/>
+      <c r="K31" s="67"/>
       <c r="L31" s="62"/>
-      <c r="M31" s="63"/>
+      <c r="M31" s="64"/>
       <c r="N31" s="32"/>
       <c r="O31"/>
       <c r="P31"/>
     </row>
     <row r="32" spans="1:16">
       <c r="A32" s="32"/>
-      <c r="B32" s="54" t="s">
+      <c r="B32" s="71" t="s">
         <v>49</v>
       </c>
-      <c r="C32" s="54"/>
-      <c r="D32" s="54"/>
-      <c r="E32" s="54"/>
-      <c r="F32" s="54"/>
-      <c r="G32" s="55" t="s">
+      <c r="C32" s="71"/>
+      <c r="D32" s="71"/>
+      <c r="E32" s="71"/>
+      <c r="F32" s="71"/>
+      <c r="G32" s="72" t="s">
         <v>50</v>
       </c>
-      <c r="H32" s="55"/>
-      <c r="I32" s="55"/>
-      <c r="J32" s="55"/>
-      <c r="K32" s="55"/>
+      <c r="H32" s="72"/>
+      <c r="I32" s="72"/>
+      <c r="J32" s="72"/>
+      <c r="K32" s="72"/>
       <c r="L32" s="75" t="s">
         <v>51</v>
       </c>
@@ -3990,42 +4005,42 @@
     </row>
     <row r="33" spans="1:16">
       <c r="A33" s="32"/>
-      <c r="B33" s="52" t="s">
+      <c r="B33" s="73" t="s">
         <v>52</v>
       </c>
-      <c r="C33" s="52"/>
-      <c r="D33" s="52"/>
-      <c r="E33" s="52"/>
-      <c r="F33" s="52"/>
-      <c r="G33" s="77" t="s">
+      <c r="C33" s="73"/>
+      <c r="D33" s="73"/>
+      <c r="E33" s="73"/>
+      <c r="F33" s="73"/>
+      <c r="G33" s="65" t="s">
         <v>48</v>
       </c>
-      <c r="H33" s="78"/>
-      <c r="I33" s="78"/>
-      <c r="J33" s="78"/>
-      <c r="K33" s="79"/>
+      <c r="H33" s="66"/>
+      <c r="I33" s="66"/>
+      <c r="J33" s="66"/>
+      <c r="K33" s="67"/>
       <c r="L33" s="62"/>
-      <c r="M33" s="63"/>
+      <c r="M33" s="64"/>
       <c r="N33" s="32"/>
       <c r="O33"/>
       <c r="P33"/>
     </row>
     <row r="34" spans="1:16">
       <c r="A34" s="32"/>
-      <c r="B34" s="54" t="s">
+      <c r="B34" s="71" t="s">
         <v>53</v>
       </c>
-      <c r="C34" s="54"/>
-      <c r="D34" s="54"/>
-      <c r="E34" s="54"/>
-      <c r="F34" s="54"/>
-      <c r="G34" s="55" t="s">
+      <c r="C34" s="71"/>
+      <c r="D34" s="71"/>
+      <c r="E34" s="71"/>
+      <c r="F34" s="71"/>
+      <c r="G34" s="72" t="s">
         <v>54</v>
       </c>
-      <c r="H34" s="55"/>
-      <c r="I34" s="55"/>
-      <c r="J34" s="55"/>
-      <c r="K34" s="55"/>
+      <c r="H34" s="72"/>
+      <c r="I34" s="72"/>
+      <c r="J34" s="72"/>
+      <c r="K34" s="72"/>
       <c r="L34" s="75" t="s">
         <v>55</v>
       </c>
@@ -4036,350 +4051,350 @@
     </row>
     <row r="35" spans="1:16">
       <c r="A35" s="32"/>
-      <c r="B35" s="52" t="s">
+      <c r="B35" s="73" t="s">
         <v>56</v>
       </c>
-      <c r="C35" s="52"/>
-      <c r="D35" s="52"/>
-      <c r="E35" s="52"/>
-      <c r="F35" s="52"/>
-      <c r="G35" s="53" t="s">
+      <c r="C35" s="73"/>
+      <c r="D35" s="73"/>
+      <c r="E35" s="73"/>
+      <c r="F35" s="73"/>
+      <c r="G35" s="74" t="s">
         <v>57</v>
       </c>
-      <c r="H35" s="53"/>
-      <c r="I35" s="53"/>
-      <c r="J35" s="53"/>
-      <c r="K35" s="53"/>
+      <c r="H35" s="74"/>
+      <c r="I35" s="74"/>
+      <c r="J35" s="74"/>
+      <c r="K35" s="74"/>
       <c r="L35" s="62"/>
-      <c r="M35" s="63"/>
+      <c r="M35" s="64"/>
       <c r="N35" s="32"/>
       <c r="O35"/>
       <c r="P35"/>
     </row>
     <row r="36" spans="1:16">
       <c r="A36" s="32"/>
-      <c r="B36" s="54" t="s">
+      <c r="B36" s="71" t="s">
         <v>58</v>
       </c>
-      <c r="C36" s="54"/>
-      <c r="D36" s="54"/>
-      <c r="E36" s="54"/>
-      <c r="F36" s="54"/>
-      <c r="G36" s="55" t="s">
+      <c r="C36" s="71"/>
+      <c r="D36" s="71"/>
+      <c r="E36" s="71"/>
+      <c r="F36" s="71"/>
+      <c r="G36" s="72" t="s">
         <v>59</v>
       </c>
-      <c r="H36" s="55"/>
-      <c r="I36" s="55"/>
-      <c r="J36" s="55"/>
-      <c r="K36" s="55"/>
-      <c r="L36" s="73"/>
-      <c r="M36" s="74"/>
+      <c r="H36" s="72"/>
+      <c r="I36" s="72"/>
+      <c r="J36" s="72"/>
+      <c r="K36" s="72"/>
+      <c r="L36" s="77"/>
+      <c r="M36" s="78"/>
       <c r="N36" s="32"/>
       <c r="O36"/>
       <c r="P36"/>
     </row>
     <row r="37" spans="1:16">
       <c r="A37" s="32"/>
-      <c r="B37" s="52" t="s">
+      <c r="B37" s="73" t="s">
         <v>60</v>
       </c>
-      <c r="C37" s="52"/>
-      <c r="D37" s="52"/>
-      <c r="E37" s="52"/>
-      <c r="F37" s="52"/>
-      <c r="G37" s="53" t="s">
+      <c r="C37" s="73"/>
+      <c r="D37" s="73"/>
+      <c r="E37" s="73"/>
+      <c r="F37" s="73"/>
+      <c r="G37" s="74" t="s">
         <v>61</v>
       </c>
-      <c r="H37" s="53"/>
-      <c r="I37" s="53"/>
-      <c r="J37" s="53"/>
-      <c r="K37" s="53"/>
-      <c r="L37" s="73"/>
-      <c r="M37" s="74"/>
+      <c r="H37" s="74"/>
+      <c r="I37" s="74"/>
+      <c r="J37" s="74"/>
+      <c r="K37" s="74"/>
+      <c r="L37" s="77"/>
+      <c r="M37" s="78"/>
       <c r="N37" s="32"/>
       <c r="O37"/>
       <c r="P37"/>
     </row>
     <row r="38" spans="1:16">
       <c r="A38" s="32"/>
-      <c r="B38" s="54" t="s">
+      <c r="B38" s="71" t="s">
         <v>62</v>
       </c>
-      <c r="C38" s="54"/>
-      <c r="D38" s="54"/>
-      <c r="E38" s="54"/>
-      <c r="F38" s="54"/>
-      <c r="G38" s="55" t="s">
+      <c r="C38" s="71"/>
+      <c r="D38" s="71"/>
+      <c r="E38" s="71"/>
+      <c r="F38" s="71"/>
+      <c r="G38" s="72" t="s">
         <v>63</v>
       </c>
-      <c r="H38" s="55"/>
-      <c r="I38" s="55"/>
-      <c r="J38" s="55"/>
-      <c r="K38" s="55"/>
+      <c r="H38" s="72"/>
+      <c r="I38" s="72"/>
+      <c r="J38" s="72"/>
+      <c r="K38" s="72"/>
       <c r="L38" s="62"/>
-      <c r="M38" s="63"/>
+      <c r="M38" s="64"/>
       <c r="N38" s="32"/>
       <c r="O38"/>
       <c r="P38"/>
     </row>
     <row r="39" spans="1:16">
       <c r="A39" s="32"/>
-      <c r="B39" s="52" t="s">
+      <c r="B39" s="73" t="s">
         <v>64</v>
       </c>
-      <c r="C39" s="52"/>
-      <c r="D39" s="52"/>
-      <c r="E39" s="52"/>
-      <c r="F39" s="52"/>
-      <c r="G39" s="53" t="s">
+      <c r="C39" s="73"/>
+      <c r="D39" s="73"/>
+      <c r="E39" s="73"/>
+      <c r="F39" s="73"/>
+      <c r="G39" s="74" t="s">
         <v>65</v>
       </c>
-      <c r="H39" s="53"/>
-      <c r="I39" s="53"/>
-      <c r="J39" s="53"/>
-      <c r="K39" s="53"/>
+      <c r="H39" s="74"/>
+      <c r="I39" s="74"/>
+      <c r="J39" s="74"/>
+      <c r="K39" s="74"/>
       <c r="L39" s="62"/>
-      <c r="M39" s="63"/>
+      <c r="M39" s="64"/>
       <c r="N39" s="32"/>
       <c r="O39"/>
       <c r="P39"/>
     </row>
     <row r="40" spans="1:16">
       <c r="A40" s="32"/>
-      <c r="B40" s="54" t="s">
+      <c r="B40" s="71" t="s">
         <v>66</v>
       </c>
-      <c r="C40" s="54"/>
-      <c r="D40" s="54"/>
-      <c r="E40" s="54"/>
-      <c r="F40" s="54"/>
-      <c r="G40" s="55" t="s">
+      <c r="C40" s="71"/>
+      <c r="D40" s="71"/>
+      <c r="E40" s="71"/>
+      <c r="F40" s="71"/>
+      <c r="G40" s="72" t="s">
         <v>67</v>
       </c>
-      <c r="H40" s="55"/>
-      <c r="I40" s="55"/>
-      <c r="J40" s="55"/>
-      <c r="K40" s="55"/>
-      <c r="L40" s="73"/>
-      <c r="M40" s="74"/>
+      <c r="H40" s="72"/>
+      <c r="I40" s="72"/>
+      <c r="J40" s="72"/>
+      <c r="K40" s="72"/>
+      <c r="L40" s="77"/>
+      <c r="M40" s="78"/>
       <c r="N40" s="32"/>
       <c r="O40"/>
       <c r="P40"/>
     </row>
     <row r="41" spans="1:16">
       <c r="A41" s="32"/>
-      <c r="B41" s="52" t="s">
+      <c r="B41" s="73" t="s">
         <v>68</v>
       </c>
-      <c r="C41" s="52"/>
-      <c r="D41" s="52"/>
-      <c r="E41" s="52"/>
-      <c r="F41" s="52"/>
-      <c r="G41" s="53" t="s">
+      <c r="C41" s="73"/>
+      <c r="D41" s="73"/>
+      <c r="E41" s="73"/>
+      <c r="F41" s="73"/>
+      <c r="G41" s="74" t="s">
         <v>69</v>
       </c>
-      <c r="H41" s="53"/>
-      <c r="I41" s="53"/>
-      <c r="J41" s="53"/>
-      <c r="K41" s="53"/>
-      <c r="L41" s="73"/>
-      <c r="M41" s="74"/>
+      <c r="H41" s="74"/>
+      <c r="I41" s="74"/>
+      <c r="J41" s="74"/>
+      <c r="K41" s="74"/>
+      <c r="L41" s="77"/>
+      <c r="M41" s="78"/>
       <c r="N41" s="32"/>
       <c r="O41"/>
       <c r="P41"/>
     </row>
     <row r="42" spans="1:16">
       <c r="A42" s="32"/>
-      <c r="B42" s="54" t="s">
+      <c r="B42" s="71" t="s">
         <v>70</v>
       </c>
-      <c r="C42" s="54"/>
-      <c r="D42" s="54"/>
-      <c r="E42" s="54"/>
-      <c r="F42" s="54"/>
-      <c r="G42" s="55" t="s">
+      <c r="C42" s="71"/>
+      <c r="D42" s="71"/>
+      <c r="E42" s="71"/>
+      <c r="F42" s="71"/>
+      <c r="G42" s="72" t="s">
         <v>71</v>
       </c>
-      <c r="H42" s="55"/>
-      <c r="I42" s="55"/>
-      <c r="J42" s="55"/>
-      <c r="K42" s="55"/>
+      <c r="H42" s="72"/>
+      <c r="I42" s="72"/>
+      <c r="J42" s="72"/>
+      <c r="K42" s="72"/>
       <c r="L42" s="62"/>
-      <c r="M42" s="63"/>
+      <c r="M42" s="64"/>
       <c r="N42" s="32"/>
       <c r="O42"/>
       <c r="P42"/>
     </row>
     <row r="43" spans="1:16">
       <c r="A43" s="32"/>
-      <c r="B43" s="52" t="s">
+      <c r="B43" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="C43" s="52"/>
-      <c r="D43" s="52"/>
-      <c r="E43" s="52"/>
-      <c r="F43" s="52"/>
-      <c r="G43" s="53" t="s">
+      <c r="C43" s="73"/>
+      <c r="D43" s="73"/>
+      <c r="E43" s="73"/>
+      <c r="F43" s="73"/>
+      <c r="G43" s="74" t="s">
         <v>73</v>
       </c>
-      <c r="H43" s="53"/>
-      <c r="I43" s="53"/>
-      <c r="J43" s="53"/>
-      <c r="K43" s="53"/>
+      <c r="H43" s="74"/>
+      <c r="I43" s="74"/>
+      <c r="J43" s="74"/>
+      <c r="K43" s="74"/>
       <c r="L43" s="62"/>
-      <c r="M43" s="63"/>
+      <c r="M43" s="64"/>
       <c r="N43" s="32"/>
       <c r="O43"/>
       <c r="P43"/>
     </row>
     <row r="44" spans="1:16">
       <c r="A44" s="32"/>
-      <c r="B44" s="54" t="s">
+      <c r="B44" s="71" t="s">
         <v>74</v>
       </c>
-      <c r="C44" s="54"/>
-      <c r="D44" s="54"/>
-      <c r="E44" s="54"/>
-      <c r="F44" s="54"/>
-      <c r="G44" s="55" t="s">
+      <c r="C44" s="71"/>
+      <c r="D44" s="71"/>
+      <c r="E44" s="71"/>
+      <c r="F44" s="71"/>
+      <c r="G44" s="72" t="s">
         <v>75</v>
       </c>
-      <c r="H44" s="55"/>
-      <c r="I44" s="55"/>
-      <c r="J44" s="55"/>
-      <c r="K44" s="55"/>
+      <c r="H44" s="72"/>
+      <c r="I44" s="72"/>
+      <c r="J44" s="72"/>
+      <c r="K44" s="72"/>
       <c r="L44" s="62"/>
-      <c r="M44" s="63"/>
+      <c r="M44" s="64"/>
       <c r="N44" s="32"/>
       <c r="O44"/>
       <c r="P44"/>
     </row>
     <row r="45" spans="1:16">
       <c r="A45" s="32"/>
-      <c r="B45" s="52" t="s">
+      <c r="B45" s="73" t="s">
         <v>76</v>
       </c>
-      <c r="C45" s="52"/>
-      <c r="D45" s="52"/>
-      <c r="E45" s="52"/>
-      <c r="F45" s="52"/>
-      <c r="G45" s="53" t="s">
+      <c r="C45" s="73"/>
+      <c r="D45" s="73"/>
+      <c r="E45" s="73"/>
+      <c r="F45" s="73"/>
+      <c r="G45" s="74" t="s">
         <v>77</v>
       </c>
-      <c r="H45" s="53"/>
-      <c r="I45" s="53"/>
-      <c r="J45" s="53"/>
-      <c r="K45" s="53"/>
-      <c r="L45" s="73"/>
-      <c r="M45" s="74"/>
+      <c r="H45" s="74"/>
+      <c r="I45" s="74"/>
+      <c r="J45" s="74"/>
+      <c r="K45" s="74"/>
+      <c r="L45" s="77"/>
+      <c r="M45" s="78"/>
       <c r="N45" s="32"/>
       <c r="O45"/>
       <c r="P45"/>
     </row>
     <row r="46" spans="1:16">
       <c r="A46" s="32"/>
-      <c r="B46" s="54" t="s">
+      <c r="B46" s="71" t="s">
         <v>78</v>
       </c>
-      <c r="C46" s="54"/>
-      <c r="D46" s="54"/>
-      <c r="E46" s="54"/>
-      <c r="F46" s="54"/>
-      <c r="G46" s="55" t="s">
+      <c r="C46" s="71"/>
+      <c r="D46" s="71"/>
+      <c r="E46" s="71"/>
+      <c r="F46" s="71"/>
+      <c r="G46" s="72" t="s">
         <v>79</v>
       </c>
-      <c r="H46" s="55"/>
-      <c r="I46" s="55"/>
-      <c r="J46" s="55"/>
-      <c r="K46" s="55"/>
+      <c r="H46" s="72"/>
+      <c r="I46" s="72"/>
+      <c r="J46" s="72"/>
+      <c r="K46" s="72"/>
       <c r="L46" s="62"/>
-      <c r="M46" s="63"/>
+      <c r="M46" s="64"/>
       <c r="N46" s="32"/>
       <c r="O46"/>
       <c r="P46"/>
     </row>
     <row r="47" spans="1:16">
       <c r="A47" s="32"/>
-      <c r="B47" s="52" t="s">
+      <c r="B47" s="73" t="s">
         <v>80</v>
       </c>
-      <c r="C47" s="52"/>
-      <c r="D47" s="52"/>
-      <c r="E47" s="52"/>
-      <c r="F47" s="52"/>
-      <c r="G47" s="53" t="s">
+      <c r="C47" s="73"/>
+      <c r="D47" s="73"/>
+      <c r="E47" s="73"/>
+      <c r="F47" s="73"/>
+      <c r="G47" s="74" t="s">
         <v>81</v>
       </c>
-      <c r="H47" s="53"/>
-      <c r="I47" s="53"/>
-      <c r="J47" s="53"/>
-      <c r="K47" s="53"/>
+      <c r="H47" s="74"/>
+      <c r="I47" s="74"/>
+      <c r="J47" s="74"/>
+      <c r="K47" s="74"/>
       <c r="L47" s="62"/>
-      <c r="M47" s="63"/>
+      <c r="M47" s="64"/>
       <c r="N47" s="32"/>
       <c r="O47"/>
       <c r="P47"/>
     </row>
     <row r="48" spans="1:16">
       <c r="A48" s="32"/>
-      <c r="B48" s="65" t="s">
+      <c r="B48" s="56" t="s">
         <v>82</v>
       </c>
-      <c r="C48" s="66"/>
-      <c r="D48" s="66"/>
-      <c r="E48" s="66"/>
-      <c r="F48" s="67"/>
-      <c r="G48" s="68" t="s">
+      <c r="C48" s="57"/>
+      <c r="D48" s="57"/>
+      <c r="E48" s="57"/>
+      <c r="F48" s="58"/>
+      <c r="G48" s="59" t="s">
         <v>83</v>
       </c>
-      <c r="H48" s="69"/>
-      <c r="I48" s="69"/>
-      <c r="J48" s="69"/>
-      <c r="K48" s="70"/>
+      <c r="H48" s="60"/>
+      <c r="I48" s="60"/>
+      <c r="J48" s="60"/>
+      <c r="K48" s="61"/>
       <c r="L48" s="62"/>
-      <c r="M48" s="63"/>
+      <c r="M48" s="64"/>
       <c r="N48" s="32"/>
       <c r="O48"/>
       <c r="P48"/>
     </row>
     <row r="49" spans="1:16">
       <c r="A49" s="32"/>
-      <c r="B49" s="71" t="s">
+      <c r="B49" s="79" t="s">
         <v>84</v>
       </c>
-      <c r="C49" s="71"/>
-      <c r="D49" s="71"/>
-      <c r="E49" s="71"/>
-      <c r="F49" s="71"/>
-      <c r="G49" s="72" t="s">
+      <c r="C49" s="79"/>
+      <c r="D49" s="79"/>
+      <c r="E49" s="79"/>
+      <c r="F49" s="79"/>
+      <c r="G49" s="80" t="s">
         <v>85</v>
       </c>
-      <c r="H49" s="72"/>
-      <c r="I49" s="72"/>
-      <c r="J49" s="72"/>
-      <c r="K49" s="72"/>
+      <c r="H49" s="80"/>
+      <c r="I49" s="80"/>
+      <c r="J49" s="80"/>
+      <c r="K49" s="80"/>
       <c r="L49" s="62"/>
-      <c r="M49" s="63"/>
+      <c r="M49" s="64"/>
       <c r="N49" s="32"/>
       <c r="O49"/>
       <c r="P49"/>
     </row>
     <row r="50" spans="1:16">
       <c r="A50" s="32"/>
-      <c r="B50" s="58" t="s">
+      <c r="B50" s="81" t="s">
         <v>86</v>
       </c>
-      <c r="C50" s="59"/>
-      <c r="D50" s="59"/>
-      <c r="E50" s="59"/>
-      <c r="F50" s="60"/>
-      <c r="G50" s="61"/>
-      <c r="H50" s="59"/>
-      <c r="I50" s="59"/>
-      <c r="J50" s="59"/>
-      <c r="K50" s="60"/>
+      <c r="C50" s="82"/>
+      <c r="D50" s="82"/>
+      <c r="E50" s="82"/>
+      <c r="F50" s="83"/>
+      <c r="G50" s="84"/>
+      <c r="H50" s="82"/>
+      <c r="I50" s="82"/>
+      <c r="J50" s="82"/>
+      <c r="K50" s="83"/>
       <c r="L50" s="62"/>
-      <c r="M50" s="63"/>
+      <c r="M50" s="64"/>
       <c r="N50" s="32"/>
       <c r="O50"/>
       <c r="P50"/>
@@ -4404,18 +4419,18 @@
     </row>
     <row r="52" spans="1:16">
       <c r="A52" s="32"/>
-      <c r="B52" s="64" t="s">
+      <c r="B52" s="68" t="s">
         <v>87</v>
       </c>
-      <c r="C52" s="64"/>
-      <c r="D52" s="64"/>
-      <c r="E52" s="64"/>
-      <c r="F52" s="64"/>
-      <c r="G52" s="64"/>
-      <c r="H52" s="64"/>
-      <c r="I52" s="64"/>
-      <c r="J52" s="64"/>
-      <c r="K52" s="64"/>
+      <c r="C52" s="68"/>
+      <c r="D52" s="68"/>
+      <c r="E52" s="68"/>
+      <c r="F52" s="68"/>
+      <c r="G52" s="68"/>
+      <c r="H52" s="68"/>
+      <c r="I52" s="68"/>
+      <c r="J52" s="68"/>
+      <c r="K52" s="68"/>
       <c r="L52" s="32"/>
       <c r="M52"/>
       <c r="N52"/>
@@ -4424,20 +4439,20 @@
     </row>
     <row r="53" spans="1:16">
       <c r="A53" s="32"/>
-      <c r="B53" s="52" t="s">
+      <c r="B53" s="73" t="s">
         <v>88</v>
       </c>
-      <c r="C53" s="52"/>
-      <c r="D53" s="52"/>
-      <c r="E53" s="52"/>
-      <c r="F53" s="52"/>
-      <c r="G53" s="53" t="s">
+      <c r="C53" s="73"/>
+      <c r="D53" s="73"/>
+      <c r="E53" s="73"/>
+      <c r="F53" s="73"/>
+      <c r="G53" s="74" t="s">
         <v>89</v>
       </c>
-      <c r="H53" s="53"/>
-      <c r="I53" s="53"/>
-      <c r="J53" s="53"/>
-      <c r="K53" s="53"/>
+      <c r="H53" s="74"/>
+      <c r="I53" s="74"/>
+      <c r="J53" s="74"/>
+      <c r="K53" s="74"/>
       <c r="L53" s="32"/>
       <c r="M53"/>
       <c r="N53"/>
@@ -4446,20 +4461,20 @@
     </row>
     <row r="54" spans="1:16">
       <c r="A54" s="32"/>
-      <c r="B54" s="54" t="s">
+      <c r="B54" s="71" t="s">
         <v>90</v>
       </c>
-      <c r="C54" s="54"/>
-      <c r="D54" s="54"/>
-      <c r="E54" s="54"/>
-      <c r="F54" s="54"/>
-      <c r="G54" s="55">
+      <c r="C54" s="71"/>
+      <c r="D54" s="71"/>
+      <c r="E54" s="71"/>
+      <c r="F54" s="71"/>
+      <c r="G54" s="72">
         <v>1349</v>
       </c>
-      <c r="H54" s="55"/>
-      <c r="I54" s="55"/>
-      <c r="J54" s="55"/>
-      <c r="K54" s="55"/>
+      <c r="H54" s="72"/>
+      <c r="I54" s="72"/>
+      <c r="J54" s="72"/>
+      <c r="K54" s="72"/>
       <c r="L54" s="32"/>
       <c r="M54"/>
       <c r="N54"/>
@@ -4468,20 +4483,20 @@
     </row>
     <row r="55" spans="1:16">
       <c r="A55" s="32"/>
-      <c r="B55" s="52" t="s">
+      <c r="B55" s="73" t="s">
         <v>91</v>
       </c>
-      <c r="C55" s="52"/>
-      <c r="D55" s="52"/>
-      <c r="E55" s="52"/>
-      <c r="F55" s="52"/>
-      <c r="G55" s="53">
+      <c r="C55" s="73"/>
+      <c r="D55" s="73"/>
+      <c r="E55" s="73"/>
+      <c r="F55" s="73"/>
+      <c r="G55" s="74">
         <v>1555</v>
       </c>
-      <c r="H55" s="53"/>
-      <c r="I55" s="53"/>
-      <c r="J55" s="53"/>
-      <c r="K55" s="53"/>
+      <c r="H55" s="74"/>
+      <c r="I55" s="74"/>
+      <c r="J55" s="74"/>
+      <c r="K55" s="74"/>
       <c r="L55" s="32"/>
       <c r="M55"/>
       <c r="N55"/>
@@ -4490,20 +4505,20 @@
     </row>
     <row r="56" spans="1:16">
       <c r="A56" s="32"/>
-      <c r="B56" s="54" t="s">
+      <c r="B56" s="71" t="s">
         <v>92</v>
       </c>
-      <c r="C56" s="54"/>
-      <c r="D56" s="54"/>
-      <c r="E56" s="54"/>
-      <c r="F56" s="54"/>
-      <c r="G56" s="55" t="s">
+      <c r="C56" s="71"/>
+      <c r="D56" s="71"/>
+      <c r="E56" s="71"/>
+      <c r="F56" s="71"/>
+      <c r="G56" s="72" t="s">
         <v>93</v>
       </c>
-      <c r="H56" s="55"/>
-      <c r="I56" s="55"/>
-      <c r="J56" s="55"/>
-      <c r="K56" s="55"/>
+      <c r="H56" s="72"/>
+      <c r="I56" s="72"/>
+      <c r="J56" s="72"/>
+      <c r="K56" s="72"/>
       <c r="L56" s="32"/>
       <c r="M56"/>
       <c r="N56"/>
@@ -4512,20 +4527,20 @@
     </row>
     <row r="57" spans="1:16">
       <c r="A57" s="32"/>
-      <c r="B57" s="52" t="s">
+      <c r="B57" s="73" t="s">
         <v>94</v>
       </c>
-      <c r="C57" s="52"/>
-      <c r="D57" s="52"/>
-      <c r="E57" s="52"/>
-      <c r="F57" s="52"/>
-      <c r="G57" s="53" t="s">
+      <c r="C57" s="73"/>
+      <c r="D57" s="73"/>
+      <c r="E57" s="73"/>
+      <c r="F57" s="73"/>
+      <c r="G57" s="74" t="s">
         <v>95</v>
       </c>
-      <c r="H57" s="53"/>
-      <c r="I57" s="53"/>
-      <c r="J57" s="53"/>
-      <c r="K57" s="53"/>
+      <c r="H57" s="74"/>
+      <c r="I57" s="74"/>
+      <c r="J57" s="74"/>
+      <c r="K57" s="74"/>
       <c r="L57" s="32"/>
       <c r="M57"/>
       <c r="N57"/>
@@ -4534,20 +4549,20 @@
     </row>
     <row r="58" spans="1:16">
       <c r="A58" s="32"/>
-      <c r="B58" s="54" t="s">
+      <c r="B58" s="71" t="s">
         <v>96</v>
       </c>
-      <c r="C58" s="54"/>
-      <c r="D58" s="54"/>
-      <c r="E58" s="54"/>
-      <c r="F58" s="54"/>
-      <c r="G58" s="55" t="s">
+      <c r="C58" s="71"/>
+      <c r="D58" s="71"/>
+      <c r="E58" s="71"/>
+      <c r="F58" s="71"/>
+      <c r="G58" s="72" t="s">
         <v>97</v>
       </c>
-      <c r="H58" s="55"/>
-      <c r="I58" s="55"/>
-      <c r="J58" s="55"/>
-      <c r="K58" s="55"/>
+      <c r="H58" s="72"/>
+      <c r="I58" s="72"/>
+      <c r="J58" s="72"/>
+      <c r="K58" s="72"/>
       <c r="L58" s="32"/>
       <c r="M58"/>
       <c r="N58"/>
@@ -4556,20 +4571,20 @@
     </row>
     <row r="59" spans="1:16">
       <c r="A59" s="32"/>
-      <c r="B59" s="52" t="s">
+      <c r="B59" s="73" t="s">
         <v>98</v>
       </c>
-      <c r="C59" s="52"/>
-      <c r="D59" s="52"/>
-      <c r="E59" s="52"/>
-      <c r="F59" s="52"/>
-      <c r="G59" s="53" t="s">
+      <c r="C59" s="73"/>
+      <c r="D59" s="73"/>
+      <c r="E59" s="73"/>
+      <c r="F59" s="73"/>
+      <c r="G59" s="74" t="s">
         <v>99</v>
       </c>
-      <c r="H59" s="53"/>
-      <c r="I59" s="53"/>
-      <c r="J59" s="53"/>
-      <c r="K59" s="53"/>
+      <c r="H59" s="74"/>
+      <c r="I59" s="74"/>
+      <c r="J59" s="74"/>
+      <c r="K59" s="74"/>
       <c r="L59" s="32"/>
       <c r="M59"/>
       <c r="N59"/>
@@ -4578,20 +4593,20 @@
     </row>
     <row r="60" spans="1:16">
       <c r="A60" s="32"/>
-      <c r="B60" s="54" t="s">
+      <c r="B60" s="71" t="s">
         <v>100</v>
       </c>
-      <c r="C60" s="54"/>
-      <c r="D60" s="54"/>
-      <c r="E60" s="54"/>
-      <c r="F60" s="54"/>
-      <c r="G60" s="55" t="s">
+      <c r="C60" s="71"/>
+      <c r="D60" s="71"/>
+      <c r="E60" s="71"/>
+      <c r="F60" s="71"/>
+      <c r="G60" s="72" t="s">
         <v>101</v>
       </c>
-      <c r="H60" s="55"/>
-      <c r="I60" s="55"/>
-      <c r="J60" s="55"/>
-      <c r="K60" s="55"/>
+      <c r="H60" s="72"/>
+      <c r="I60" s="72"/>
+      <c r="J60" s="72"/>
+      <c r="K60" s="72"/>
       <c r="L60" s="32"/>
       <c r="M60"/>
       <c r="N60"/>
@@ -4600,20 +4615,20 @@
     </row>
     <row r="61" spans="1:16">
       <c r="A61" s="32"/>
-      <c r="B61" s="52" t="s">
+      <c r="B61" s="73" t="s">
         <v>102</v>
       </c>
-      <c r="C61" s="52"/>
-      <c r="D61" s="52"/>
-      <c r="E61" s="52"/>
-      <c r="F61" s="52"/>
-      <c r="G61" s="53" t="s">
+      <c r="C61" s="73"/>
+      <c r="D61" s="73"/>
+      <c r="E61" s="73"/>
+      <c r="F61" s="73"/>
+      <c r="G61" s="74" t="s">
         <v>103</v>
       </c>
-      <c r="H61" s="53"/>
-      <c r="I61" s="53"/>
-      <c r="J61" s="53"/>
-      <c r="K61" s="53"/>
+      <c r="H61" s="74"/>
+      <c r="I61" s="74"/>
+      <c r="J61" s="74"/>
+      <c r="K61" s="74"/>
       <c r="L61" s="32"/>
       <c r="M61"/>
       <c r="N61"/>
@@ -4622,20 +4637,20 @@
     </row>
     <row r="62" spans="1:16">
       <c r="A62" s="32"/>
-      <c r="B62" s="54" t="s">
+      <c r="B62" s="71" t="s">
         <v>104</v>
       </c>
-      <c r="C62" s="54"/>
-      <c r="D62" s="54"/>
-      <c r="E62" s="54"/>
-      <c r="F62" s="54"/>
-      <c r="G62" s="55" t="s">
+      <c r="C62" s="71"/>
+      <c r="D62" s="71"/>
+      <c r="E62" s="71"/>
+      <c r="F62" s="71"/>
+      <c r="G62" s="72" t="s">
         <v>105</v>
       </c>
-      <c r="H62" s="55"/>
-      <c r="I62" s="55"/>
-      <c r="J62" s="55"/>
-      <c r="K62" s="55"/>
+      <c r="H62" s="72"/>
+      <c r="I62" s="72"/>
+      <c r="J62" s="72"/>
+      <c r="K62" s="72"/>
       <c r="L62" s="32"/>
       <c r="M62"/>
       <c r="N62"/>
@@ -4644,20 +4659,20 @@
     </row>
     <row r="63" spans="1:16">
       <c r="A63" s="32"/>
-      <c r="B63" s="52" t="s">
+      <c r="B63" s="73" t="s">
         <v>106</v>
       </c>
-      <c r="C63" s="52"/>
-      <c r="D63" s="52"/>
-      <c r="E63" s="52"/>
-      <c r="F63" s="52"/>
-      <c r="G63" s="53" t="s">
+      <c r="C63" s="73"/>
+      <c r="D63" s="73"/>
+      <c r="E63" s="73"/>
+      <c r="F63" s="73"/>
+      <c r="G63" s="74" t="s">
         <v>107</v>
       </c>
-      <c r="H63" s="53"/>
-      <c r="I63" s="53"/>
-      <c r="J63" s="53"/>
-      <c r="K63" s="53"/>
+      <c r="H63" s="74"/>
+      <c r="I63" s="74"/>
+      <c r="J63" s="74"/>
+      <c r="K63" s="74"/>
       <c r="L63" s="32"/>
       <c r="M63"/>
       <c r="N63"/>
@@ -4666,20 +4681,20 @@
     </row>
     <row r="64" spans="1:16">
       <c r="A64" s="32"/>
-      <c r="B64" s="54" t="s">
+      <c r="B64" s="71" t="s">
         <v>108</v>
       </c>
-      <c r="C64" s="54"/>
-      <c r="D64" s="54"/>
-      <c r="E64" s="54"/>
-      <c r="F64" s="54"/>
-      <c r="G64" s="55">
+      <c r="C64" s="71"/>
+      <c r="D64" s="71"/>
+      <c r="E64" s="71"/>
+      <c r="F64" s="71"/>
+      <c r="G64" s="72">
         <v>166</v>
       </c>
-      <c r="H64" s="55"/>
-      <c r="I64" s="55"/>
-      <c r="J64" s="55"/>
-      <c r="K64" s="55"/>
+      <c r="H64" s="72"/>
+      <c r="I64" s="72"/>
+      <c r="J64" s="72"/>
+      <c r="K64" s="72"/>
       <c r="L64" s="32"/>
       <c r="M64"/>
       <c r="N64"/>
@@ -4688,20 +4703,20 @@
     </row>
     <row r="65" spans="1:16">
       <c r="A65" s="32"/>
-      <c r="B65" s="52" t="s">
+      <c r="B65" s="73" t="s">
         <v>109</v>
       </c>
-      <c r="C65" s="52"/>
-      <c r="D65" s="52"/>
-      <c r="E65" s="52"/>
-      <c r="F65" s="52"/>
-      <c r="G65" s="53" t="s">
+      <c r="C65" s="73"/>
+      <c r="D65" s="73"/>
+      <c r="E65" s="73"/>
+      <c r="F65" s="73"/>
+      <c r="G65" s="74" t="s">
         <v>110</v>
       </c>
-      <c r="H65" s="53"/>
-      <c r="I65" s="53"/>
-      <c r="J65" s="53"/>
-      <c r="K65" s="53"/>
+      <c r="H65" s="74"/>
+      <c r="I65" s="74"/>
+      <c r="J65" s="74"/>
+      <c r="K65" s="74"/>
       <c r="L65" s="32"/>
       <c r="M65"/>
       <c r="N65"/>
@@ -4710,20 +4725,20 @@
     </row>
     <row r="66" spans="1:16">
       <c r="A66" s="32"/>
-      <c r="B66" s="54" t="s">
+      <c r="B66" s="71" t="s">
         <v>111</v>
       </c>
-      <c r="C66" s="54"/>
-      <c r="D66" s="54"/>
-      <c r="E66" s="54"/>
-      <c r="F66" s="54"/>
-      <c r="G66" s="55" t="s">
+      <c r="C66" s="71"/>
+      <c r="D66" s="71"/>
+      <c r="E66" s="71"/>
+      <c r="F66" s="71"/>
+      <c r="G66" s="72" t="s">
         <v>112</v>
       </c>
-      <c r="H66" s="55"/>
-      <c r="I66" s="55"/>
-      <c r="J66" s="55"/>
-      <c r="K66" s="55"/>
+      <c r="H66" s="72"/>
+      <c r="I66" s="72"/>
+      <c r="J66" s="72"/>
+      <c r="K66" s="72"/>
       <c r="L66" s="32"/>
       <c r="M66"/>
       <c r="N66"/>
@@ -4732,20 +4747,20 @@
     </row>
     <row r="67" spans="1:16">
       <c r="A67" s="32"/>
-      <c r="B67" s="52" t="s">
+      <c r="B67" s="73" t="s">
         <v>113</v>
       </c>
-      <c r="C67" s="52"/>
-      <c r="D67" s="52"/>
-      <c r="E67" s="52"/>
-      <c r="F67" s="52"/>
-      <c r="G67" s="53" t="s">
+      <c r="C67" s="73"/>
+      <c r="D67" s="73"/>
+      <c r="E67" s="73"/>
+      <c r="F67" s="73"/>
+      <c r="G67" s="74" t="s">
         <v>114</v>
       </c>
-      <c r="H67" s="53"/>
-      <c r="I67" s="53"/>
-      <c r="J67" s="53"/>
-      <c r="K67" s="53"/>
+      <c r="H67" s="74"/>
+      <c r="I67" s="74"/>
+      <c r="J67" s="74"/>
+      <c r="K67" s="74"/>
       <c r="L67" s="32"/>
       <c r="M67"/>
       <c r="N67"/>
@@ -4754,20 +4769,20 @@
     </row>
     <row r="68" spans="1:16">
       <c r="A68" s="32"/>
-      <c r="B68" s="54" t="s">
+      <c r="B68" s="71" t="s">
         <v>115</v>
       </c>
-      <c r="C68" s="54"/>
-      <c r="D68" s="54"/>
-      <c r="E68" s="54"/>
-      <c r="F68" s="54"/>
-      <c r="G68" s="55" t="s">
+      <c r="C68" s="71"/>
+      <c r="D68" s="71"/>
+      <c r="E68" s="71"/>
+      <c r="F68" s="71"/>
+      <c r="G68" s="72" t="s">
         <v>116</v>
       </c>
-      <c r="H68" s="55"/>
-      <c r="I68" s="55"/>
-      <c r="J68" s="55"/>
-      <c r="K68" s="55"/>
+      <c r="H68" s="72"/>
+      <c r="I68" s="72"/>
+      <c r="J68" s="72"/>
+      <c r="K68" s="72"/>
       <c r="L68" s="32"/>
       <c r="M68"/>
       <c r="N68"/>
@@ -4776,20 +4791,20 @@
     </row>
     <row r="69" spans="1:16">
       <c r="A69" s="32"/>
-      <c r="B69" s="52" t="s">
+      <c r="B69" s="73" t="s">
         <v>117</v>
       </c>
-      <c r="C69" s="52"/>
-      <c r="D69" s="52"/>
-      <c r="E69" s="52"/>
-      <c r="F69" s="52"/>
-      <c r="G69" s="53" t="s">
+      <c r="C69" s="73"/>
+      <c r="D69" s="73"/>
+      <c r="E69" s="73"/>
+      <c r="F69" s="73"/>
+      <c r="G69" s="74" t="s">
         <v>118</v>
       </c>
-      <c r="H69" s="53"/>
-      <c r="I69" s="53"/>
-      <c r="J69" s="53"/>
-      <c r="K69" s="53"/>
+      <c r="H69" s="74"/>
+      <c r="I69" s="74"/>
+      <c r="J69" s="74"/>
+      <c r="K69" s="74"/>
       <c r="L69" s="32"/>
       <c r="M69"/>
       <c r="N69"/>
@@ -4798,20 +4813,20 @@
     </row>
     <row r="70" spans="1:16">
       <c r="A70" s="32"/>
-      <c r="B70" s="54" t="s">
+      <c r="B70" s="71" t="s">
         <v>119</v>
       </c>
-      <c r="C70" s="54"/>
-      <c r="D70" s="54"/>
-      <c r="E70" s="54"/>
-      <c r="F70" s="54"/>
-      <c r="G70" s="55" t="s">
+      <c r="C70" s="71"/>
+      <c r="D70" s="71"/>
+      <c r="E70" s="71"/>
+      <c r="F70" s="71"/>
+      <c r="G70" s="72" t="s">
         <v>120</v>
       </c>
-      <c r="H70" s="55"/>
-      <c r="I70" s="55"/>
-      <c r="J70" s="55"/>
-      <c r="K70" s="55"/>
+      <c r="H70" s="72"/>
+      <c r="I70" s="72"/>
+      <c r="J70" s="72"/>
+      <c r="K70" s="72"/>
       <c r="L70" s="32"/>
       <c r="M70"/>
       <c r="N70"/>
@@ -4820,20 +4835,20 @@
     </row>
     <row r="71" spans="1:16">
       <c r="A71" s="32"/>
-      <c r="B71" s="52" t="s">
+      <c r="B71" s="73" t="s">
         <v>121</v>
       </c>
-      <c r="C71" s="52"/>
-      <c r="D71" s="52"/>
-      <c r="E71" s="52"/>
-      <c r="F71" s="52"/>
-      <c r="G71" s="53" t="s">
+      <c r="C71" s="73"/>
+      <c r="D71" s="73"/>
+      <c r="E71" s="73"/>
+      <c r="F71" s="73"/>
+      <c r="G71" s="74" t="s">
         <v>122</v>
       </c>
-      <c r="H71" s="53"/>
-      <c r="I71" s="53"/>
-      <c r="J71" s="53"/>
-      <c r="K71" s="53"/>
+      <c r="H71" s="74"/>
+      <c r="I71" s="74"/>
+      <c r="J71" s="74"/>
+      <c r="K71" s="74"/>
       <c r="L71" s="32"/>
       <c r="M71"/>
       <c r="N71"/>
@@ -4842,20 +4857,20 @@
     </row>
     <row r="72" spans="1:16">
       <c r="A72" s="32"/>
-      <c r="B72" s="54" t="s">
+      <c r="B72" s="71" t="s">
         <v>123</v>
       </c>
-      <c r="C72" s="54"/>
-      <c r="D72" s="54"/>
-      <c r="E72" s="54"/>
-      <c r="F72" s="54"/>
-      <c r="G72" s="55" t="s">
+      <c r="C72" s="71"/>
+      <c r="D72" s="71"/>
+      <c r="E72" s="71"/>
+      <c r="F72" s="71"/>
+      <c r="G72" s="72" t="s">
         <v>124</v>
       </c>
-      <c r="H72" s="55"/>
-      <c r="I72" s="55"/>
-      <c r="J72" s="55"/>
-      <c r="K72" s="55"/>
+      <c r="H72" s="72"/>
+      <c r="I72" s="72"/>
+      <c r="J72" s="72"/>
+      <c r="K72" s="72"/>
       <c r="L72" s="32"/>
       <c r="M72"/>
       <c r="N72"/>
@@ -4864,20 +4879,20 @@
     </row>
     <row r="73" spans="1:16">
       <c r="A73" s="32"/>
-      <c r="B73" s="52" t="s">
+      <c r="B73" s="73" t="s">
         <v>125</v>
       </c>
-      <c r="C73" s="52"/>
-      <c r="D73" s="52"/>
-      <c r="E73" s="52"/>
-      <c r="F73" s="52"/>
-      <c r="G73" s="56" t="s">
+      <c r="C73" s="73"/>
+      <c r="D73" s="73"/>
+      <c r="E73" s="73"/>
+      <c r="F73" s="73"/>
+      <c r="G73" s="86" t="s">
         <v>126</v>
       </c>
-      <c r="H73" s="56"/>
-      <c r="I73" s="56"/>
-      <c r="J73" s="56"/>
-      <c r="K73" s="56"/>
+      <c r="H73" s="86"/>
+      <c r="I73" s="86"/>
+      <c r="J73" s="86"/>
+      <c r="K73" s="86"/>
       <c r="L73" s="32"/>
       <c r="M73"/>
       <c r="N73"/>
@@ -4886,20 +4901,20 @@
     </row>
     <row r="74" spans="1:16">
       <c r="A74" s="32"/>
-      <c r="B74" s="54" t="s">
+      <c r="B74" s="71" t="s">
         <v>127</v>
       </c>
-      <c r="C74" s="54"/>
-      <c r="D74" s="54"/>
-      <c r="E74" s="54"/>
-      <c r="F74" s="54"/>
-      <c r="G74" s="57" t="s">
+      <c r="C74" s="71"/>
+      <c r="D74" s="71"/>
+      <c r="E74" s="71"/>
+      <c r="F74" s="71"/>
+      <c r="G74" s="87" t="s">
         <v>128</v>
       </c>
-      <c r="H74" s="57"/>
-      <c r="I74" s="57"/>
-      <c r="J74" s="57"/>
-      <c r="K74" s="57"/>
+      <c r="H74" s="87"/>
+      <c r="I74" s="87"/>
+      <c r="J74" s="87"/>
+      <c r="K74" s="87"/>
       <c r="L74" s="32"/>
       <c r="M74"/>
       <c r="N74"/>
@@ -5036,148 +5051,6 @@
     <row r="120" customFormat="1"/>
   </sheetData>
   <mergeCells count="166">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="B9:K9"/>
-    <mergeCell ref="B12:K12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="E13:G13"/>
-    <mergeCell ref="H13:K13"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="E14:G14"/>
-    <mergeCell ref="H14:K14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="H15:K15"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="E16:G16"/>
-    <mergeCell ref="H16:K16"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="E17:G17"/>
-    <mergeCell ref="H17:K17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="H18:K18"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="H19:K19"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="H20:K20"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="H21:K21"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="H22:K22"/>
-    <mergeCell ref="B24:K24"/>
-    <mergeCell ref="B25:F25"/>
-    <mergeCell ref="G25:K25"/>
-    <mergeCell ref="L25:M25"/>
-    <mergeCell ref="B26:F26"/>
-    <mergeCell ref="G26:K26"/>
-    <mergeCell ref="L26:M26"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="G27:K27"/>
-    <mergeCell ref="L27:M27"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="G28:K28"/>
-    <mergeCell ref="L28:M28"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="G29:K29"/>
-    <mergeCell ref="L29:M29"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="G30:K30"/>
-    <mergeCell ref="L30:M30"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="G31:K31"/>
-    <mergeCell ref="L31:M31"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="G32:K32"/>
-    <mergeCell ref="L32:M32"/>
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="G33:K33"/>
-    <mergeCell ref="L33:M33"/>
-    <mergeCell ref="B34:F34"/>
-    <mergeCell ref="G34:K34"/>
-    <mergeCell ref="L34:M34"/>
-    <mergeCell ref="B35:F35"/>
-    <mergeCell ref="G35:K35"/>
-    <mergeCell ref="L35:M35"/>
-    <mergeCell ref="B36:F36"/>
-    <mergeCell ref="G36:K36"/>
-    <mergeCell ref="L36:M36"/>
-    <mergeCell ref="B37:F37"/>
-    <mergeCell ref="G37:K37"/>
-    <mergeCell ref="L37:M37"/>
-    <mergeCell ref="B38:F38"/>
-    <mergeCell ref="G38:K38"/>
-    <mergeCell ref="L38:M38"/>
-    <mergeCell ref="B39:F39"/>
-    <mergeCell ref="G39:K39"/>
-    <mergeCell ref="L39:M39"/>
-    <mergeCell ref="B40:F40"/>
-    <mergeCell ref="G40:K40"/>
-    <mergeCell ref="L40:M40"/>
-    <mergeCell ref="B41:F41"/>
-    <mergeCell ref="G41:K41"/>
-    <mergeCell ref="L41:M41"/>
-    <mergeCell ref="B42:F42"/>
-    <mergeCell ref="G42:K42"/>
-    <mergeCell ref="L42:M42"/>
-    <mergeCell ref="B43:F43"/>
-    <mergeCell ref="G43:K43"/>
-    <mergeCell ref="L43:M43"/>
-    <mergeCell ref="B44:F44"/>
-    <mergeCell ref="G44:K44"/>
-    <mergeCell ref="L44:M44"/>
-    <mergeCell ref="B45:F45"/>
-    <mergeCell ref="G45:K45"/>
-    <mergeCell ref="L45:M45"/>
-    <mergeCell ref="B46:F46"/>
-    <mergeCell ref="G46:K46"/>
-    <mergeCell ref="L46:M46"/>
-    <mergeCell ref="B47:F47"/>
-    <mergeCell ref="G47:K47"/>
-    <mergeCell ref="L47:M47"/>
-    <mergeCell ref="B48:F48"/>
-    <mergeCell ref="G48:K48"/>
-    <mergeCell ref="L48:M48"/>
-    <mergeCell ref="B49:F49"/>
-    <mergeCell ref="G49:K49"/>
-    <mergeCell ref="L49:M49"/>
-    <mergeCell ref="B50:F50"/>
-    <mergeCell ref="G50:K50"/>
-    <mergeCell ref="L50:M50"/>
-    <mergeCell ref="B52:K52"/>
-    <mergeCell ref="B53:F53"/>
-    <mergeCell ref="G53:K53"/>
-    <mergeCell ref="B54:F54"/>
-    <mergeCell ref="G54:K54"/>
-    <mergeCell ref="B55:F55"/>
-    <mergeCell ref="G55:K55"/>
-    <mergeCell ref="B56:F56"/>
-    <mergeCell ref="G56:K56"/>
-    <mergeCell ref="B57:F57"/>
-    <mergeCell ref="G57:K57"/>
-    <mergeCell ref="B58:F58"/>
-    <mergeCell ref="G58:K58"/>
-    <mergeCell ref="B59:F59"/>
-    <mergeCell ref="G59:K59"/>
-    <mergeCell ref="B60:F60"/>
-    <mergeCell ref="G60:K60"/>
-    <mergeCell ref="G69:K69"/>
-    <mergeCell ref="B70:F70"/>
-    <mergeCell ref="G70:K70"/>
-    <mergeCell ref="B61:F61"/>
-    <mergeCell ref="G61:K61"/>
-    <mergeCell ref="B62:F62"/>
-    <mergeCell ref="G62:K62"/>
-    <mergeCell ref="B63:F63"/>
-    <mergeCell ref="G63:K63"/>
-    <mergeCell ref="B64:F64"/>
-    <mergeCell ref="G64:K64"/>
-    <mergeCell ref="B65:F65"/>
-    <mergeCell ref="G65:K65"/>
     <mergeCell ref="B77:F77"/>
     <mergeCell ref="G77:K77"/>
     <mergeCell ref="B78:F78"/>
@@ -5202,6 +5075,148 @@
     <mergeCell ref="B68:F68"/>
     <mergeCell ref="G68:K68"/>
     <mergeCell ref="B69:F69"/>
+    <mergeCell ref="G69:K69"/>
+    <mergeCell ref="B70:F70"/>
+    <mergeCell ref="G70:K70"/>
+    <mergeCell ref="B61:F61"/>
+    <mergeCell ref="G61:K61"/>
+    <mergeCell ref="B62:F62"/>
+    <mergeCell ref="G62:K62"/>
+    <mergeCell ref="B63:F63"/>
+    <mergeCell ref="G63:K63"/>
+    <mergeCell ref="B64:F64"/>
+    <mergeCell ref="G64:K64"/>
+    <mergeCell ref="B65:F65"/>
+    <mergeCell ref="G65:K65"/>
+    <mergeCell ref="B56:F56"/>
+    <mergeCell ref="G56:K56"/>
+    <mergeCell ref="B57:F57"/>
+    <mergeCell ref="G57:K57"/>
+    <mergeCell ref="B58:F58"/>
+    <mergeCell ref="G58:K58"/>
+    <mergeCell ref="B59:F59"/>
+    <mergeCell ref="G59:K59"/>
+    <mergeCell ref="B60:F60"/>
+    <mergeCell ref="G60:K60"/>
+    <mergeCell ref="B50:F50"/>
+    <mergeCell ref="G50:K50"/>
+    <mergeCell ref="L50:M50"/>
+    <mergeCell ref="B52:K52"/>
+    <mergeCell ref="B53:F53"/>
+    <mergeCell ref="G53:K53"/>
+    <mergeCell ref="B54:F54"/>
+    <mergeCell ref="G54:K54"/>
+    <mergeCell ref="B55:F55"/>
+    <mergeCell ref="G55:K55"/>
+    <mergeCell ref="B47:F47"/>
+    <mergeCell ref="G47:K47"/>
+    <mergeCell ref="L47:M47"/>
+    <mergeCell ref="B48:F48"/>
+    <mergeCell ref="G48:K48"/>
+    <mergeCell ref="L48:M48"/>
+    <mergeCell ref="B49:F49"/>
+    <mergeCell ref="G49:K49"/>
+    <mergeCell ref="L49:M49"/>
+    <mergeCell ref="B44:F44"/>
+    <mergeCell ref="G44:K44"/>
+    <mergeCell ref="L44:M44"/>
+    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="G45:K45"/>
+    <mergeCell ref="L45:M45"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="G46:K46"/>
+    <mergeCell ref="L46:M46"/>
+    <mergeCell ref="B41:F41"/>
+    <mergeCell ref="G41:K41"/>
+    <mergeCell ref="L41:M41"/>
+    <mergeCell ref="B42:F42"/>
+    <mergeCell ref="G42:K42"/>
+    <mergeCell ref="L42:M42"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="G43:K43"/>
+    <mergeCell ref="L43:M43"/>
+    <mergeCell ref="B38:F38"/>
+    <mergeCell ref="G38:K38"/>
+    <mergeCell ref="L38:M38"/>
+    <mergeCell ref="B39:F39"/>
+    <mergeCell ref="G39:K39"/>
+    <mergeCell ref="L39:M39"/>
+    <mergeCell ref="B40:F40"/>
+    <mergeCell ref="G40:K40"/>
+    <mergeCell ref="L40:M40"/>
+    <mergeCell ref="B35:F35"/>
+    <mergeCell ref="G35:K35"/>
+    <mergeCell ref="L35:M35"/>
+    <mergeCell ref="B36:F36"/>
+    <mergeCell ref="G36:K36"/>
+    <mergeCell ref="L36:M36"/>
+    <mergeCell ref="B37:F37"/>
+    <mergeCell ref="G37:K37"/>
+    <mergeCell ref="L37:M37"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="G32:K32"/>
+    <mergeCell ref="L32:M32"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="G33:K33"/>
+    <mergeCell ref="L33:M33"/>
+    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="G34:K34"/>
+    <mergeCell ref="L34:M34"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="G29:K29"/>
+    <mergeCell ref="L29:M29"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="G30:K30"/>
+    <mergeCell ref="L30:M30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="G31:K31"/>
+    <mergeCell ref="L31:M31"/>
+    <mergeCell ref="L25:M25"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="G26:K26"/>
+    <mergeCell ref="L26:M26"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="G27:K27"/>
+    <mergeCell ref="L27:M27"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="G28:K28"/>
+    <mergeCell ref="L28:M28"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="H21:K21"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="H22:K22"/>
+    <mergeCell ref="B24:K24"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="G25:K25"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="H18:K18"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="H19:K19"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="H20:K20"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="H15:K15"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="H16:K16"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="E17:G17"/>
+    <mergeCell ref="H17:K17"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="B9:K9"/>
+    <mergeCell ref="B12:K12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="H13:K13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="H14:K14"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="L30" r:id="rId1" tooltip="mailto:ccfi_sugbu@yahoo.com" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -6645,7 +6660,7 @@
         <v>449</v>
       </c>
       <c r="D2" s="35" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>132</v>
@@ -6687,7 +6702,7 @@
         <v>458</v>
       </c>
       <c r="D3" s="36" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>459</v>
@@ -6721,7 +6736,7 @@
         <v>463</v>
       </c>
       <c r="D4" s="36" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>464</v>
@@ -6763,7 +6778,7 @@
         <v>470</v>
       </c>
       <c r="D5" s="36" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>471</v>
@@ -6805,7 +6820,7 @@
         <v>477</v>
       </c>
       <c r="D6" s="36" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>478</v>
@@ -6847,10 +6862,10 @@
         <v>484</v>
       </c>
       <c r="D7" s="36" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>485</v>
@@ -6889,10 +6904,10 @@
         <v>491</v>
       </c>
       <c r="D8" s="36" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>492</v>
@@ -6910,7 +6925,7 @@
         <v>30</v>
       </c>
       <c r="K8" s="44" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="L8" s="6">
         <v>2</v>
@@ -6931,7 +6946,7 @@
         <v>497</v>
       </c>
       <c r="D9" s="36" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>498</v>
@@ -6952,7 +6967,7 @@
         <v>30</v>
       </c>
       <c r="K9" s="45" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="L9" s="3">
         <v>30</v>
@@ -6973,7 +6988,7 @@
         <v>503</v>
       </c>
       <c r="D10" s="36" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>504</v>
@@ -7007,7 +7022,7 @@
         <v>510</v>
       </c>
       <c r="D11" s="36" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>511</v>
@@ -7041,10 +7056,10 @@
         <v>517</v>
       </c>
       <c r="D12" s="36" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>518</v>
@@ -7075,7 +7090,7 @@
         <v>522</v>
       </c>
       <c r="D13" s="36" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>511</v>
@@ -7096,7 +7111,7 @@
         <v>57</v>
       </c>
       <c r="K13" s="45" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="L13" s="3">
         <v>26</v>
@@ -7110,27 +7125,27 @@
       <c r="A14" s="5">
         <v>13</v>
       </c>
-      <c r="B14" s="89" t="s">
+      <c r="B14" s="92" t="s">
+        <v>727</v>
+      </c>
+      <c r="C14" s="92"/>
+      <c r="D14" s="93" t="s">
+        <v>722</v>
+      </c>
+      <c r="E14" s="92" t="s">
         <v>527</v>
       </c>
-      <c r="C14" s="89"/>
-      <c r="D14" s="91" t="s">
-        <v>724</v>
-      </c>
-      <c r="E14" s="89" t="s">
+      <c r="F14" s="6" t="s">
         <v>528</v>
       </c>
-      <c r="F14" s="6" t="s">
-        <v>529</v>
-      </c>
       <c r="G14" s="6" t="s">
+        <v>533</v>
+      </c>
+      <c r="H14" s="34" t="s">
         <v>530</v>
       </c>
-      <c r="H14" s="34" t="s">
+      <c r="I14" s="7" t="s">
         <v>531</v>
-      </c>
-      <c r="I14" s="7" t="s">
-        <v>532</v>
       </c>
       <c r="J14" s="6"/>
       <c r="K14" s="43"/>
@@ -7140,20 +7155,24 @@
     </row>
     <row r="15" spans="1:14" ht="83.25">
       <c r="A15" s="5"/>
-      <c r="B15" s="89"/>
-      <c r="C15" s="89"/>
-      <c r="D15" s="91"/>
-      <c r="E15" s="89"/>
+      <c r="B15" s="92" t="s">
+        <v>728</v>
+      </c>
+      <c r="C15" s="92"/>
+      <c r="D15" s="93"/>
+      <c r="E15" s="6" t="s">
+        <v>726</v>
+      </c>
       <c r="F15" s="6" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="G15" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="H15" s="34" t="s">
         <v>534</v>
       </c>
-      <c r="H15" s="34" t="s">
-        <v>535</v>
-      </c>
-      <c r="I15" s="7"/>
+      <c r="I15" s="94"/>
       <c r="J15" s="6"/>
       <c r="K15" s="43"/>
       <c r="L15" s="6"/>
@@ -7165,34 +7184,34 @@
         <v>14</v>
       </c>
       <c r="B16" s="3" t="s">
+        <v>535</v>
+      </c>
+      <c r="C16" s="3" t="s">
         <v>536</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="D16" s="36" t="s">
+        <v>722</v>
+      </c>
+      <c r="E16" s="3" t="s">
         <v>537</v>
       </c>
-      <c r="D16" s="36" t="s">
-        <v>724</v>
-      </c>
-      <c r="E16" s="3" t="s">
+      <c r="F16" s="3" t="s">
         <v>538</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="G16" s="3" t="s">
         <v>539</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="H16" s="33" t="s">
         <v>540</v>
       </c>
-      <c r="H16" s="33" t="s">
+      <c r="I16" s="4" t="s">
         <v>541</v>
-      </c>
-      <c r="I16" s="4" t="s">
-        <v>542</v>
       </c>
       <c r="J16" s="3">
         <v>20</v>
       </c>
       <c r="K16" s="46" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="L16" s="3"/>
       <c r="M16" s="3">
@@ -7205,26 +7224,26 @@
         <v>15</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="C17" s="6"/>
       <c r="D17" s="36" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>504</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="G17" s="6" t="s">
         <v>506</v>
       </c>
       <c r="H17" s="6" t="s">
+        <v>544</v>
+      </c>
+      <c r="I17" s="7" t="s">
         <v>545</v>
-      </c>
-      <c r="I17" s="7" t="s">
-        <v>546</v>
       </c>
       <c r="J17" s="6"/>
       <c r="K17" s="43"/>
@@ -7237,28 +7256,28 @@
         <v>16</v>
       </c>
       <c r="B18" s="3" t="s">
+        <v>546</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>547</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="D18" s="36" t="s">
+        <v>722</v>
+      </c>
+      <c r="E18" s="3" t="s">
         <v>548</v>
       </c>
-      <c r="D18" s="36" t="s">
-        <v>724</v>
-      </c>
-      <c r="E18" s="3" t="s">
+      <c r="F18" s="3" t="s">
         <v>549</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>550</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>461</v>
       </c>
       <c r="H18" s="33" t="s">
+        <v>550</v>
+      </c>
+      <c r="I18" s="4" t="s">
         <v>551</v>
-      </c>
-      <c r="I18" s="4" t="s">
-        <v>552</v>
       </c>
       <c r="J18" s="3"/>
       <c r="K18" s="10"/>
@@ -7271,34 +7290,34 @@
         <v>17</v>
       </c>
       <c r="B19" s="6" t="s">
+        <v>552</v>
+      </c>
+      <c r="C19" s="6" t="s">
         <v>553</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="D19" s="36" t="s">
+        <v>722</v>
+      </c>
+      <c r="E19" s="6" t="s">
         <v>554</v>
       </c>
-      <c r="D19" s="36" t="s">
-        <v>724</v>
-      </c>
-      <c r="E19" s="6" t="s">
+      <c r="F19" s="6" t="s">
         <v>555</v>
-      </c>
-      <c r="F19" s="6" t="s">
-        <v>556</v>
       </c>
       <c r="G19" s="6" t="s">
         <v>506</v>
       </c>
       <c r="H19" s="34" t="s">
+        <v>556</v>
+      </c>
+      <c r="I19" s="7" t="s">
         <v>557</v>
-      </c>
-      <c r="I19" s="7" t="s">
-        <v>558</v>
       </c>
       <c r="J19" s="6">
         <v>21</v>
       </c>
       <c r="K19" s="44" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="L19" s="6">
         <v>6</v>
@@ -7313,28 +7332,28 @@
         <v>18</v>
       </c>
       <c r="B20" s="3" t="s">
+        <v>558</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>559</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="D20" s="36" t="s">
+        <v>698</v>
+      </c>
+      <c r="E20" s="3" t="s">
         <v>560</v>
       </c>
-      <c r="D20" s="36" t="s">
-        <v>700</v>
-      </c>
-      <c r="E20" s="3" t="s">
+      <c r="F20" s="3" t="s">
         <v>561</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>562</v>
       </c>
       <c r="G20" s="3" t="s">
         <v>506</v>
       </c>
       <c r="H20" s="33" t="s">
+        <v>562</v>
+      </c>
+      <c r="I20" s="4" t="s">
         <v>563</v>
-      </c>
-      <c r="I20" s="4" t="s">
-        <v>564</v>
       </c>
       <c r="J20" s="3"/>
       <c r="K20" s="10"/>
@@ -7347,28 +7366,28 @@
         <v>19</v>
       </c>
       <c r="B21" s="6" t="s">
+        <v>564</v>
+      </c>
+      <c r="C21" s="6" t="s">
         <v>565</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="D21" s="36" t="s">
+        <v>722</v>
+      </c>
+      <c r="E21" s="6" t="s">
         <v>566</v>
       </c>
-      <c r="D21" s="36" t="s">
-        <v>724</v>
-      </c>
-      <c r="E21" s="6" t="s">
+      <c r="F21" s="6" t="s">
         <v>567</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="G21" s="6" t="s">
         <v>568</v>
       </c>
-      <c r="G21" s="6" t="s">
+      <c r="H21" s="34" t="s">
         <v>569</v>
       </c>
-      <c r="H21" s="34" t="s">
+      <c r="I21" s="7" t="s">
         <v>570</v>
-      </c>
-      <c r="I21" s="7" t="s">
-        <v>571</v>
       </c>
       <c r="J21" s="6"/>
       <c r="K21" s="43"/>
@@ -7381,34 +7400,34 @@
         <v>20</v>
       </c>
       <c r="B22" s="3" t="s">
+        <v>571</v>
+      </c>
+      <c r="C22" s="3" t="s">
         <v>572</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="D22" s="36" t="s">
+        <v>722</v>
+      </c>
+      <c r="E22" s="3" t="s">
         <v>573</v>
       </c>
-      <c r="D22" s="36" t="s">
-        <v>724</v>
-      </c>
-      <c r="E22" s="3" t="s">
+      <c r="F22" s="3" t="s">
         <v>574</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="G22" s="3" t="s">
         <v>575</v>
       </c>
-      <c r="G22" s="3" t="s">
+      <c r="H22" s="33" t="s">
         <v>576</v>
       </c>
-      <c r="H22" s="33" t="s">
+      <c r="I22" s="4" t="s">
         <v>577</v>
-      </c>
-      <c r="I22" s="4" t="s">
-        <v>578</v>
       </c>
       <c r="J22" s="3">
         <v>25</v>
       </c>
       <c r="K22" s="45" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="L22" s="3">
         <v>12</v>
@@ -7423,34 +7442,34 @@
         <v>21</v>
       </c>
       <c r="B23" s="6" t="s">
+        <v>578</v>
+      </c>
+      <c r="C23" s="37" t="s">
+        <v>700</v>
+      </c>
+      <c r="D23" s="36" t="s">
+        <v>722</v>
+      </c>
+      <c r="E23" s="6" t="s">
         <v>579</v>
       </c>
-      <c r="C23" s="37" t="s">
-        <v>702</v>
-      </c>
-      <c r="D23" s="36" t="s">
-        <v>724</v>
-      </c>
-      <c r="E23" s="6" t="s">
+      <c r="F23" s="6" t="s">
         <v>580</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="G23" s="6" t="s">
         <v>581</v>
       </c>
-      <c r="G23" s="6" t="s">
+      <c r="H23" s="34" t="s">
         <v>582</v>
       </c>
-      <c r="H23" s="34" t="s">
+      <c r="I23" s="7" t="s">
         <v>583</v>
-      </c>
-      <c r="I23" s="7" t="s">
-        <v>584</v>
       </c>
       <c r="J23" s="6">
         <v>21</v>
       </c>
       <c r="K23" s="49" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="L23" s="6">
         <v>7</v>
@@ -7465,28 +7484,28 @@
         <v>22</v>
       </c>
       <c r="B24" s="3" t="s">
+        <v>584</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>585</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="D24" s="36" t="s">
+        <v>722</v>
+      </c>
+      <c r="E24" s="3" t="s">
         <v>586</v>
       </c>
-      <c r="D24" s="36" t="s">
-        <v>724</v>
-      </c>
-      <c r="E24" s="3" t="s">
+      <c r="F24" s="3" t="s">
         <v>587</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>588</v>
       </c>
       <c r="G24" s="3" t="s">
         <v>506</v>
       </c>
       <c r="H24" s="33" t="s">
+        <v>588</v>
+      </c>
+      <c r="I24" s="4" t="s">
         <v>589</v>
-      </c>
-      <c r="I24" s="4" t="s">
-        <v>590</v>
       </c>
       <c r="J24" s="3"/>
       <c r="K24" s="10"/>
@@ -7499,34 +7518,34 @@
         <v>23</v>
       </c>
       <c r="B25" s="6" t="s">
+        <v>590</v>
+      </c>
+      <c r="C25" s="6" t="s">
         <v>591</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="D25" s="36" t="s">
+        <v>722</v>
+      </c>
+      <c r="E25" s="6" t="s">
         <v>592</v>
       </c>
-      <c r="D25" s="36" t="s">
-        <v>724</v>
-      </c>
-      <c r="E25" s="6" t="s">
+      <c r="F25" s="6" t="s">
         <v>593</v>
       </c>
-      <c r="F25" s="6" t="s">
+      <c r="G25" s="6" t="s">
         <v>594</v>
       </c>
-      <c r="G25" s="6" t="s">
+      <c r="H25" s="34" t="s">
         <v>595</v>
       </c>
-      <c r="H25" s="34" t="s">
+      <c r="I25" s="7" t="s">
         <v>596</v>
-      </c>
-      <c r="I25" s="7" t="s">
-        <v>597</v>
       </c>
       <c r="J25" s="6">
         <v>18</v>
       </c>
       <c r="K25" s="43" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="L25" s="6"/>
       <c r="M25" s="6">
@@ -7539,34 +7558,34 @@
         <v>24</v>
       </c>
       <c r="B26" s="3" t="s">
+        <v>598</v>
+      </c>
+      <c r="C26" s="3" t="s">
         <v>599</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="D26" s="36" t="s">
+        <v>722</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>527</v>
+      </c>
+      <c r="F26" s="3" t="s">
         <v>600</v>
-      </c>
-      <c r="D26" s="36" t="s">
-        <v>724</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>528</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>601</v>
       </c>
       <c r="G26" s="3" t="s">
         <v>493</v>
       </c>
       <c r="H26" s="3" t="s">
+        <v>601</v>
+      </c>
+      <c r="I26" s="4" t="s">
         <v>602</v>
-      </c>
-      <c r="I26" s="4" t="s">
-        <v>603</v>
       </c>
       <c r="J26" s="3">
         <v>22</v>
       </c>
       <c r="K26" s="45" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="L26" s="3">
         <v>0</v>
@@ -7581,34 +7600,34 @@
         <v>25</v>
       </c>
       <c r="B27" s="6" t="s">
+        <v>603</v>
+      </c>
+      <c r="C27" s="6" t="s">
         <v>604</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="D27" s="36" t="s">
+        <v>721</v>
+      </c>
+      <c r="E27" s="6" t="s">
         <v>605</v>
       </c>
-      <c r="D27" s="36" t="s">
-        <v>723</v>
-      </c>
-      <c r="E27" s="6" t="s">
+      <c r="F27" s="6" t="s">
         <v>606</v>
       </c>
-      <c r="F27" s="6" t="s">
+      <c r="G27" s="6" t="s">
+        <v>575</v>
+      </c>
+      <c r="H27" s="34" t="s">
         <v>607</v>
       </c>
-      <c r="G27" s="6" t="s">
-        <v>576</v>
-      </c>
-      <c r="H27" s="34" t="s">
+      <c r="I27" s="7" t="s">
         <v>608</v>
-      </c>
-      <c r="I27" s="7" t="s">
-        <v>609</v>
       </c>
       <c r="J27" s="6">
         <v>15</v>
       </c>
       <c r="K27" s="43" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="L27" s="6">
         <v>5</v>
@@ -7623,34 +7642,34 @@
         <v>26</v>
       </c>
       <c r="B28" s="3" t="s">
+        <v>610</v>
+      </c>
+      <c r="C28" s="3" t="s">
         <v>611</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="D28" s="36" t="s">
+        <v>722</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>717</v>
+      </c>
+      <c r="F28" s="3" t="s">
         <v>612</v>
-      </c>
-      <c r="D28" s="36" t="s">
-        <v>724</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>719</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>613</v>
       </c>
       <c r="G28" s="3" t="s">
         <v>506</v>
       </c>
       <c r="H28" s="33" t="s">
+        <v>613</v>
+      </c>
+      <c r="I28" s="4" t="s">
         <v>614</v>
-      </c>
-      <c r="I28" s="4" t="s">
-        <v>615</v>
       </c>
       <c r="J28" s="3">
         <v>25</v>
       </c>
       <c r="K28" s="10" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="L28" s="3">
         <v>2</v>
@@ -7665,34 +7684,34 @@
         <v>27</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="C29" s="6" t="s">
         <v>470</v>
       </c>
       <c r="D29" s="36" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="E29" s="6" t="s">
+        <v>617</v>
+      </c>
+      <c r="F29" s="6" t="s">
         <v>618</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>619</v>
       </c>
       <c r="G29" s="6" t="s">
         <v>486</v>
       </c>
       <c r="H29" s="34" t="s">
+        <v>619</v>
+      </c>
+      <c r="I29" s="7" t="s">
         <v>620</v>
-      </c>
-      <c r="I29" s="7" t="s">
-        <v>621</v>
       </c>
       <c r="J29" s="6">
         <v>27</v>
       </c>
       <c r="K29" s="43" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="L29" s="6">
         <v>0</v>
@@ -7707,28 +7726,28 @@
         <v>28</v>
       </c>
       <c r="B30" s="3" t="s">
+        <v>622</v>
+      </c>
+      <c r="C30" s="3" t="s">
         <v>623</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="D30" s="36" t="s">
+        <v>720</v>
+      </c>
+      <c r="E30" s="3" t="s">
         <v>624</v>
       </c>
-      <c r="D30" s="36" t="s">
-        <v>722</v>
-      </c>
-      <c r="E30" s="3" t="s">
+      <c r="F30" s="3" t="s">
         <v>625</v>
       </c>
-      <c r="F30" s="3" t="s">
+      <c r="G30" s="3" t="s">
         <v>626</v>
       </c>
-      <c r="G30" s="3" t="s">
+      <c r="H30" s="33" t="s">
         <v>627</v>
       </c>
-      <c r="H30" s="33" t="s">
+      <c r="I30" s="4" t="s">
         <v>628</v>
-      </c>
-      <c r="I30" s="4" t="s">
-        <v>629</v>
       </c>
       <c r="J30" s="3"/>
       <c r="K30" s="10"/>
@@ -7741,34 +7760,34 @@
         <v>29</v>
       </c>
       <c r="B31" s="6" t="s">
+        <v>629</v>
+      </c>
+      <c r="C31" s="6" t="s">
         <v>630</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="D31" s="36" t="s">
+        <v>720</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>718</v>
+      </c>
+      <c r="F31" s="6" t="s">
         <v>631</v>
-      </c>
-      <c r="D31" s="36" t="s">
-        <v>722</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>720</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>632</v>
       </c>
       <c r="G31" s="6" t="s">
         <v>473</v>
       </c>
       <c r="H31" s="34" t="s">
+        <v>632</v>
+      </c>
+      <c r="I31" s="7" t="s">
         <v>633</v>
-      </c>
-      <c r="I31" s="7" t="s">
-        <v>634</v>
       </c>
       <c r="J31" s="6">
         <v>62</v>
       </c>
       <c r="K31" s="43" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="L31" s="6">
         <v>14</v>
@@ -7783,25 +7802,25 @@
         <v>30</v>
       </c>
       <c r="B32" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="C32" s="3" t="s">
         <v>636</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="D32" s="36" t="s">
+        <v>722</v>
+      </c>
+      <c r="E32" s="3" t="s">
         <v>637</v>
       </c>
-      <c r="D32" s="36" t="s">
-        <v>724</v>
-      </c>
-      <c r="E32" s="3" t="s">
+      <c r="F32" s="3" t="s">
         <v>638</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>639</v>
       </c>
       <c r="G32" s="3" t="s">
         <v>473</v>
       </c>
       <c r="H32" s="33" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="I32" s="4" t="s">
         <v>46</v>
@@ -7817,40 +7836,41 @@
         <v>31</v>
       </c>
       <c r="B33" s="6" t="s">
+        <v>640</v>
+      </c>
+      <c r="C33" s="6" t="s">
         <v>641</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="D33" s="36" t="s">
+        <v>722</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>729</v>
+      </c>
+      <c r="F33" s="6" t="s">
         <v>642</v>
       </c>
-      <c r="D33" s="36" t="s">
-        <v>724</v>
-      </c>
-      <c r="E33" s="6" t="s">
+      <c r="G33" s="6" t="s">
         <v>643</v>
       </c>
-      <c r="F33" s="6" t="s">
+      <c r="H33" s="34" t="s">
         <v>644</v>
       </c>
-      <c r="G33" s="6" t="s">
+      <c r="I33" s="7" t="s">
         <v>645</v>
       </c>
-      <c r="H33" s="34" t="s">
-        <v>646</v>
-      </c>
-      <c r="I33" s="7" t="s">
-        <v>647</v>
-      </c>
       <c r="J33" s="6">
-        <v>68</v>
+        <f>SUM(L33+M33)</f>
+        <v>74</v>
       </c>
       <c r="K33" s="49" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="L33" s="6">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M33" s="6">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="N33" s="14"/>
     </row>
@@ -7859,40 +7879,40 @@
         <v>32</v>
       </c>
       <c r="B34" s="3" t="s">
+        <v>646</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>647</v>
+      </c>
+      <c r="D34" s="36" t="s">
+        <v>698</v>
+      </c>
+      <c r="E34" s="3" t="s">
         <v>648</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="F34" s="3" t="s">
         <v>649</v>
       </c>
-      <c r="D34" s="36" t="s">
-        <v>700</v>
-      </c>
-      <c r="E34" s="3" t="s">
+      <c r="G34" s="3" t="s">
         <v>650</v>
       </c>
-      <c r="F34" s="3" t="s">
+      <c r="H34" s="33" t="s">
         <v>651</v>
       </c>
-      <c r="G34" s="3" t="s">
+      <c r="I34" s="4" t="s">
         <v>652</v>
       </c>
-      <c r="H34" s="33" t="s">
+      <c r="J34" s="3" t="s">
         <v>653</v>
       </c>
-      <c r="I34" s="4" t="s">
+      <c r="K34" s="10" t="s">
         <v>654</v>
-      </c>
-      <c r="J34" s="3" t="s">
-        <v>655</v>
-      </c>
-      <c r="K34" s="10" t="s">
-        <v>656</v>
       </c>
       <c r="L34" s="3">
         <v>10</v>
       </c>
       <c r="M34" s="3" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="N34" s="3"/>
     </row>
@@ -7901,34 +7921,34 @@
         <v>33</v>
       </c>
       <c r="B35" s="6" t="s">
+        <v>656</v>
+      </c>
+      <c r="C35" s="37" t="s">
+        <v>657</v>
+      </c>
+      <c r="D35" s="36" t="s">
+        <v>722</v>
+      </c>
+      <c r="E35" s="6" t="s">
         <v>658</v>
       </c>
-      <c r="C35" s="37" t="s">
+      <c r="F35" s="6" t="s">
         <v>659</v>
       </c>
-      <c r="D35" s="36" t="s">
-        <v>724</v>
-      </c>
-      <c r="E35" s="6" t="s">
+      <c r="G35" s="6" t="s">
         <v>660</v>
       </c>
-      <c r="F35" s="6" t="s">
+      <c r="H35" s="34" t="s">
         <v>661</v>
       </c>
-      <c r="G35" s="6" t="s">
+      <c r="I35" s="7" t="s">
         <v>662</v>
-      </c>
-      <c r="H35" s="34" t="s">
-        <v>663</v>
-      </c>
-      <c r="I35" s="7" t="s">
-        <v>664</v>
       </c>
       <c r="J35" s="6">
         <v>14</v>
       </c>
       <c r="K35" s="49" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="L35" s="6">
         <v>14</v>
@@ -7943,32 +7963,32 @@
         <v>34</v>
       </c>
       <c r="B36" s="3" t="s">
+        <v>663</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D36" s="36" t="s">
+        <v>722</v>
+      </c>
+      <c r="E36" s="3" t="s">
         <v>665</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="F36" s="3" t="s">
         <v>666</v>
-      </c>
-      <c r="D36" s="36" t="s">
-        <v>724</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>667</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>668</v>
       </c>
       <c r="G36" s="3"/>
       <c r="H36" s="33" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="J36" s="3">
         <v>25</v>
       </c>
       <c r="K36" s="45" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="L36" s="3">
         <v>23</v>
@@ -7983,26 +8003,26 @@
         <v>35</v>
       </c>
       <c r="B37" s="89" t="s">
+        <v>669</v>
+      </c>
+      <c r="C37" s="90" t="s">
+        <v>670</v>
+      </c>
+      <c r="D37" s="91" t="s">
+        <v>722</v>
+      </c>
+      <c r="E37" s="89" t="s">
+        <v>719</v>
+      </c>
+      <c r="F37" s="6" t="s">
         <v>671</v>
-      </c>
-      <c r="C37" s="90" t="s">
-        <v>672</v>
-      </c>
-      <c r="D37" s="91" t="s">
-        <v>724</v>
-      </c>
-      <c r="E37" s="89" t="s">
-        <v>721</v>
-      </c>
-      <c r="F37" s="6" t="s">
-        <v>673</v>
       </c>
       <c r="G37" s="6"/>
       <c r="H37" s="34" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="I37" s="7" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="J37" s="6"/>
       <c r="K37" s="43"/>
@@ -8017,14 +8037,14 @@
       <c r="D38" s="91"/>
       <c r="E38" s="89"/>
       <c r="F38" s="6" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="G38" s="6"/>
       <c r="H38" s="34" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="I38" s="7" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="J38" s="6"/>
       <c r="K38" s="43"/>
@@ -8037,26 +8057,26 @@
         <v>36</v>
       </c>
       <c r="B39" s="3" t="s">
+        <v>677</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>678</v>
+      </c>
+      <c r="D39" s="36" t="s">
+        <v>722</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>715</v>
+      </c>
+      <c r="F39" s="3" t="s">
         <v>679</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>680</v>
-      </c>
-      <c r="D39" s="36" t="s">
-        <v>724</v>
-      </c>
-      <c r="E39" s="3" t="s">
-        <v>717</v>
-      </c>
-      <c r="F39" s="3" t="s">
-        <v>681</v>
       </c>
       <c r="G39" s="3"/>
       <c r="H39" s="33" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="J39" s="3"/>
       <c r="K39" s="10"/>
@@ -8069,32 +8089,32 @@
         <v>37</v>
       </c>
       <c r="B40" s="6" t="s">
+        <v>682</v>
+      </c>
+      <c r="C40" s="37" t="s">
+        <v>683</v>
+      </c>
+      <c r="D40" s="36" t="s">
+        <v>722</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>713</v>
+      </c>
+      <c r="F40" s="6" t="s">
         <v>684</v>
-      </c>
-      <c r="C40" s="37" t="s">
-        <v>685</v>
-      </c>
-      <c r="D40" s="36" t="s">
-        <v>724</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>715</v>
-      </c>
-      <c r="F40" s="6" t="s">
-        <v>686</v>
       </c>
       <c r="G40" s="6"/>
       <c r="H40" s="34" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="I40" s="7" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="J40" s="6">
         <v>60</v>
       </c>
       <c r="K40" s="49" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="L40" s="6">
         <v>60</v>
@@ -8107,26 +8127,26 @@
         <v>38</v>
       </c>
       <c r="B41" s="3" t="s">
+        <v>687</v>
+      </c>
+      <c r="C41" s="38" t="s">
+        <v>699</v>
+      </c>
+      <c r="D41" s="36" t="s">
+        <v>698</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>688</v>
+      </c>
+      <c r="F41" s="3" t="s">
         <v>689</v>
-      </c>
-      <c r="C41" s="38" t="s">
-        <v>701</v>
-      </c>
-      <c r="D41" s="36" t="s">
-        <v>700</v>
-      </c>
-      <c r="E41" s="3" t="s">
-        <v>690</v>
-      </c>
-      <c r="F41" s="3" t="s">
-        <v>691</v>
       </c>
       <c r="G41" s="3"/>
       <c r="H41" s="33" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="I41" s="4" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="J41" s="3"/>
       <c r="K41" s="10"/>
@@ -8139,26 +8159,26 @@
         <v>39</v>
       </c>
       <c r="B42" s="6" t="s">
+        <v>692</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="D42" s="36" t="s">
+        <v>722</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>716</v>
+      </c>
+      <c r="F42" s="6" t="s">
         <v>694</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>695</v>
-      </c>
-      <c r="D42" s="36" t="s">
-        <v>724</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>718</v>
-      </c>
-      <c r="F42" s="6" t="s">
-        <v>696</v>
       </c>
       <c r="G42" s="6"/>
       <c r="H42" s="34" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="I42" s="7" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="J42" s="6">
         <v>16</v>
@@ -8183,7 +8203,7 @@
       </c>
       <c r="C43" s="3"/>
       <c r="D43" s="35" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="E43" s="3" t="s">
         <v>300</v>
@@ -8203,16 +8223,12 @@
       <c r="N43" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="5">
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="B14:B15"/>
     <mergeCell ref="B37:B38"/>
-    <mergeCell ref="C14:C15"/>
     <mergeCell ref="C37:C38"/>
-    <mergeCell ref="E14:E15"/>
     <mergeCell ref="E37:E38"/>
     <mergeCell ref="D37:D38"/>
-    <mergeCell ref="D14:D15"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="I3" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
@@ -8283,37 +8299,37 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="15" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="15" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="15" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="15" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="15" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="15" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="15" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed donor visual bugs
</commit_message>
<xml_diff>
--- a/FoodBank Files/Food Bank recipients.xlsx
+++ b/FoodBank Files/Food Bank recipients.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\icarusjay\Downloads\xampp\htdocs\FoodBank Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C20F9425-96FB-4211-8011-E4FA1899A20A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{618136FB-3F3A-418A-8A8D-376CF29FCE3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13740" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="730">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="731">
   <si>
     <t>PHASE 4 - B UNIT 1 HVG ARCADE, SUBANGDAKO, MANDAUE CITY</t>
   </si>
@@ -2249,6 +2249,9 @@
   </si>
   <si>
     <t>Ilihan, Toledo City Cebu</t>
+  </si>
+  <si>
+    <t>Kids Life Foundation (BALAY AMOMA)</t>
   </si>
 </sst>
 </file>
@@ -2771,120 +2774,129 @@
     <xf numFmtId="49" fontId="18" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2896,15 +2908,6 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3500,9 +3503,9 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="32"/>
-      <c r="C4" s="50"/>
-      <c r="D4" s="50"/>
-      <c r="E4" s="50"/>
+      <c r="C4" s="53"/>
+      <c r="D4" s="53"/>
+      <c r="E4" s="53"/>
       <c r="L4" s="32"/>
     </row>
     <row r="5" spans="1:12">
@@ -3523,264 +3526,264 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" s="32"/>
-      <c r="B9" s="51" t="s">
+      <c r="B9" s="89" t="s">
         <v>0</v>
       </c>
-      <c r="C9" s="50"/>
-      <c r="D9" s="50"/>
-      <c r="E9" s="50"/>
-      <c r="F9" s="50"/>
-      <c r="G9" s="50"/>
-      <c r="H9" s="50"/>
-      <c r="I9" s="50"/>
-      <c r="J9" s="50"/>
-      <c r="K9" s="50"/>
+      <c r="C9" s="53"/>
+      <c r="D9" s="53"/>
+      <c r="E9" s="53"/>
+      <c r="F9" s="53"/>
+      <c r="G9" s="53"/>
+      <c r="H9" s="53"/>
+      <c r="I9" s="53"/>
+      <c r="J9" s="53"/>
+      <c r="K9" s="53"/>
       <c r="L9" s="32"/>
     </row>
     <row r="10" spans="1:12">
       <c r="A10" s="32"/>
-      <c r="B10" s="85" t="s">
+      <c r="B10" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="C10" s="85"/>
-      <c r="D10" s="85"/>
-      <c r="E10" s="85"/>
-      <c r="F10" s="85"/>
-      <c r="G10" s="85"/>
-      <c r="H10" s="85"/>
-      <c r="I10" s="85"/>
-      <c r="J10" s="85"/>
-      <c r="K10" s="85"/>
+      <c r="C10" s="54"/>
+      <c r="D10" s="54"/>
+      <c r="E10" s="54"/>
+      <c r="F10" s="54"/>
+      <c r="G10" s="54"/>
+      <c r="H10" s="54"/>
+      <c r="I10" s="54"/>
+      <c r="J10" s="54"/>
+      <c r="K10" s="54"/>
       <c r="L10" s="32"/>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" s="32"/>
-      <c r="B11" s="85"/>
-      <c r="C11" s="85"/>
-      <c r="D11" s="85"/>
-      <c r="E11" s="85"/>
-      <c r="F11" s="85"/>
-      <c r="G11" s="85"/>
-      <c r="H11" s="85"/>
-      <c r="I11" s="85"/>
-      <c r="J11" s="85"/>
-      <c r="K11" s="85"/>
+      <c r="B11" s="54"/>
+      <c r="C11" s="54"/>
+      <c r="D11" s="54"/>
+      <c r="E11" s="54"/>
+      <c r="F11" s="54"/>
+      <c r="G11" s="54"/>
+      <c r="H11" s="54"/>
+      <c r="I11" s="54"/>
+      <c r="J11" s="54"/>
+      <c r="K11" s="54"/>
       <c r="L11" s="32"/>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" s="32"/>
-      <c r="B12" s="52" t="s">
+      <c r="B12" s="90" t="s">
         <v>2</v>
       </c>
-      <c r="C12" s="52"/>
-      <c r="D12" s="52"/>
-      <c r="E12" s="52"/>
-      <c r="F12" s="52"/>
-      <c r="G12" s="52"/>
-      <c r="H12" s="52"/>
-      <c r="I12" s="52"/>
-      <c r="J12" s="52"/>
-      <c r="K12" s="52"/>
+      <c r="C12" s="90"/>
+      <c r="D12" s="90"/>
+      <c r="E12" s="90"/>
+      <c r="F12" s="90"/>
+      <c r="G12" s="90"/>
+      <c r="H12" s="90"/>
+      <c r="I12" s="90"/>
+      <c r="J12" s="90"/>
+      <c r="K12" s="90"/>
       <c r="L12" s="32"/>
     </row>
     <row r="13" spans="1:12">
       <c r="A13" s="32"/>
-      <c r="B13" s="53" t="s">
+      <c r="B13" s="84" t="s">
         <v>3</v>
       </c>
-      <c r="C13" s="54"/>
-      <c r="D13" s="55"/>
-      <c r="E13" s="53" t="s">
+      <c r="C13" s="85"/>
+      <c r="D13" s="86"/>
+      <c r="E13" s="84" t="s">
         <v>4</v>
       </c>
-      <c r="F13" s="54"/>
-      <c r="G13" s="55"/>
-      <c r="H13" s="53" t="s">
+      <c r="F13" s="85"/>
+      <c r="G13" s="86"/>
+      <c r="H13" s="84" t="s">
         <v>5</v>
       </c>
-      <c r="I13" s="54"/>
-      <c r="J13" s="54"/>
-      <c r="K13" s="55"/>
+      <c r="I13" s="85"/>
+      <c r="J13" s="85"/>
+      <c r="K13" s="86"/>
       <c r="L13" s="32"/>
     </row>
     <row r="14" spans="1:12">
       <c r="A14" s="32"/>
-      <c r="B14" s="56" t="s">
+      <c r="B14" s="68" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="57"/>
-      <c r="D14" s="58"/>
-      <c r="E14" s="56" t="s">
+      <c r="C14" s="69"/>
+      <c r="D14" s="70"/>
+      <c r="E14" s="68" t="s">
         <v>7</v>
       </c>
-      <c r="F14" s="57"/>
-      <c r="G14" s="58"/>
-      <c r="H14" s="59" t="s">
+      <c r="F14" s="69"/>
+      <c r="G14" s="70"/>
+      <c r="H14" s="71" t="s">
         <v>8</v>
       </c>
-      <c r="I14" s="60"/>
-      <c r="J14" s="60"/>
-      <c r="K14" s="61"/>
+      <c r="I14" s="72"/>
+      <c r="J14" s="72"/>
+      <c r="K14" s="73"/>
       <c r="L14" s="32"/>
     </row>
     <row r="15" spans="1:12">
       <c r="A15" s="32"/>
-      <c r="B15" s="62" t="s">
+      <c r="B15" s="65" t="s">
         <v>9</v>
       </c>
-      <c r="C15" s="63"/>
-      <c r="D15" s="64"/>
-      <c r="E15" s="62" t="s">
+      <c r="C15" s="83"/>
+      <c r="D15" s="66"/>
+      <c r="E15" s="65" t="s">
         <v>10</v>
       </c>
-      <c r="F15" s="63"/>
-      <c r="G15" s="64"/>
-      <c r="H15" s="65" t="s">
+      <c r="F15" s="83"/>
+      <c r="G15" s="66"/>
+      <c r="H15" s="80" t="s">
         <v>11</v>
       </c>
-      <c r="I15" s="66"/>
-      <c r="J15" s="66"/>
-      <c r="K15" s="67"/>
+      <c r="I15" s="81"/>
+      <c r="J15" s="81"/>
+      <c r="K15" s="82"/>
       <c r="L15" s="32"/>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" s="32"/>
-      <c r="B16" s="56" t="s">
+      <c r="B16" s="68" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="57"/>
-      <c r="D16" s="58"/>
-      <c r="E16" s="56" t="s">
+      <c r="C16" s="69"/>
+      <c r="D16" s="70"/>
+      <c r="E16" s="68" t="s">
         <v>13</v>
       </c>
-      <c r="F16" s="57"/>
-      <c r="G16" s="58"/>
-      <c r="H16" s="59" t="s">
+      <c r="F16" s="69"/>
+      <c r="G16" s="70"/>
+      <c r="H16" s="71" t="s">
         <v>14</v>
       </c>
-      <c r="I16" s="60"/>
-      <c r="J16" s="60"/>
-      <c r="K16" s="61"/>
+      <c r="I16" s="72"/>
+      <c r="J16" s="72"/>
+      <c r="K16" s="73"/>
       <c r="L16" s="32"/>
     </row>
     <row r="17" spans="1:16">
       <c r="A17" s="32"/>
-      <c r="B17" s="62" t="s">
+      <c r="B17" s="65" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="63"/>
-      <c r="D17" s="64"/>
-      <c r="E17" s="62" t="s">
+      <c r="C17" s="83"/>
+      <c r="D17" s="66"/>
+      <c r="E17" s="65" t="s">
         <v>16</v>
       </c>
-      <c r="F17" s="63"/>
-      <c r="G17" s="64"/>
-      <c r="H17" s="65" t="s">
+      <c r="F17" s="83"/>
+      <c r="G17" s="66"/>
+      <c r="H17" s="80" t="s">
         <v>17</v>
       </c>
-      <c r="I17" s="66"/>
-      <c r="J17" s="66"/>
-      <c r="K17" s="67"/>
+      <c r="I17" s="81"/>
+      <c r="J17" s="81"/>
+      <c r="K17" s="82"/>
       <c r="L17" s="32"/>
     </row>
     <row r="18" spans="1:16">
       <c r="A18" s="32"/>
-      <c r="B18" s="56" t="s">
+      <c r="B18" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="57"/>
-      <c r="D18" s="58"/>
-      <c r="E18" s="56" t="s">
+      <c r="C18" s="69"/>
+      <c r="D18" s="70"/>
+      <c r="E18" s="68" t="s">
         <v>19</v>
       </c>
-      <c r="F18" s="57"/>
-      <c r="G18" s="58"/>
-      <c r="H18" s="59" t="s">
+      <c r="F18" s="69"/>
+      <c r="G18" s="70"/>
+      <c r="H18" s="71" t="s">
         <v>20</v>
       </c>
-      <c r="I18" s="60"/>
-      <c r="J18" s="60"/>
-      <c r="K18" s="61"/>
+      <c r="I18" s="72"/>
+      <c r="J18" s="72"/>
+      <c r="K18" s="73"/>
       <c r="L18" s="32"/>
     </row>
     <row r="19" spans="1:16">
       <c r="A19" s="32"/>
-      <c r="B19" s="62" t="s">
+      <c r="B19" s="65" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="63"/>
-      <c r="D19" s="64"/>
-      <c r="E19" s="62" t="s">
+      <c r="C19" s="83"/>
+      <c r="D19" s="66"/>
+      <c r="E19" s="65" t="s">
         <v>22</v>
       </c>
-      <c r="F19" s="63"/>
-      <c r="G19" s="64"/>
-      <c r="H19" s="65" t="s">
+      <c r="F19" s="83"/>
+      <c r="G19" s="66"/>
+      <c r="H19" s="80" t="s">
         <v>23</v>
       </c>
-      <c r="I19" s="66"/>
-      <c r="J19" s="66"/>
-      <c r="K19" s="67"/>
+      <c r="I19" s="81"/>
+      <c r="J19" s="81"/>
+      <c r="K19" s="82"/>
       <c r="L19" s="32"/>
     </row>
     <row r="20" spans="1:16">
       <c r="A20" s="32"/>
-      <c r="B20" s="56" t="s">
+      <c r="B20" s="68" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="57"/>
-      <c r="D20" s="58"/>
-      <c r="E20" s="56" t="s">
+      <c r="C20" s="69"/>
+      <c r="D20" s="70"/>
+      <c r="E20" s="68" t="s">
         <v>25</v>
       </c>
-      <c r="F20" s="57"/>
-      <c r="G20" s="58"/>
-      <c r="H20" s="59" t="s">
+      <c r="F20" s="69"/>
+      <c r="G20" s="70"/>
+      <c r="H20" s="71" t="s">
         <v>26</v>
       </c>
-      <c r="I20" s="60"/>
-      <c r="J20" s="60"/>
-      <c r="K20" s="61"/>
+      <c r="I20" s="72"/>
+      <c r="J20" s="72"/>
+      <c r="K20" s="73"/>
       <c r="L20" s="32"/>
     </row>
     <row r="21" spans="1:16">
       <c r="A21" s="32"/>
-      <c r="B21" s="62" t="s">
+      <c r="B21" s="65" t="s">
         <v>27</v>
       </c>
-      <c r="C21" s="63"/>
-      <c r="D21" s="64"/>
-      <c r="E21" s="62" t="s">
+      <c r="C21" s="83"/>
+      <c r="D21" s="66"/>
+      <c r="E21" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="F21" s="63"/>
-      <c r="G21" s="64"/>
-      <c r="H21" s="65" t="s">
+      <c r="F21" s="83"/>
+      <c r="G21" s="66"/>
+      <c r="H21" s="80" t="s">
         <v>29</v>
       </c>
-      <c r="I21" s="66"/>
-      <c r="J21" s="66"/>
-      <c r="K21" s="67"/>
+      <c r="I21" s="81"/>
+      <c r="J21" s="81"/>
+      <c r="K21" s="82"/>
       <c r="L21" s="32"/>
     </row>
     <row r="22" spans="1:16">
       <c r="A22" s="32"/>
-      <c r="B22" s="56" t="s">
+      <c r="B22" s="68" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="57"/>
-      <c r="D22" s="58"/>
-      <c r="E22" s="56" t="s">
+      <c r="C22" s="69"/>
+      <c r="D22" s="70"/>
+      <c r="E22" s="68" t="s">
         <v>31</v>
       </c>
-      <c r="F22" s="57"/>
-      <c r="G22" s="58"/>
-      <c r="H22" s="59" t="s">
+      <c r="F22" s="69"/>
+      <c r="G22" s="70"/>
+      <c r="H22" s="71" t="s">
         <v>32</v>
       </c>
-      <c r="I22" s="60"/>
-      <c r="J22" s="60"/>
-      <c r="K22" s="61"/>
+      <c r="I22" s="72"/>
+      <c r="J22" s="72"/>
+      <c r="K22" s="73"/>
       <c r="L22" s="32"/>
     </row>
     <row r="23" spans="1:16">
@@ -3803,18 +3806,18 @@
     </row>
     <row r="24" spans="1:16">
       <c r="A24" s="32"/>
-      <c r="B24" s="68" t="s">
+      <c r="B24" s="67" t="s">
         <v>33</v>
       </c>
-      <c r="C24" s="68"/>
-      <c r="D24" s="68"/>
-      <c r="E24" s="68"/>
-      <c r="F24" s="68"/>
-      <c r="G24" s="68"/>
-      <c r="H24" s="68"/>
-      <c r="I24" s="68"/>
-      <c r="J24" s="68"/>
-      <c r="K24" s="68"/>
+      <c r="C24" s="67"/>
+      <c r="D24" s="67"/>
+      <c r="E24" s="67"/>
+      <c r="F24" s="67"/>
+      <c r="G24" s="67"/>
+      <c r="H24" s="67"/>
+      <c r="I24" s="67"/>
+      <c r="J24" s="67"/>
+      <c r="K24" s="67"/>
       <c r="L24" s="32"/>
       <c r="M24" s="32"/>
       <c r="N24" s="32"/>
@@ -3823,578 +3826,578 @@
     </row>
     <row r="25" spans="1:16">
       <c r="A25" s="32"/>
-      <c r="B25" s="53" t="s">
+      <c r="B25" s="84" t="s">
         <v>34</v>
       </c>
-      <c r="C25" s="54"/>
-      <c r="D25" s="54"/>
-      <c r="E25" s="54"/>
-      <c r="F25" s="55"/>
-      <c r="G25" s="53" t="s">
+      <c r="C25" s="85"/>
+      <c r="D25" s="85"/>
+      <c r="E25" s="85"/>
+      <c r="F25" s="86"/>
+      <c r="G25" s="84" t="s">
         <v>5</v>
       </c>
-      <c r="H25" s="69"/>
-      <c r="I25" s="69"/>
-      <c r="J25" s="69"/>
-      <c r="K25" s="70"/>
-      <c r="L25" s="62"/>
-      <c r="M25" s="64"/>
+      <c r="H25" s="87"/>
+      <c r="I25" s="87"/>
+      <c r="J25" s="87"/>
+      <c r="K25" s="88"/>
+      <c r="L25" s="65"/>
+      <c r="M25" s="66"/>
       <c r="N25" s="32"/>
       <c r="O25"/>
       <c r="P25"/>
     </row>
     <row r="26" spans="1:16">
       <c r="A26" s="32"/>
-      <c r="B26" s="71" t="s">
+      <c r="B26" s="57" t="s">
         <v>35</v>
       </c>
-      <c r="C26" s="71"/>
-      <c r="D26" s="71"/>
-      <c r="E26" s="71"/>
-      <c r="F26" s="71"/>
-      <c r="G26" s="72" t="s">
+      <c r="C26" s="57"/>
+      <c r="D26" s="57"/>
+      <c r="E26" s="57"/>
+      <c r="F26" s="57"/>
+      <c r="G26" s="58" t="s">
         <v>36</v>
       </c>
-      <c r="H26" s="72"/>
-      <c r="I26" s="72"/>
-      <c r="J26" s="72"/>
-      <c r="K26" s="72"/>
-      <c r="L26" s="62"/>
-      <c r="M26" s="64"/>
+      <c r="H26" s="58"/>
+      <c r="I26" s="58"/>
+      <c r="J26" s="58"/>
+      <c r="K26" s="58"/>
+      <c r="L26" s="65"/>
+      <c r="M26" s="66"/>
       <c r="N26" s="32"/>
       <c r="O26"/>
       <c r="P26"/>
     </row>
     <row r="27" spans="1:16">
       <c r="A27" s="32"/>
-      <c r="B27" s="73" t="s">
+      <c r="B27" s="55" t="s">
         <v>37</v>
       </c>
-      <c r="C27" s="73"/>
-      <c r="D27" s="73"/>
-      <c r="E27" s="73"/>
-      <c r="F27" s="73"/>
-      <c r="G27" s="74" t="s">
+      <c r="C27" s="55"/>
+      <c r="D27" s="55"/>
+      <c r="E27" s="55"/>
+      <c r="F27" s="55"/>
+      <c r="G27" s="56" t="s">
         <v>38</v>
       </c>
-      <c r="H27" s="74"/>
-      <c r="I27" s="74"/>
-      <c r="J27" s="74"/>
-      <c r="K27" s="74"/>
-      <c r="L27" s="75" t="s">
+      <c r="H27" s="56"/>
+      <c r="I27" s="56"/>
+      <c r="J27" s="56"/>
+      <c r="K27" s="56"/>
+      <c r="L27" s="78" t="s">
         <v>39</v>
       </c>
-      <c r="M27" s="76"/>
+      <c r="M27" s="79"/>
       <c r="N27" s="32"/>
       <c r="O27"/>
       <c r="P27"/>
     </row>
     <row r="28" spans="1:16">
       <c r="A28" s="32"/>
-      <c r="B28" s="71" t="s">
+      <c r="B28" s="57" t="s">
         <v>40</v>
       </c>
-      <c r="C28" s="71"/>
-      <c r="D28" s="71"/>
-      <c r="E28" s="71"/>
-      <c r="F28" s="71"/>
-      <c r="G28" s="72" t="s">
+      <c r="C28" s="57"/>
+      <c r="D28" s="57"/>
+      <c r="E28" s="57"/>
+      <c r="F28" s="57"/>
+      <c r="G28" s="58" t="s">
         <v>41</v>
       </c>
-      <c r="H28" s="72"/>
-      <c r="I28" s="72"/>
-      <c r="J28" s="72"/>
-      <c r="K28" s="72"/>
-      <c r="L28" s="62"/>
-      <c r="M28" s="64"/>
+      <c r="H28" s="58"/>
+      <c r="I28" s="58"/>
+      <c r="J28" s="58"/>
+      <c r="K28" s="58"/>
+      <c r="L28" s="65"/>
+      <c r="M28" s="66"/>
       <c r="N28" s="32"/>
       <c r="O28"/>
       <c r="P28"/>
     </row>
     <row r="29" spans="1:16">
       <c r="A29" s="32"/>
-      <c r="B29" s="73" t="s">
+      <c r="B29" s="55" t="s">
         <v>42</v>
       </c>
-      <c r="C29" s="73"/>
-      <c r="D29" s="73"/>
-      <c r="E29" s="73"/>
-      <c r="F29" s="73"/>
-      <c r="G29" s="74" t="s">
+      <c r="C29" s="55"/>
+      <c r="D29" s="55"/>
+      <c r="E29" s="55"/>
+      <c r="F29" s="55"/>
+      <c r="G29" s="56" t="s">
         <v>43</v>
       </c>
-      <c r="H29" s="74"/>
-      <c r="I29" s="74"/>
-      <c r="J29" s="74"/>
-      <c r="K29" s="74"/>
-      <c r="L29" s="62"/>
-      <c r="M29" s="64"/>
+      <c r="H29" s="56"/>
+      <c r="I29" s="56"/>
+      <c r="J29" s="56"/>
+      <c r="K29" s="56"/>
+      <c r="L29" s="65"/>
+      <c r="M29" s="66"/>
       <c r="N29" s="32"/>
       <c r="O29"/>
       <c r="P29"/>
     </row>
     <row r="30" spans="1:16">
       <c r="A30" s="32"/>
-      <c r="B30" s="71" t="s">
+      <c r="B30" s="57" t="s">
         <v>44</v>
       </c>
-      <c r="C30" s="71"/>
-      <c r="D30" s="71"/>
-      <c r="E30" s="71"/>
-      <c r="F30" s="71"/>
-      <c r="G30" s="72" t="s">
+      <c r="C30" s="57"/>
+      <c r="D30" s="57"/>
+      <c r="E30" s="57"/>
+      <c r="F30" s="57"/>
+      <c r="G30" s="58" t="s">
         <v>45</v>
       </c>
-      <c r="H30" s="72"/>
-      <c r="I30" s="72"/>
-      <c r="J30" s="72"/>
-      <c r="K30" s="72"/>
-      <c r="L30" s="75" t="s">
+      <c r="H30" s="58"/>
+      <c r="I30" s="58"/>
+      <c r="J30" s="58"/>
+      <c r="K30" s="58"/>
+      <c r="L30" s="78" t="s">
         <v>46</v>
       </c>
-      <c r="M30" s="76"/>
+      <c r="M30" s="79"/>
       <c r="N30" s="32"/>
       <c r="O30"/>
       <c r="P30"/>
     </row>
     <row r="31" spans="1:16">
       <c r="A31" s="32"/>
-      <c r="B31" s="73" t="s">
+      <c r="B31" s="55" t="s">
         <v>47</v>
       </c>
-      <c r="C31" s="73"/>
-      <c r="D31" s="73"/>
-      <c r="E31" s="73"/>
-      <c r="F31" s="73"/>
-      <c r="G31" s="65" t="s">
+      <c r="C31" s="55"/>
+      <c r="D31" s="55"/>
+      <c r="E31" s="55"/>
+      <c r="F31" s="55"/>
+      <c r="G31" s="80" t="s">
         <v>48</v>
       </c>
-      <c r="H31" s="66"/>
-      <c r="I31" s="66"/>
-      <c r="J31" s="66"/>
-      <c r="K31" s="67"/>
-      <c r="L31" s="62"/>
-      <c r="M31" s="64"/>
+      <c r="H31" s="81"/>
+      <c r="I31" s="81"/>
+      <c r="J31" s="81"/>
+      <c r="K31" s="82"/>
+      <c r="L31" s="65"/>
+      <c r="M31" s="66"/>
       <c r="N31" s="32"/>
       <c r="O31"/>
       <c r="P31"/>
     </row>
     <row r="32" spans="1:16">
       <c r="A32" s="32"/>
-      <c r="B32" s="71" t="s">
+      <c r="B32" s="57" t="s">
         <v>49</v>
       </c>
-      <c r="C32" s="71"/>
-      <c r="D32" s="71"/>
-      <c r="E32" s="71"/>
-      <c r="F32" s="71"/>
-      <c r="G32" s="72" t="s">
+      <c r="C32" s="57"/>
+      <c r="D32" s="57"/>
+      <c r="E32" s="57"/>
+      <c r="F32" s="57"/>
+      <c r="G32" s="58" t="s">
         <v>50</v>
       </c>
-      <c r="H32" s="72"/>
-      <c r="I32" s="72"/>
-      <c r="J32" s="72"/>
-      <c r="K32" s="72"/>
-      <c r="L32" s="75" t="s">
+      <c r="H32" s="58"/>
+      <c r="I32" s="58"/>
+      <c r="J32" s="58"/>
+      <c r="K32" s="58"/>
+      <c r="L32" s="78" t="s">
         <v>51</v>
       </c>
-      <c r="M32" s="76"/>
+      <c r="M32" s="79"/>
       <c r="N32" s="32"/>
       <c r="O32"/>
       <c r="P32"/>
     </row>
     <row r="33" spans="1:16">
       <c r="A33" s="32"/>
-      <c r="B33" s="73" t="s">
+      <c r="B33" s="55" t="s">
         <v>52</v>
       </c>
-      <c r="C33" s="73"/>
-      <c r="D33" s="73"/>
-      <c r="E33" s="73"/>
-      <c r="F33" s="73"/>
-      <c r="G33" s="65" t="s">
+      <c r="C33" s="55"/>
+      <c r="D33" s="55"/>
+      <c r="E33" s="55"/>
+      <c r="F33" s="55"/>
+      <c r="G33" s="80" t="s">
         <v>48</v>
       </c>
-      <c r="H33" s="66"/>
-      <c r="I33" s="66"/>
-      <c r="J33" s="66"/>
-      <c r="K33" s="67"/>
-      <c r="L33" s="62"/>
-      <c r="M33" s="64"/>
+      <c r="H33" s="81"/>
+      <c r="I33" s="81"/>
+      <c r="J33" s="81"/>
+      <c r="K33" s="82"/>
+      <c r="L33" s="65"/>
+      <c r="M33" s="66"/>
       <c r="N33" s="32"/>
       <c r="O33"/>
       <c r="P33"/>
     </row>
     <row r="34" spans="1:16">
       <c r="A34" s="32"/>
-      <c r="B34" s="71" t="s">
+      <c r="B34" s="57" t="s">
         <v>53</v>
       </c>
-      <c r="C34" s="71"/>
-      <c r="D34" s="71"/>
-      <c r="E34" s="71"/>
-      <c r="F34" s="71"/>
-      <c r="G34" s="72" t="s">
+      <c r="C34" s="57"/>
+      <c r="D34" s="57"/>
+      <c r="E34" s="57"/>
+      <c r="F34" s="57"/>
+      <c r="G34" s="58" t="s">
         <v>54</v>
       </c>
-      <c r="H34" s="72"/>
-      <c r="I34" s="72"/>
-      <c r="J34" s="72"/>
-      <c r="K34" s="72"/>
-      <c r="L34" s="75" t="s">
+      <c r="H34" s="58"/>
+      <c r="I34" s="58"/>
+      <c r="J34" s="58"/>
+      <c r="K34" s="58"/>
+      <c r="L34" s="78" t="s">
         <v>55</v>
       </c>
-      <c r="M34" s="76"/>
+      <c r="M34" s="79"/>
       <c r="N34" s="32"/>
       <c r="O34"/>
       <c r="P34"/>
     </row>
     <row r="35" spans="1:16">
       <c r="A35" s="32"/>
-      <c r="B35" s="73" t="s">
+      <c r="B35" s="55" t="s">
         <v>56</v>
       </c>
-      <c r="C35" s="73"/>
-      <c r="D35" s="73"/>
-      <c r="E35" s="73"/>
-      <c r="F35" s="73"/>
-      <c r="G35" s="74" t="s">
+      <c r="C35" s="55"/>
+      <c r="D35" s="55"/>
+      <c r="E35" s="55"/>
+      <c r="F35" s="55"/>
+      <c r="G35" s="56" t="s">
         <v>57</v>
       </c>
-      <c r="H35" s="74"/>
-      <c r="I35" s="74"/>
-      <c r="J35" s="74"/>
-      <c r="K35" s="74"/>
-      <c r="L35" s="62"/>
-      <c r="M35" s="64"/>
+      <c r="H35" s="56"/>
+      <c r="I35" s="56"/>
+      <c r="J35" s="56"/>
+      <c r="K35" s="56"/>
+      <c r="L35" s="65"/>
+      <c r="M35" s="66"/>
       <c r="N35" s="32"/>
       <c r="O35"/>
       <c r="P35"/>
     </row>
     <row r="36" spans="1:16">
       <c r="A36" s="32"/>
-      <c r="B36" s="71" t="s">
+      <c r="B36" s="57" t="s">
         <v>58</v>
       </c>
-      <c r="C36" s="71"/>
-      <c r="D36" s="71"/>
-      <c r="E36" s="71"/>
-      <c r="F36" s="71"/>
-      <c r="G36" s="72" t="s">
+      <c r="C36" s="57"/>
+      <c r="D36" s="57"/>
+      <c r="E36" s="57"/>
+      <c r="F36" s="57"/>
+      <c r="G36" s="58" t="s">
         <v>59</v>
       </c>
-      <c r="H36" s="72"/>
-      <c r="I36" s="72"/>
-      <c r="J36" s="72"/>
-      <c r="K36" s="72"/>
-      <c r="L36" s="77"/>
-      <c r="M36" s="78"/>
+      <c r="H36" s="58"/>
+      <c r="I36" s="58"/>
+      <c r="J36" s="58"/>
+      <c r="K36" s="58"/>
+      <c r="L36" s="76"/>
+      <c r="M36" s="77"/>
       <c r="N36" s="32"/>
       <c r="O36"/>
       <c r="P36"/>
     </row>
     <row r="37" spans="1:16">
       <c r="A37" s="32"/>
-      <c r="B37" s="73" t="s">
+      <c r="B37" s="55" t="s">
         <v>60</v>
       </c>
-      <c r="C37" s="73"/>
-      <c r="D37" s="73"/>
-      <c r="E37" s="73"/>
-      <c r="F37" s="73"/>
-      <c r="G37" s="74" t="s">
+      <c r="C37" s="55"/>
+      <c r="D37" s="55"/>
+      <c r="E37" s="55"/>
+      <c r="F37" s="55"/>
+      <c r="G37" s="56" t="s">
         <v>61</v>
       </c>
-      <c r="H37" s="74"/>
-      <c r="I37" s="74"/>
-      <c r="J37" s="74"/>
-      <c r="K37" s="74"/>
-      <c r="L37" s="77"/>
-      <c r="M37" s="78"/>
+      <c r="H37" s="56"/>
+      <c r="I37" s="56"/>
+      <c r="J37" s="56"/>
+      <c r="K37" s="56"/>
+      <c r="L37" s="76"/>
+      <c r="M37" s="77"/>
       <c r="N37" s="32"/>
       <c r="O37"/>
       <c r="P37"/>
     </row>
     <row r="38" spans="1:16">
       <c r="A38" s="32"/>
-      <c r="B38" s="71" t="s">
+      <c r="B38" s="57" t="s">
         <v>62</v>
       </c>
-      <c r="C38" s="71"/>
-      <c r="D38" s="71"/>
-      <c r="E38" s="71"/>
-      <c r="F38" s="71"/>
-      <c r="G38" s="72" t="s">
+      <c r="C38" s="57"/>
+      <c r="D38" s="57"/>
+      <c r="E38" s="57"/>
+      <c r="F38" s="57"/>
+      <c r="G38" s="58" t="s">
         <v>63</v>
       </c>
-      <c r="H38" s="72"/>
-      <c r="I38" s="72"/>
-      <c r="J38" s="72"/>
-      <c r="K38" s="72"/>
-      <c r="L38" s="62"/>
-      <c r="M38" s="64"/>
+      <c r="H38" s="58"/>
+      <c r="I38" s="58"/>
+      <c r="J38" s="58"/>
+      <c r="K38" s="58"/>
+      <c r="L38" s="65"/>
+      <c r="M38" s="66"/>
       <c r="N38" s="32"/>
       <c r="O38"/>
       <c r="P38"/>
     </row>
     <row r="39" spans="1:16">
       <c r="A39" s="32"/>
-      <c r="B39" s="73" t="s">
+      <c r="B39" s="55" t="s">
         <v>64</v>
       </c>
-      <c r="C39" s="73"/>
-      <c r="D39" s="73"/>
-      <c r="E39" s="73"/>
-      <c r="F39" s="73"/>
-      <c r="G39" s="74" t="s">
+      <c r="C39" s="55"/>
+      <c r="D39" s="55"/>
+      <c r="E39" s="55"/>
+      <c r="F39" s="55"/>
+      <c r="G39" s="56" t="s">
         <v>65</v>
       </c>
-      <c r="H39" s="74"/>
-      <c r="I39" s="74"/>
-      <c r="J39" s="74"/>
-      <c r="K39" s="74"/>
-      <c r="L39" s="62"/>
-      <c r="M39" s="64"/>
+      <c r="H39" s="56"/>
+      <c r="I39" s="56"/>
+      <c r="J39" s="56"/>
+      <c r="K39" s="56"/>
+      <c r="L39" s="65"/>
+      <c r="M39" s="66"/>
       <c r="N39" s="32"/>
       <c r="O39"/>
       <c r="P39"/>
     </row>
     <row r="40" spans="1:16">
       <c r="A40" s="32"/>
-      <c r="B40" s="71" t="s">
+      <c r="B40" s="57" t="s">
         <v>66</v>
       </c>
-      <c r="C40" s="71"/>
-      <c r="D40" s="71"/>
-      <c r="E40" s="71"/>
-      <c r="F40" s="71"/>
-      <c r="G40" s="72" t="s">
+      <c r="C40" s="57"/>
+      <c r="D40" s="57"/>
+      <c r="E40" s="57"/>
+      <c r="F40" s="57"/>
+      <c r="G40" s="58" t="s">
         <v>67</v>
       </c>
-      <c r="H40" s="72"/>
-      <c r="I40" s="72"/>
-      <c r="J40" s="72"/>
-      <c r="K40" s="72"/>
-      <c r="L40" s="77"/>
-      <c r="M40" s="78"/>
+      <c r="H40" s="58"/>
+      <c r="I40" s="58"/>
+      <c r="J40" s="58"/>
+      <c r="K40" s="58"/>
+      <c r="L40" s="76"/>
+      <c r="M40" s="77"/>
       <c r="N40" s="32"/>
       <c r="O40"/>
       <c r="P40"/>
     </row>
     <row r="41" spans="1:16">
       <c r="A41" s="32"/>
-      <c r="B41" s="73" t="s">
+      <c r="B41" s="55" t="s">
         <v>68</v>
       </c>
-      <c r="C41" s="73"/>
-      <c r="D41" s="73"/>
-      <c r="E41" s="73"/>
-      <c r="F41" s="73"/>
-      <c r="G41" s="74" t="s">
+      <c r="C41" s="55"/>
+      <c r="D41" s="55"/>
+      <c r="E41" s="55"/>
+      <c r="F41" s="55"/>
+      <c r="G41" s="56" t="s">
         <v>69</v>
       </c>
-      <c r="H41" s="74"/>
-      <c r="I41" s="74"/>
-      <c r="J41" s="74"/>
-      <c r="K41" s="74"/>
-      <c r="L41" s="77"/>
-      <c r="M41" s="78"/>
+      <c r="H41" s="56"/>
+      <c r="I41" s="56"/>
+      <c r="J41" s="56"/>
+      <c r="K41" s="56"/>
+      <c r="L41" s="76"/>
+      <c r="M41" s="77"/>
       <c r="N41" s="32"/>
       <c r="O41"/>
       <c r="P41"/>
     </row>
     <row r="42" spans="1:16">
       <c r="A42" s="32"/>
-      <c r="B42" s="71" t="s">
+      <c r="B42" s="57" t="s">
         <v>70</v>
       </c>
-      <c r="C42" s="71"/>
-      <c r="D42" s="71"/>
-      <c r="E42" s="71"/>
-      <c r="F42" s="71"/>
-      <c r="G42" s="72" t="s">
+      <c r="C42" s="57"/>
+      <c r="D42" s="57"/>
+      <c r="E42" s="57"/>
+      <c r="F42" s="57"/>
+      <c r="G42" s="58" t="s">
         <v>71</v>
       </c>
-      <c r="H42" s="72"/>
-      <c r="I42" s="72"/>
-      <c r="J42" s="72"/>
-      <c r="K42" s="72"/>
-      <c r="L42" s="62"/>
-      <c r="M42" s="64"/>
+      <c r="H42" s="58"/>
+      <c r="I42" s="58"/>
+      <c r="J42" s="58"/>
+      <c r="K42" s="58"/>
+      <c r="L42" s="65"/>
+      <c r="M42" s="66"/>
       <c r="N42" s="32"/>
       <c r="O42"/>
       <c r="P42"/>
     </row>
     <row r="43" spans="1:16">
       <c r="A43" s="32"/>
-      <c r="B43" s="73" t="s">
+      <c r="B43" s="55" t="s">
         <v>72</v>
       </c>
-      <c r="C43" s="73"/>
-      <c r="D43" s="73"/>
-      <c r="E43" s="73"/>
-      <c r="F43" s="73"/>
-      <c r="G43" s="74" t="s">
+      <c r="C43" s="55"/>
+      <c r="D43" s="55"/>
+      <c r="E43" s="55"/>
+      <c r="F43" s="55"/>
+      <c r="G43" s="56" t="s">
         <v>73</v>
       </c>
-      <c r="H43" s="74"/>
-      <c r="I43" s="74"/>
-      <c r="J43" s="74"/>
-      <c r="K43" s="74"/>
-      <c r="L43" s="62"/>
-      <c r="M43" s="64"/>
+      <c r="H43" s="56"/>
+      <c r="I43" s="56"/>
+      <c r="J43" s="56"/>
+      <c r="K43" s="56"/>
+      <c r="L43" s="65"/>
+      <c r="M43" s="66"/>
       <c r="N43" s="32"/>
       <c r="O43"/>
       <c r="P43"/>
     </row>
     <row r="44" spans="1:16">
       <c r="A44" s="32"/>
-      <c r="B44" s="71" t="s">
+      <c r="B44" s="57" t="s">
         <v>74</v>
       </c>
-      <c r="C44" s="71"/>
-      <c r="D44" s="71"/>
-      <c r="E44" s="71"/>
-      <c r="F44" s="71"/>
-      <c r="G44" s="72" t="s">
+      <c r="C44" s="57"/>
+      <c r="D44" s="57"/>
+      <c r="E44" s="57"/>
+      <c r="F44" s="57"/>
+      <c r="G44" s="58" t="s">
         <v>75</v>
       </c>
-      <c r="H44" s="72"/>
-      <c r="I44" s="72"/>
-      <c r="J44" s="72"/>
-      <c r="K44" s="72"/>
-      <c r="L44" s="62"/>
-      <c r="M44" s="64"/>
+      <c r="H44" s="58"/>
+      <c r="I44" s="58"/>
+      <c r="J44" s="58"/>
+      <c r="K44" s="58"/>
+      <c r="L44" s="65"/>
+      <c r="M44" s="66"/>
       <c r="N44" s="32"/>
       <c r="O44"/>
       <c r="P44"/>
     </row>
     <row r="45" spans="1:16">
       <c r="A45" s="32"/>
-      <c r="B45" s="73" t="s">
+      <c r="B45" s="55" t="s">
         <v>76</v>
       </c>
-      <c r="C45" s="73"/>
-      <c r="D45" s="73"/>
-      <c r="E45" s="73"/>
-      <c r="F45" s="73"/>
-      <c r="G45" s="74" t="s">
+      <c r="C45" s="55"/>
+      <c r="D45" s="55"/>
+      <c r="E45" s="55"/>
+      <c r="F45" s="55"/>
+      <c r="G45" s="56" t="s">
         <v>77</v>
       </c>
-      <c r="H45" s="74"/>
-      <c r="I45" s="74"/>
-      <c r="J45" s="74"/>
-      <c r="K45" s="74"/>
-      <c r="L45" s="77"/>
-      <c r="M45" s="78"/>
+      <c r="H45" s="56"/>
+      <c r="I45" s="56"/>
+      <c r="J45" s="56"/>
+      <c r="K45" s="56"/>
+      <c r="L45" s="76"/>
+      <c r="M45" s="77"/>
       <c r="N45" s="32"/>
       <c r="O45"/>
       <c r="P45"/>
     </row>
     <row r="46" spans="1:16">
       <c r="A46" s="32"/>
-      <c r="B46" s="71" t="s">
+      <c r="B46" s="57" t="s">
         <v>78</v>
       </c>
-      <c r="C46" s="71"/>
-      <c r="D46" s="71"/>
-      <c r="E46" s="71"/>
-      <c r="F46" s="71"/>
-      <c r="G46" s="72" t="s">
+      <c r="C46" s="57"/>
+      <c r="D46" s="57"/>
+      <c r="E46" s="57"/>
+      <c r="F46" s="57"/>
+      <c r="G46" s="58" t="s">
         <v>79</v>
       </c>
-      <c r="H46" s="72"/>
-      <c r="I46" s="72"/>
-      <c r="J46" s="72"/>
-      <c r="K46" s="72"/>
-      <c r="L46" s="62"/>
-      <c r="M46" s="64"/>
+      <c r="H46" s="58"/>
+      <c r="I46" s="58"/>
+      <c r="J46" s="58"/>
+      <c r="K46" s="58"/>
+      <c r="L46" s="65"/>
+      <c r="M46" s="66"/>
       <c r="N46" s="32"/>
       <c r="O46"/>
       <c r="P46"/>
     </row>
     <row r="47" spans="1:16">
       <c r="A47" s="32"/>
-      <c r="B47" s="73" t="s">
+      <c r="B47" s="55" t="s">
         <v>80</v>
       </c>
-      <c r="C47" s="73"/>
-      <c r="D47" s="73"/>
-      <c r="E47" s="73"/>
-      <c r="F47" s="73"/>
-      <c r="G47" s="74" t="s">
+      <c r="C47" s="55"/>
+      <c r="D47" s="55"/>
+      <c r="E47" s="55"/>
+      <c r="F47" s="55"/>
+      <c r="G47" s="56" t="s">
         <v>81</v>
       </c>
-      <c r="H47" s="74"/>
-      <c r="I47" s="74"/>
-      <c r="J47" s="74"/>
-      <c r="K47" s="74"/>
-      <c r="L47" s="62"/>
-      <c r="M47" s="64"/>
+      <c r="H47" s="56"/>
+      <c r="I47" s="56"/>
+      <c r="J47" s="56"/>
+      <c r="K47" s="56"/>
+      <c r="L47" s="65"/>
+      <c r="M47" s="66"/>
       <c r="N47" s="32"/>
       <c r="O47"/>
       <c r="P47"/>
     </row>
     <row r="48" spans="1:16">
       <c r="A48" s="32"/>
-      <c r="B48" s="56" t="s">
+      <c r="B48" s="68" t="s">
         <v>82</v>
       </c>
-      <c r="C48" s="57"/>
-      <c r="D48" s="57"/>
-      <c r="E48" s="57"/>
-      <c r="F48" s="58"/>
-      <c r="G48" s="59" t="s">
+      <c r="C48" s="69"/>
+      <c r="D48" s="69"/>
+      <c r="E48" s="69"/>
+      <c r="F48" s="70"/>
+      <c r="G48" s="71" t="s">
         <v>83</v>
       </c>
-      <c r="H48" s="60"/>
-      <c r="I48" s="60"/>
-      <c r="J48" s="60"/>
-      <c r="K48" s="61"/>
-      <c r="L48" s="62"/>
-      <c r="M48" s="64"/>
+      <c r="H48" s="72"/>
+      <c r="I48" s="72"/>
+      <c r="J48" s="72"/>
+      <c r="K48" s="73"/>
+      <c r="L48" s="65"/>
+      <c r="M48" s="66"/>
       <c r="N48" s="32"/>
       <c r="O48"/>
       <c r="P48"/>
     </row>
     <row r="49" spans="1:16">
       <c r="A49" s="32"/>
-      <c r="B49" s="79" t="s">
+      <c r="B49" s="74" t="s">
         <v>84</v>
       </c>
-      <c r="C49" s="79"/>
-      <c r="D49" s="79"/>
-      <c r="E49" s="79"/>
-      <c r="F49" s="79"/>
-      <c r="G49" s="80" t="s">
+      <c r="C49" s="74"/>
+      <c r="D49" s="74"/>
+      <c r="E49" s="74"/>
+      <c r="F49" s="74"/>
+      <c r="G49" s="75" t="s">
         <v>85</v>
       </c>
-      <c r="H49" s="80"/>
-      <c r="I49" s="80"/>
-      <c r="J49" s="80"/>
-      <c r="K49" s="80"/>
-      <c r="L49" s="62"/>
-      <c r="M49" s="64"/>
+      <c r="H49" s="75"/>
+      <c r="I49" s="75"/>
+      <c r="J49" s="75"/>
+      <c r="K49" s="75"/>
+      <c r="L49" s="65"/>
+      <c r="M49" s="66"/>
       <c r="N49" s="32"/>
       <c r="O49"/>
       <c r="P49"/>
     </row>
     <row r="50" spans="1:16">
       <c r="A50" s="32"/>
-      <c r="B50" s="81" t="s">
+      <c r="B50" s="61" t="s">
         <v>86</v>
       </c>
-      <c r="C50" s="82"/>
-      <c r="D50" s="82"/>
-      <c r="E50" s="82"/>
-      <c r="F50" s="83"/>
-      <c r="G50" s="84"/>
-      <c r="H50" s="82"/>
-      <c r="I50" s="82"/>
-      <c r="J50" s="82"/>
-      <c r="K50" s="83"/>
-      <c r="L50" s="62"/>
-      <c r="M50" s="64"/>
+      <c r="C50" s="62"/>
+      <c r="D50" s="62"/>
+      <c r="E50" s="62"/>
+      <c r="F50" s="63"/>
+      <c r="G50" s="64"/>
+      <c r="H50" s="62"/>
+      <c r="I50" s="62"/>
+      <c r="J50" s="62"/>
+      <c r="K50" s="63"/>
+      <c r="L50" s="65"/>
+      <c r="M50" s="66"/>
       <c r="N50" s="32"/>
       <c r="O50"/>
       <c r="P50"/>
@@ -4419,18 +4422,18 @@
     </row>
     <row r="52" spans="1:16">
       <c r="A52" s="32"/>
-      <c r="B52" s="68" t="s">
+      <c r="B52" s="67" t="s">
         <v>87</v>
       </c>
-      <c r="C52" s="68"/>
-      <c r="D52" s="68"/>
-      <c r="E52" s="68"/>
-      <c r="F52" s="68"/>
-      <c r="G52" s="68"/>
-      <c r="H52" s="68"/>
-      <c r="I52" s="68"/>
-      <c r="J52" s="68"/>
-      <c r="K52" s="68"/>
+      <c r="C52" s="67"/>
+      <c r="D52" s="67"/>
+      <c r="E52" s="67"/>
+      <c r="F52" s="67"/>
+      <c r="G52" s="67"/>
+      <c r="H52" s="67"/>
+      <c r="I52" s="67"/>
+      <c r="J52" s="67"/>
+      <c r="K52" s="67"/>
       <c r="L52" s="32"/>
       <c r="M52"/>
       <c r="N52"/>
@@ -4439,20 +4442,20 @@
     </row>
     <row r="53" spans="1:16">
       <c r="A53" s="32"/>
-      <c r="B53" s="73" t="s">
+      <c r="B53" s="55" t="s">
         <v>88</v>
       </c>
-      <c r="C53" s="73"/>
-      <c r="D53" s="73"/>
-      <c r="E53" s="73"/>
-      <c r="F53" s="73"/>
-      <c r="G53" s="74" t="s">
+      <c r="C53" s="55"/>
+      <c r="D53" s="55"/>
+      <c r="E53" s="55"/>
+      <c r="F53" s="55"/>
+      <c r="G53" s="56" t="s">
         <v>89</v>
       </c>
-      <c r="H53" s="74"/>
-      <c r="I53" s="74"/>
-      <c r="J53" s="74"/>
-      <c r="K53" s="74"/>
+      <c r="H53" s="56"/>
+      <c r="I53" s="56"/>
+      <c r="J53" s="56"/>
+      <c r="K53" s="56"/>
       <c r="L53" s="32"/>
       <c r="M53"/>
       <c r="N53"/>
@@ -4461,20 +4464,20 @@
     </row>
     <row r="54" spans="1:16">
       <c r="A54" s="32"/>
-      <c r="B54" s="71" t="s">
+      <c r="B54" s="57" t="s">
         <v>90</v>
       </c>
-      <c r="C54" s="71"/>
-      <c r="D54" s="71"/>
-      <c r="E54" s="71"/>
-      <c r="F54" s="71"/>
-      <c r="G54" s="72">
+      <c r="C54" s="57"/>
+      <c r="D54" s="57"/>
+      <c r="E54" s="57"/>
+      <c r="F54" s="57"/>
+      <c r="G54" s="58">
         <v>1349</v>
       </c>
-      <c r="H54" s="72"/>
-      <c r="I54" s="72"/>
-      <c r="J54" s="72"/>
-      <c r="K54" s="72"/>
+      <c r="H54" s="58"/>
+      <c r="I54" s="58"/>
+      <c r="J54" s="58"/>
+      <c r="K54" s="58"/>
       <c r="L54" s="32"/>
       <c r="M54"/>
       <c r="N54"/>
@@ -4483,20 +4486,20 @@
     </row>
     <row r="55" spans="1:16">
       <c r="A55" s="32"/>
-      <c r="B55" s="73" t="s">
+      <c r="B55" s="55" t="s">
         <v>91</v>
       </c>
-      <c r="C55" s="73"/>
-      <c r="D55" s="73"/>
-      <c r="E55" s="73"/>
-      <c r="F55" s="73"/>
-      <c r="G55" s="74">
+      <c r="C55" s="55"/>
+      <c r="D55" s="55"/>
+      <c r="E55" s="55"/>
+      <c r="F55" s="55"/>
+      <c r="G55" s="56">
         <v>1555</v>
       </c>
-      <c r="H55" s="74"/>
-      <c r="I55" s="74"/>
-      <c r="J55" s="74"/>
-      <c r="K55" s="74"/>
+      <c r="H55" s="56"/>
+      <c r="I55" s="56"/>
+      <c r="J55" s="56"/>
+      <c r="K55" s="56"/>
       <c r="L55" s="32"/>
       <c r="M55"/>
       <c r="N55"/>
@@ -4505,20 +4508,20 @@
     </row>
     <row r="56" spans="1:16">
       <c r="A56" s="32"/>
-      <c r="B56" s="71" t="s">
+      <c r="B56" s="57" t="s">
         <v>92</v>
       </c>
-      <c r="C56" s="71"/>
-      <c r="D56" s="71"/>
-      <c r="E56" s="71"/>
-      <c r="F56" s="71"/>
-      <c r="G56" s="72" t="s">
+      <c r="C56" s="57"/>
+      <c r="D56" s="57"/>
+      <c r="E56" s="57"/>
+      <c r="F56" s="57"/>
+      <c r="G56" s="58" t="s">
         <v>93</v>
       </c>
-      <c r="H56" s="72"/>
-      <c r="I56" s="72"/>
-      <c r="J56" s="72"/>
-      <c r="K56" s="72"/>
+      <c r="H56" s="58"/>
+      <c r="I56" s="58"/>
+      <c r="J56" s="58"/>
+      <c r="K56" s="58"/>
       <c r="L56" s="32"/>
       <c r="M56"/>
       <c r="N56"/>
@@ -4527,20 +4530,20 @@
     </row>
     <row r="57" spans="1:16">
       <c r="A57" s="32"/>
-      <c r="B57" s="73" t="s">
+      <c r="B57" s="55" t="s">
         <v>94</v>
       </c>
-      <c r="C57" s="73"/>
-      <c r="D57" s="73"/>
-      <c r="E57" s="73"/>
-      <c r="F57" s="73"/>
-      <c r="G57" s="74" t="s">
+      <c r="C57" s="55"/>
+      <c r="D57" s="55"/>
+      <c r="E57" s="55"/>
+      <c r="F57" s="55"/>
+      <c r="G57" s="56" t="s">
         <v>95</v>
       </c>
-      <c r="H57" s="74"/>
-      <c r="I57" s="74"/>
-      <c r="J57" s="74"/>
-      <c r="K57" s="74"/>
+      <c r="H57" s="56"/>
+      <c r="I57" s="56"/>
+      <c r="J57" s="56"/>
+      <c r="K57" s="56"/>
       <c r="L57" s="32"/>
       <c r="M57"/>
       <c r="N57"/>
@@ -4549,20 +4552,20 @@
     </row>
     <row r="58" spans="1:16">
       <c r="A58" s="32"/>
-      <c r="B58" s="71" t="s">
+      <c r="B58" s="57" t="s">
         <v>96</v>
       </c>
-      <c r="C58" s="71"/>
-      <c r="D58" s="71"/>
-      <c r="E58" s="71"/>
-      <c r="F58" s="71"/>
-      <c r="G58" s="72" t="s">
+      <c r="C58" s="57"/>
+      <c r="D58" s="57"/>
+      <c r="E58" s="57"/>
+      <c r="F58" s="57"/>
+      <c r="G58" s="58" t="s">
         <v>97</v>
       </c>
-      <c r="H58" s="72"/>
-      <c r="I58" s="72"/>
-      <c r="J58" s="72"/>
-      <c r="K58" s="72"/>
+      <c r="H58" s="58"/>
+      <c r="I58" s="58"/>
+      <c r="J58" s="58"/>
+      <c r="K58" s="58"/>
       <c r="L58" s="32"/>
       <c r="M58"/>
       <c r="N58"/>
@@ -4571,20 +4574,20 @@
     </row>
     <row r="59" spans="1:16">
       <c r="A59" s="32"/>
-      <c r="B59" s="73" t="s">
+      <c r="B59" s="55" t="s">
         <v>98</v>
       </c>
-      <c r="C59" s="73"/>
-      <c r="D59" s="73"/>
-      <c r="E59" s="73"/>
-      <c r="F59" s="73"/>
-      <c r="G59" s="74" t="s">
+      <c r="C59" s="55"/>
+      <c r="D59" s="55"/>
+      <c r="E59" s="55"/>
+      <c r="F59" s="55"/>
+      <c r="G59" s="56" t="s">
         <v>99</v>
       </c>
-      <c r="H59" s="74"/>
-      <c r="I59" s="74"/>
-      <c r="J59" s="74"/>
-      <c r="K59" s="74"/>
+      <c r="H59" s="56"/>
+      <c r="I59" s="56"/>
+      <c r="J59" s="56"/>
+      <c r="K59" s="56"/>
       <c r="L59" s="32"/>
       <c r="M59"/>
       <c r="N59"/>
@@ -4593,20 +4596,20 @@
     </row>
     <row r="60" spans="1:16">
       <c r="A60" s="32"/>
-      <c r="B60" s="71" t="s">
+      <c r="B60" s="57" t="s">
         <v>100</v>
       </c>
-      <c r="C60" s="71"/>
-      <c r="D60" s="71"/>
-      <c r="E60" s="71"/>
-      <c r="F60" s="71"/>
-      <c r="G60" s="72" t="s">
+      <c r="C60" s="57"/>
+      <c r="D60" s="57"/>
+      <c r="E60" s="57"/>
+      <c r="F60" s="57"/>
+      <c r="G60" s="58" t="s">
         <v>101</v>
       </c>
-      <c r="H60" s="72"/>
-      <c r="I60" s="72"/>
-      <c r="J60" s="72"/>
-      <c r="K60" s="72"/>
+      <c r="H60" s="58"/>
+      <c r="I60" s="58"/>
+      <c r="J60" s="58"/>
+      <c r="K60" s="58"/>
       <c r="L60" s="32"/>
       <c r="M60"/>
       <c r="N60"/>
@@ -4615,20 +4618,20 @@
     </row>
     <row r="61" spans="1:16">
       <c r="A61" s="32"/>
-      <c r="B61" s="73" t="s">
+      <c r="B61" s="55" t="s">
         <v>102</v>
       </c>
-      <c r="C61" s="73"/>
-      <c r="D61" s="73"/>
-      <c r="E61" s="73"/>
-      <c r="F61" s="73"/>
-      <c r="G61" s="74" t="s">
+      <c r="C61" s="55"/>
+      <c r="D61" s="55"/>
+      <c r="E61" s="55"/>
+      <c r="F61" s="55"/>
+      <c r="G61" s="56" t="s">
         <v>103</v>
       </c>
-      <c r="H61" s="74"/>
-      <c r="I61" s="74"/>
-      <c r="J61" s="74"/>
-      <c r="K61" s="74"/>
+      <c r="H61" s="56"/>
+      <c r="I61" s="56"/>
+      <c r="J61" s="56"/>
+      <c r="K61" s="56"/>
       <c r="L61" s="32"/>
       <c r="M61"/>
       <c r="N61"/>
@@ -4637,20 +4640,20 @@
     </row>
     <row r="62" spans="1:16">
       <c r="A62" s="32"/>
-      <c r="B62" s="71" t="s">
+      <c r="B62" s="57" t="s">
         <v>104</v>
       </c>
-      <c r="C62" s="71"/>
-      <c r="D62" s="71"/>
-      <c r="E62" s="71"/>
-      <c r="F62" s="71"/>
-      <c r="G62" s="72" t="s">
+      <c r="C62" s="57"/>
+      <c r="D62" s="57"/>
+      <c r="E62" s="57"/>
+      <c r="F62" s="57"/>
+      <c r="G62" s="58" t="s">
         <v>105</v>
       </c>
-      <c r="H62" s="72"/>
-      <c r="I62" s="72"/>
-      <c r="J62" s="72"/>
-      <c r="K62" s="72"/>
+      <c r="H62" s="58"/>
+      <c r="I62" s="58"/>
+      <c r="J62" s="58"/>
+      <c r="K62" s="58"/>
       <c r="L62" s="32"/>
       <c r="M62"/>
       <c r="N62"/>
@@ -4659,20 +4662,20 @@
     </row>
     <row r="63" spans="1:16">
       <c r="A63" s="32"/>
-      <c r="B63" s="73" t="s">
+      <c r="B63" s="55" t="s">
         <v>106</v>
       </c>
-      <c r="C63" s="73"/>
-      <c r="D63" s="73"/>
-      <c r="E63" s="73"/>
-      <c r="F63" s="73"/>
-      <c r="G63" s="74" t="s">
+      <c r="C63" s="55"/>
+      <c r="D63" s="55"/>
+      <c r="E63" s="55"/>
+      <c r="F63" s="55"/>
+      <c r="G63" s="56" t="s">
         <v>107</v>
       </c>
-      <c r="H63" s="74"/>
-      <c r="I63" s="74"/>
-      <c r="J63" s="74"/>
-      <c r="K63" s="74"/>
+      <c r="H63" s="56"/>
+      <c r="I63" s="56"/>
+      <c r="J63" s="56"/>
+      <c r="K63" s="56"/>
       <c r="L63" s="32"/>
       <c r="M63"/>
       <c r="N63"/>
@@ -4681,20 +4684,20 @@
     </row>
     <row r="64" spans="1:16">
       <c r="A64" s="32"/>
-      <c r="B64" s="71" t="s">
+      <c r="B64" s="57" t="s">
         <v>108</v>
       </c>
-      <c r="C64" s="71"/>
-      <c r="D64" s="71"/>
-      <c r="E64" s="71"/>
-      <c r="F64" s="71"/>
-      <c r="G64" s="72">
+      <c r="C64" s="57"/>
+      <c r="D64" s="57"/>
+      <c r="E64" s="57"/>
+      <c r="F64" s="57"/>
+      <c r="G64" s="58">
         <v>166</v>
       </c>
-      <c r="H64" s="72"/>
-      <c r="I64" s="72"/>
-      <c r="J64" s="72"/>
-      <c r="K64" s="72"/>
+      <c r="H64" s="58"/>
+      <c r="I64" s="58"/>
+      <c r="J64" s="58"/>
+      <c r="K64" s="58"/>
       <c r="L64" s="32"/>
       <c r="M64"/>
       <c r="N64"/>
@@ -4703,20 +4706,20 @@
     </row>
     <row r="65" spans="1:16">
       <c r="A65" s="32"/>
-      <c r="B65" s="73" t="s">
+      <c r="B65" s="55" t="s">
         <v>109</v>
       </c>
-      <c r="C65" s="73"/>
-      <c r="D65" s="73"/>
-      <c r="E65" s="73"/>
-      <c r="F65" s="73"/>
-      <c r="G65" s="74" t="s">
+      <c r="C65" s="55"/>
+      <c r="D65" s="55"/>
+      <c r="E65" s="55"/>
+      <c r="F65" s="55"/>
+      <c r="G65" s="56" t="s">
         <v>110</v>
       </c>
-      <c r="H65" s="74"/>
-      <c r="I65" s="74"/>
-      <c r="J65" s="74"/>
-      <c r="K65" s="74"/>
+      <c r="H65" s="56"/>
+      <c r="I65" s="56"/>
+      <c r="J65" s="56"/>
+      <c r="K65" s="56"/>
       <c r="L65" s="32"/>
       <c r="M65"/>
       <c r="N65"/>
@@ -4725,20 +4728,20 @@
     </row>
     <row r="66" spans="1:16">
       <c r="A66" s="32"/>
-      <c r="B66" s="71" t="s">
+      <c r="B66" s="57" t="s">
         <v>111</v>
       </c>
-      <c r="C66" s="71"/>
-      <c r="D66" s="71"/>
-      <c r="E66" s="71"/>
-      <c r="F66" s="71"/>
-      <c r="G66" s="72" t="s">
+      <c r="C66" s="57"/>
+      <c r="D66" s="57"/>
+      <c r="E66" s="57"/>
+      <c r="F66" s="57"/>
+      <c r="G66" s="58" t="s">
         <v>112</v>
       </c>
-      <c r="H66" s="72"/>
-      <c r="I66" s="72"/>
-      <c r="J66" s="72"/>
-      <c r="K66" s="72"/>
+      <c r="H66" s="58"/>
+      <c r="I66" s="58"/>
+      <c r="J66" s="58"/>
+      <c r="K66" s="58"/>
       <c r="L66" s="32"/>
       <c r="M66"/>
       <c r="N66"/>
@@ -4747,20 +4750,20 @@
     </row>
     <row r="67" spans="1:16">
       <c r="A67" s="32"/>
-      <c r="B67" s="73" t="s">
+      <c r="B67" s="55" t="s">
         <v>113</v>
       </c>
-      <c r="C67" s="73"/>
-      <c r="D67" s="73"/>
-      <c r="E67" s="73"/>
-      <c r="F67" s="73"/>
-      <c r="G67" s="74" t="s">
+      <c r="C67" s="55"/>
+      <c r="D67" s="55"/>
+      <c r="E67" s="55"/>
+      <c r="F67" s="55"/>
+      <c r="G67" s="56" t="s">
         <v>114</v>
       </c>
-      <c r="H67" s="74"/>
-      <c r="I67" s="74"/>
-      <c r="J67" s="74"/>
-      <c r="K67" s="74"/>
+      <c r="H67" s="56"/>
+      <c r="I67" s="56"/>
+      <c r="J67" s="56"/>
+      <c r="K67" s="56"/>
       <c r="L67" s="32"/>
       <c r="M67"/>
       <c r="N67"/>
@@ -4769,20 +4772,20 @@
     </row>
     <row r="68" spans="1:16">
       <c r="A68" s="32"/>
-      <c r="B68" s="71" t="s">
+      <c r="B68" s="57" t="s">
         <v>115</v>
       </c>
-      <c r="C68" s="71"/>
-      <c r="D68" s="71"/>
-      <c r="E68" s="71"/>
-      <c r="F68" s="71"/>
-      <c r="G68" s="72" t="s">
+      <c r="C68" s="57"/>
+      <c r="D68" s="57"/>
+      <c r="E68" s="57"/>
+      <c r="F68" s="57"/>
+      <c r="G68" s="58" t="s">
         <v>116</v>
       </c>
-      <c r="H68" s="72"/>
-      <c r="I68" s="72"/>
-      <c r="J68" s="72"/>
-      <c r="K68" s="72"/>
+      <c r="H68" s="58"/>
+      <c r="I68" s="58"/>
+      <c r="J68" s="58"/>
+      <c r="K68" s="58"/>
       <c r="L68" s="32"/>
       <c r="M68"/>
       <c r="N68"/>
@@ -4791,20 +4794,20 @@
     </row>
     <row r="69" spans="1:16">
       <c r="A69" s="32"/>
-      <c r="B69" s="73" t="s">
+      <c r="B69" s="55" t="s">
         <v>117</v>
       </c>
-      <c r="C69" s="73"/>
-      <c r="D69" s="73"/>
-      <c r="E69" s="73"/>
-      <c r="F69" s="73"/>
-      <c r="G69" s="74" t="s">
+      <c r="C69" s="55"/>
+      <c r="D69" s="55"/>
+      <c r="E69" s="55"/>
+      <c r="F69" s="55"/>
+      <c r="G69" s="56" t="s">
         <v>118</v>
       </c>
-      <c r="H69" s="74"/>
-      <c r="I69" s="74"/>
-      <c r="J69" s="74"/>
-      <c r="K69" s="74"/>
+      <c r="H69" s="56"/>
+      <c r="I69" s="56"/>
+      <c r="J69" s="56"/>
+      <c r="K69" s="56"/>
       <c r="L69" s="32"/>
       <c r="M69"/>
       <c r="N69"/>
@@ -4813,20 +4816,20 @@
     </row>
     <row r="70" spans="1:16">
       <c r="A70" s="32"/>
-      <c r="B70" s="71" t="s">
+      <c r="B70" s="57" t="s">
         <v>119</v>
       </c>
-      <c r="C70" s="71"/>
-      <c r="D70" s="71"/>
-      <c r="E70" s="71"/>
-      <c r="F70" s="71"/>
-      <c r="G70" s="72" t="s">
+      <c r="C70" s="57"/>
+      <c r="D70" s="57"/>
+      <c r="E70" s="57"/>
+      <c r="F70" s="57"/>
+      <c r="G70" s="58" t="s">
         <v>120</v>
       </c>
-      <c r="H70" s="72"/>
-      <c r="I70" s="72"/>
-      <c r="J70" s="72"/>
-      <c r="K70" s="72"/>
+      <c r="H70" s="58"/>
+      <c r="I70" s="58"/>
+      <c r="J70" s="58"/>
+      <c r="K70" s="58"/>
       <c r="L70" s="32"/>
       <c r="M70"/>
       <c r="N70"/>
@@ -4835,20 +4838,20 @@
     </row>
     <row r="71" spans="1:16">
       <c r="A71" s="32"/>
-      <c r="B71" s="73" t="s">
+      <c r="B71" s="55" t="s">
         <v>121</v>
       </c>
-      <c r="C71" s="73"/>
-      <c r="D71" s="73"/>
-      <c r="E71" s="73"/>
-      <c r="F71" s="73"/>
-      <c r="G71" s="74" t="s">
+      <c r="C71" s="55"/>
+      <c r="D71" s="55"/>
+      <c r="E71" s="55"/>
+      <c r="F71" s="55"/>
+      <c r="G71" s="56" t="s">
         <v>122</v>
       </c>
-      <c r="H71" s="74"/>
-      <c r="I71" s="74"/>
-      <c r="J71" s="74"/>
-      <c r="K71" s="74"/>
+      <c r="H71" s="56"/>
+      <c r="I71" s="56"/>
+      <c r="J71" s="56"/>
+      <c r="K71" s="56"/>
       <c r="L71" s="32"/>
       <c r="M71"/>
       <c r="N71"/>
@@ -4857,20 +4860,20 @@
     </row>
     <row r="72" spans="1:16">
       <c r="A72" s="32"/>
-      <c r="B72" s="71" t="s">
+      <c r="B72" s="57" t="s">
         <v>123</v>
       </c>
-      <c r="C72" s="71"/>
-      <c r="D72" s="71"/>
-      <c r="E72" s="71"/>
-      <c r="F72" s="71"/>
-      <c r="G72" s="72" t="s">
+      <c r="C72" s="57"/>
+      <c r="D72" s="57"/>
+      <c r="E72" s="57"/>
+      <c r="F72" s="57"/>
+      <c r="G72" s="58" t="s">
         <v>124</v>
       </c>
-      <c r="H72" s="72"/>
-      <c r="I72" s="72"/>
-      <c r="J72" s="72"/>
-      <c r="K72" s="72"/>
+      <c r="H72" s="58"/>
+      <c r="I72" s="58"/>
+      <c r="J72" s="58"/>
+      <c r="K72" s="58"/>
       <c r="L72" s="32"/>
       <c r="M72"/>
       <c r="N72"/>
@@ -4879,20 +4882,20 @@
     </row>
     <row r="73" spans="1:16">
       <c r="A73" s="32"/>
-      <c r="B73" s="73" t="s">
+      <c r="B73" s="55" t="s">
         <v>125</v>
       </c>
-      <c r="C73" s="73"/>
-      <c r="D73" s="73"/>
-      <c r="E73" s="73"/>
-      <c r="F73" s="73"/>
-      <c r="G73" s="86" t="s">
+      <c r="C73" s="55"/>
+      <c r="D73" s="55"/>
+      <c r="E73" s="55"/>
+      <c r="F73" s="55"/>
+      <c r="G73" s="59" t="s">
         <v>126</v>
       </c>
-      <c r="H73" s="86"/>
-      <c r="I73" s="86"/>
-      <c r="J73" s="86"/>
-      <c r="K73" s="86"/>
+      <c r="H73" s="59"/>
+      <c r="I73" s="59"/>
+      <c r="J73" s="59"/>
+      <c r="K73" s="59"/>
       <c r="L73" s="32"/>
       <c r="M73"/>
       <c r="N73"/>
@@ -4901,20 +4904,20 @@
     </row>
     <row r="74" spans="1:16">
       <c r="A74" s="32"/>
-      <c r="B74" s="71" t="s">
+      <c r="B74" s="57" t="s">
         <v>127</v>
       </c>
-      <c r="C74" s="71"/>
-      <c r="D74" s="71"/>
-      <c r="E74" s="71"/>
-      <c r="F74" s="71"/>
-      <c r="G74" s="87" t="s">
+      <c r="C74" s="57"/>
+      <c r="D74" s="57"/>
+      <c r="E74" s="57"/>
+      <c r="F74" s="57"/>
+      <c r="G74" s="60" t="s">
         <v>128</v>
       </c>
-      <c r="H74" s="87"/>
-      <c r="I74" s="87"/>
-      <c r="J74" s="87"/>
-      <c r="K74" s="87"/>
+      <c r="H74" s="60"/>
+      <c r="I74" s="60"/>
+      <c r="J74" s="60"/>
+      <c r="K74" s="60"/>
       <c r="L74" s="32"/>
       <c r="M74"/>
       <c r="N74"/>
@@ -4940,64 +4943,64 @@
       <c r="P75"/>
     </row>
     <row r="76" spans="1:16">
-      <c r="B76" s="50"/>
-      <c r="C76" s="50"/>
-      <c r="D76" s="50"/>
-      <c r="E76" s="50"/>
-      <c r="F76" s="50"/>
-      <c r="G76" s="50"/>
-      <c r="H76" s="50"/>
-      <c r="I76" s="50"/>
-      <c r="J76" s="50"/>
-      <c r="K76" s="50"/>
+      <c r="B76" s="53"/>
+      <c r="C76" s="53"/>
+      <c r="D76" s="53"/>
+      <c r="E76" s="53"/>
+      <c r="F76" s="53"/>
+      <c r="G76" s="53"/>
+      <c r="H76" s="53"/>
+      <c r="I76" s="53"/>
+      <c r="J76" s="53"/>
+      <c r="K76" s="53"/>
       <c r="M76"/>
       <c r="N76"/>
       <c r="O76"/>
       <c r="P76"/>
     </row>
     <row r="77" spans="1:16">
-      <c r="B77" s="50"/>
-      <c r="C77" s="50"/>
-      <c r="D77" s="50"/>
-      <c r="E77" s="50"/>
-      <c r="F77" s="50"/>
-      <c r="G77" s="50"/>
-      <c r="H77" s="50"/>
-      <c r="I77" s="50"/>
-      <c r="J77" s="50"/>
-      <c r="K77" s="50"/>
+      <c r="B77" s="53"/>
+      <c r="C77" s="53"/>
+      <c r="D77" s="53"/>
+      <c r="E77" s="53"/>
+      <c r="F77" s="53"/>
+      <c r="G77" s="53"/>
+      <c r="H77" s="53"/>
+      <c r="I77" s="53"/>
+      <c r="J77" s="53"/>
+      <c r="K77" s="53"/>
       <c r="M77"/>
       <c r="N77"/>
       <c r="O77"/>
       <c r="P77"/>
     </row>
     <row r="78" spans="1:16">
-      <c r="B78" s="50"/>
-      <c r="C78" s="50"/>
-      <c r="D78" s="50"/>
-      <c r="E78" s="50"/>
-      <c r="F78" s="50"/>
-      <c r="G78" s="50"/>
-      <c r="H78" s="50"/>
-      <c r="I78" s="50"/>
-      <c r="J78" s="50"/>
-      <c r="K78" s="50"/>
+      <c r="B78" s="53"/>
+      <c r="C78" s="53"/>
+      <c r="D78" s="53"/>
+      <c r="E78" s="53"/>
+      <c r="F78" s="53"/>
+      <c r="G78" s="53"/>
+      <c r="H78" s="53"/>
+      <c r="I78" s="53"/>
+      <c r="J78" s="53"/>
+      <c r="K78" s="53"/>
       <c r="M78"/>
       <c r="N78"/>
       <c r="O78"/>
       <c r="P78"/>
     </row>
     <row r="79" spans="1:16">
-      <c r="B79" s="50"/>
-      <c r="C79" s="50"/>
-      <c r="D79" s="50"/>
-      <c r="E79" s="50"/>
-      <c r="F79" s="50"/>
-      <c r="G79" s="50"/>
-      <c r="H79" s="50"/>
-      <c r="I79" s="50"/>
-      <c r="J79" s="50"/>
-      <c r="K79" s="50"/>
+      <c r="B79" s="53"/>
+      <c r="C79" s="53"/>
+      <c r="D79" s="53"/>
+      <c r="E79" s="53"/>
+      <c r="F79" s="53"/>
+      <c r="G79" s="53"/>
+      <c r="H79" s="53"/>
+      <c r="I79" s="53"/>
+      <c r="J79" s="53"/>
+      <c r="K79" s="53"/>
       <c r="M79"/>
       <c r="N79"/>
       <c r="O79"/>
@@ -5051,6 +5054,148 @@
     <row r="120" customFormat="1"/>
   </sheetData>
   <mergeCells count="166">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="B9:K9"/>
+    <mergeCell ref="B12:K12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="H13:K13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="H14:K14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="H15:K15"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="H16:K16"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="E17:G17"/>
+    <mergeCell ref="H17:K17"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="H18:K18"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="H19:K19"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="H20:K20"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="H21:K21"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="H22:K22"/>
+    <mergeCell ref="B24:K24"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="G25:K25"/>
+    <mergeCell ref="L25:M25"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="G26:K26"/>
+    <mergeCell ref="L26:M26"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="G27:K27"/>
+    <mergeCell ref="L27:M27"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="G28:K28"/>
+    <mergeCell ref="L28:M28"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="G29:K29"/>
+    <mergeCell ref="L29:M29"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="G30:K30"/>
+    <mergeCell ref="L30:M30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="G31:K31"/>
+    <mergeCell ref="L31:M31"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="G32:K32"/>
+    <mergeCell ref="L32:M32"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="G33:K33"/>
+    <mergeCell ref="L33:M33"/>
+    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="G34:K34"/>
+    <mergeCell ref="L34:M34"/>
+    <mergeCell ref="B35:F35"/>
+    <mergeCell ref="G35:K35"/>
+    <mergeCell ref="L35:M35"/>
+    <mergeCell ref="B36:F36"/>
+    <mergeCell ref="G36:K36"/>
+    <mergeCell ref="L36:M36"/>
+    <mergeCell ref="B37:F37"/>
+    <mergeCell ref="G37:K37"/>
+    <mergeCell ref="L37:M37"/>
+    <mergeCell ref="B38:F38"/>
+    <mergeCell ref="G38:K38"/>
+    <mergeCell ref="L38:M38"/>
+    <mergeCell ref="B39:F39"/>
+    <mergeCell ref="G39:K39"/>
+    <mergeCell ref="L39:M39"/>
+    <mergeCell ref="B40:F40"/>
+    <mergeCell ref="G40:K40"/>
+    <mergeCell ref="L40:M40"/>
+    <mergeCell ref="B41:F41"/>
+    <mergeCell ref="G41:K41"/>
+    <mergeCell ref="L41:M41"/>
+    <mergeCell ref="B42:F42"/>
+    <mergeCell ref="G42:K42"/>
+    <mergeCell ref="L42:M42"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="G43:K43"/>
+    <mergeCell ref="L43:M43"/>
+    <mergeCell ref="B44:F44"/>
+    <mergeCell ref="G44:K44"/>
+    <mergeCell ref="L44:M44"/>
+    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="G45:K45"/>
+    <mergeCell ref="L45:M45"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="G46:K46"/>
+    <mergeCell ref="L46:M46"/>
+    <mergeCell ref="B47:F47"/>
+    <mergeCell ref="G47:K47"/>
+    <mergeCell ref="L47:M47"/>
+    <mergeCell ref="B48:F48"/>
+    <mergeCell ref="G48:K48"/>
+    <mergeCell ref="L48:M48"/>
+    <mergeCell ref="B49:F49"/>
+    <mergeCell ref="G49:K49"/>
+    <mergeCell ref="L49:M49"/>
+    <mergeCell ref="B50:F50"/>
+    <mergeCell ref="G50:K50"/>
+    <mergeCell ref="L50:M50"/>
+    <mergeCell ref="B52:K52"/>
+    <mergeCell ref="B53:F53"/>
+    <mergeCell ref="G53:K53"/>
+    <mergeCell ref="B54:F54"/>
+    <mergeCell ref="G54:K54"/>
+    <mergeCell ref="B55:F55"/>
+    <mergeCell ref="G55:K55"/>
+    <mergeCell ref="B56:F56"/>
+    <mergeCell ref="G56:K56"/>
+    <mergeCell ref="B57:F57"/>
+    <mergeCell ref="G57:K57"/>
+    <mergeCell ref="B58:F58"/>
+    <mergeCell ref="G58:K58"/>
+    <mergeCell ref="B59:F59"/>
+    <mergeCell ref="G59:K59"/>
+    <mergeCell ref="B60:F60"/>
+    <mergeCell ref="G60:K60"/>
+    <mergeCell ref="G69:K69"/>
+    <mergeCell ref="B70:F70"/>
+    <mergeCell ref="G70:K70"/>
+    <mergeCell ref="B61:F61"/>
+    <mergeCell ref="G61:K61"/>
+    <mergeCell ref="B62:F62"/>
+    <mergeCell ref="G62:K62"/>
+    <mergeCell ref="B63:F63"/>
+    <mergeCell ref="G63:K63"/>
+    <mergeCell ref="B64:F64"/>
+    <mergeCell ref="G64:K64"/>
+    <mergeCell ref="B65:F65"/>
+    <mergeCell ref="G65:K65"/>
     <mergeCell ref="B77:F77"/>
     <mergeCell ref="G77:K77"/>
     <mergeCell ref="B78:F78"/>
@@ -5075,148 +5220,6 @@
     <mergeCell ref="B68:F68"/>
     <mergeCell ref="G68:K68"/>
     <mergeCell ref="B69:F69"/>
-    <mergeCell ref="G69:K69"/>
-    <mergeCell ref="B70:F70"/>
-    <mergeCell ref="G70:K70"/>
-    <mergeCell ref="B61:F61"/>
-    <mergeCell ref="G61:K61"/>
-    <mergeCell ref="B62:F62"/>
-    <mergeCell ref="G62:K62"/>
-    <mergeCell ref="B63:F63"/>
-    <mergeCell ref="G63:K63"/>
-    <mergeCell ref="B64:F64"/>
-    <mergeCell ref="G64:K64"/>
-    <mergeCell ref="B65:F65"/>
-    <mergeCell ref="G65:K65"/>
-    <mergeCell ref="B56:F56"/>
-    <mergeCell ref="G56:K56"/>
-    <mergeCell ref="B57:F57"/>
-    <mergeCell ref="G57:K57"/>
-    <mergeCell ref="B58:F58"/>
-    <mergeCell ref="G58:K58"/>
-    <mergeCell ref="B59:F59"/>
-    <mergeCell ref="G59:K59"/>
-    <mergeCell ref="B60:F60"/>
-    <mergeCell ref="G60:K60"/>
-    <mergeCell ref="B50:F50"/>
-    <mergeCell ref="G50:K50"/>
-    <mergeCell ref="L50:M50"/>
-    <mergeCell ref="B52:K52"/>
-    <mergeCell ref="B53:F53"/>
-    <mergeCell ref="G53:K53"/>
-    <mergeCell ref="B54:F54"/>
-    <mergeCell ref="G54:K54"/>
-    <mergeCell ref="B55:F55"/>
-    <mergeCell ref="G55:K55"/>
-    <mergeCell ref="B47:F47"/>
-    <mergeCell ref="G47:K47"/>
-    <mergeCell ref="L47:M47"/>
-    <mergeCell ref="B48:F48"/>
-    <mergeCell ref="G48:K48"/>
-    <mergeCell ref="L48:M48"/>
-    <mergeCell ref="B49:F49"/>
-    <mergeCell ref="G49:K49"/>
-    <mergeCell ref="L49:M49"/>
-    <mergeCell ref="B44:F44"/>
-    <mergeCell ref="G44:K44"/>
-    <mergeCell ref="L44:M44"/>
-    <mergeCell ref="B45:F45"/>
-    <mergeCell ref="G45:K45"/>
-    <mergeCell ref="L45:M45"/>
-    <mergeCell ref="B46:F46"/>
-    <mergeCell ref="G46:K46"/>
-    <mergeCell ref="L46:M46"/>
-    <mergeCell ref="B41:F41"/>
-    <mergeCell ref="G41:K41"/>
-    <mergeCell ref="L41:M41"/>
-    <mergeCell ref="B42:F42"/>
-    <mergeCell ref="G42:K42"/>
-    <mergeCell ref="L42:M42"/>
-    <mergeCell ref="B43:F43"/>
-    <mergeCell ref="G43:K43"/>
-    <mergeCell ref="L43:M43"/>
-    <mergeCell ref="B38:F38"/>
-    <mergeCell ref="G38:K38"/>
-    <mergeCell ref="L38:M38"/>
-    <mergeCell ref="B39:F39"/>
-    <mergeCell ref="G39:K39"/>
-    <mergeCell ref="L39:M39"/>
-    <mergeCell ref="B40:F40"/>
-    <mergeCell ref="G40:K40"/>
-    <mergeCell ref="L40:M40"/>
-    <mergeCell ref="B35:F35"/>
-    <mergeCell ref="G35:K35"/>
-    <mergeCell ref="L35:M35"/>
-    <mergeCell ref="B36:F36"/>
-    <mergeCell ref="G36:K36"/>
-    <mergeCell ref="L36:M36"/>
-    <mergeCell ref="B37:F37"/>
-    <mergeCell ref="G37:K37"/>
-    <mergeCell ref="L37:M37"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="G32:K32"/>
-    <mergeCell ref="L32:M32"/>
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="G33:K33"/>
-    <mergeCell ref="L33:M33"/>
-    <mergeCell ref="B34:F34"/>
-    <mergeCell ref="G34:K34"/>
-    <mergeCell ref="L34:M34"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="G29:K29"/>
-    <mergeCell ref="L29:M29"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="G30:K30"/>
-    <mergeCell ref="L30:M30"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="G31:K31"/>
-    <mergeCell ref="L31:M31"/>
-    <mergeCell ref="L25:M25"/>
-    <mergeCell ref="B26:F26"/>
-    <mergeCell ref="G26:K26"/>
-    <mergeCell ref="L26:M26"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="G27:K27"/>
-    <mergeCell ref="L27:M27"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="G28:K28"/>
-    <mergeCell ref="L28:M28"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="H21:K21"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="H22:K22"/>
-    <mergeCell ref="B24:K24"/>
-    <mergeCell ref="B25:F25"/>
-    <mergeCell ref="G25:K25"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="H18:K18"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="H19:K19"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="H20:K20"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="H15:K15"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="E16:G16"/>
-    <mergeCell ref="H16:K16"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="E17:G17"/>
-    <mergeCell ref="H17:K17"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="B9:K9"/>
-    <mergeCell ref="B12:K12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="E13:G13"/>
-    <mergeCell ref="H13:K13"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="E14:G14"/>
-    <mergeCell ref="H14:K14"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="L30" r:id="rId1" tooltip="mailto:ccfi_sugbu@yahoo.com" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -6633,20 +6636,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
-      <c r="A1" s="88" t="s">
+      <c r="A1" s="91" t="s">
         <v>447</v>
       </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="91"/>
       <c r="N1"/>
     </row>
     <row r="2" spans="1:14" ht="138.75">
@@ -7125,14 +7128,14 @@
       <c r="A14" s="5">
         <v>13</v>
       </c>
-      <c r="B14" s="92" t="s">
+      <c r="B14" s="50" t="s">
         <v>727</v>
       </c>
-      <c r="C14" s="92"/>
-      <c r="D14" s="93" t="s">
+      <c r="C14" s="50"/>
+      <c r="D14" s="51" t="s">
         <v>722</v>
       </c>
-      <c r="E14" s="92" t="s">
+      <c r="E14" s="50" t="s">
         <v>527</v>
       </c>
       <c r="F14" s="6" t="s">
@@ -7155,11 +7158,11 @@
     </row>
     <row r="15" spans="1:14" ht="83.25">
       <c r="A15" s="5"/>
-      <c r="B15" s="92" t="s">
+      <c r="B15" s="50" t="s">
         <v>728</v>
       </c>
-      <c r="C15" s="92"/>
-      <c r="D15" s="93"/>
+      <c r="C15" s="50"/>
+      <c r="D15" s="51"/>
       <c r="E15" s="6" t="s">
         <v>726</v>
       </c>
@@ -7172,7 +7175,7 @@
       <c r="H15" s="34" t="s">
         <v>534</v>
       </c>
-      <c r="I15" s="94"/>
+      <c r="I15" s="52"/>
       <c r="J15" s="6"/>
       <c r="K15" s="43"/>
       <c r="L15" s="6"/>
@@ -8002,16 +8005,16 @@
       <c r="A37" s="5">
         <v>35</v>
       </c>
-      <c r="B37" s="89" t="s">
+      <c r="B37" s="92" t="s">
         <v>669</v>
       </c>
-      <c r="C37" s="90" t="s">
+      <c r="C37" s="93" t="s">
         <v>670</v>
       </c>
-      <c r="D37" s="91" t="s">
+      <c r="D37" s="94" t="s">
         <v>722</v>
       </c>
-      <c r="E37" s="89" t="s">
+      <c r="E37" s="92" t="s">
         <v>719</v>
       </c>
       <c r="F37" s="6" t="s">
@@ -8032,10 +8035,10 @@
     </row>
     <row r="38" spans="1:14" ht="55.5">
       <c r="A38" s="5"/>
-      <c r="B38" s="89"/>
-      <c r="C38" s="89"/>
-      <c r="D38" s="91"/>
-      <c r="E38" s="89"/>
+      <c r="B38" s="92"/>
+      <c r="C38" s="92"/>
+      <c r="D38" s="94"/>
+      <c r="E38" s="92"/>
       <c r="F38" s="6" t="s">
         <v>674</v>
       </c>
@@ -8194,12 +8197,12 @@
       </c>
       <c r="N42" s="6"/>
     </row>
-    <row r="43" spans="1:14" ht="83.25">
+    <row r="43" spans="1:14" ht="55.5">
       <c r="A43" s="8">
         <v>40</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>298</v>
+        <v>730</v>
       </c>
       <c r="C43" s="3"/>
       <c r="D43" s="35" t="s">

</xml_diff>